<commit_message>
chore: updated the urls for the new jsons
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1586C45E-DEA8-4DBF-87D5-695904905001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B79A0EB-7146-4C10-9515-8E76BD80662D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="132" windowWidth="23040" windowHeight="12024" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5582" uniqueCount="2411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5603" uniqueCount="2431">
   <si>
     <t>DbId</t>
   </si>
@@ -7261,6 +7261,66 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/air_temperature/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/daily_aqi_nitrogen_dioxide/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_ammonium_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_ammonium_nitrate_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_black_carbon_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_ammonium_sulfate_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_biomass_burning_aerosol_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_dust_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_sulfate_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_nitrate_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_nitrogen_dioxide_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_nox_expressed_as_nitrogen_dioxide_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_organic_carbon_from_fossil_fuel_combustion_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/mc_secondary_particulate_organic_matter_in_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/relative_humidity/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/mc_pm2p5_dry_aerosol_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/daily_aqi_nitrogen_dioxide/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/daily_aqi_pm2p5_dry_aerosol/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/mc_nitrogen_dioxide_in_air/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/mc_nox_expressed_as_nitrogen_dioxide_in_air/info.json</t>
   </si>
 </sst>
 </file>
@@ -10354,7 +10414,9 @@
       <c r="M43">
         <v>7002</v>
       </c>
-      <c r="O43" s="3"/>
+      <c r="O43" s="3" t="s">
+        <v>2411</v>
+      </c>
       <c r="P43">
         <v>2</v>
       </c>
@@ -10411,6 +10473,9 @@
       <c r="M44">
         <v>7003</v>
       </c>
+      <c r="O44" s="3" t="s">
+        <v>2411</v>
+      </c>
       <c r="P44">
         <v>2</v>
       </c>
@@ -10526,6 +10591,9 @@
       <c r="M46">
         <v>7005</v>
       </c>
+      <c r="O46" s="3" t="s">
+        <v>2412</v>
+      </c>
       <c r="P46">
         <v>2</v>
       </c>
@@ -10582,6 +10650,9 @@
       <c r="M47">
         <v>7006</v>
       </c>
+      <c r="O47" s="3" t="s">
+        <v>2413</v>
+      </c>
       <c r="P47">
         <v>2</v>
       </c>
@@ -10638,6 +10709,9 @@
       <c r="M48">
         <v>7007</v>
       </c>
+      <c r="O48" s="3" t="s">
+        <v>2415</v>
+      </c>
       <c r="P48">
         <v>2</v>
       </c>
@@ -10694,6 +10768,9 @@
       <c r="M49">
         <v>7008</v>
       </c>
+      <c r="O49" s="3" t="s">
+        <v>2416</v>
+      </c>
       <c r="P49">
         <v>2</v>
       </c>
@@ -10750,6 +10827,9 @@
       <c r="M50">
         <v>7009</v>
       </c>
+      <c r="O50" s="3" t="s">
+        <v>2414</v>
+      </c>
       <c r="P50">
         <v>2</v>
       </c>
@@ -10806,6 +10886,9 @@
       <c r="M51">
         <v>7010</v>
       </c>
+      <c r="O51" s="3" t="s">
+        <v>2417</v>
+      </c>
       <c r="P51">
         <v>2</v>
       </c>
@@ -10862,6 +10945,9 @@
       <c r="M52">
         <v>7011</v>
       </c>
+      <c r="O52" s="3" t="s">
+        <v>2419</v>
+      </c>
       <c r="P52">
         <v>2</v>
       </c>
@@ -10918,6 +11004,9 @@
       <c r="M53">
         <v>7012</v>
       </c>
+      <c r="O53" s="3" t="s">
+        <v>2420</v>
+      </c>
       <c r="P53">
         <v>2</v>
       </c>
@@ -10974,6 +11063,9 @@
       <c r="M54">
         <v>7013</v>
       </c>
+      <c r="O54" s="3" t="s">
+        <v>2421</v>
+      </c>
       <c r="P54">
         <v>2</v>
       </c>
@@ -11030,6 +11122,9 @@
       <c r="M55">
         <v>7014</v>
       </c>
+      <c r="O55" s="3" t="s">
+        <v>2425</v>
+      </c>
       <c r="P55">
         <v>2</v>
       </c>
@@ -11086,6 +11181,9 @@
       <c r="M56">
         <v>7015</v>
       </c>
+      <c r="O56" s="3" t="s">
+        <v>2424</v>
+      </c>
       <c r="P56">
         <v>2</v>
       </c>
@@ -11142,6 +11240,9 @@
       <c r="M57">
         <v>7016</v>
       </c>
+      <c r="O57" s="3" t="s">
+        <v>2418</v>
+      </c>
       <c r="P57">
         <v>2</v>
       </c>
@@ -11198,6 +11299,9 @@
       <c r="M58">
         <v>7017</v>
       </c>
+      <c r="O58" s="3" t="s">
+        <v>2422</v>
+      </c>
       <c r="P58">
         <v>2</v>
       </c>
@@ -11254,6 +11358,9 @@
       <c r="M59">
         <v>7018</v>
       </c>
+      <c r="O59" s="3" t="s">
+        <v>2423</v>
+      </c>
       <c r="P59">
         <v>2</v>
       </c>
@@ -11307,6 +11414,7 @@
       <c r="M60">
         <v>8001</v>
       </c>
+      <c r="O60" s="3"/>
       <c r="P60">
         <v>2</v>
       </c>
@@ -11363,6 +11471,9 @@
       <c r="M61">
         <v>8002</v>
       </c>
+      <c r="O61" s="3" t="s">
+        <v>2427</v>
+      </c>
       <c r="P61">
         <v>2</v>
       </c>
@@ -11419,6 +11530,9 @@
       <c r="M62">
         <v>8003</v>
       </c>
+      <c r="O62" s="3" t="s">
+        <v>2428</v>
+      </c>
       <c r="P62">
         <v>2</v>
       </c>
@@ -11475,6 +11589,9 @@
       <c r="M63">
         <v>8004</v>
       </c>
+      <c r="O63" s="3" t="s">
+        <v>2429</v>
+      </c>
       <c r="P63">
         <v>2</v>
       </c>
@@ -11531,6 +11648,9 @@
       <c r="M64">
         <v>8005</v>
       </c>
+      <c r="O64" s="3" t="s">
+        <v>2430</v>
+      </c>
       <c r="P64">
         <v>2</v>
       </c>
@@ -11586,6 +11706,9 @@
       </c>
       <c r="M65">
         <v>8006</v>
+      </c>
+      <c r="O65" s="3" t="s">
+        <v>2426</v>
       </c>
       <c r="P65">
         <v>2</v>
@@ -11616,6 +11739,28 @@
     <hyperlink ref="O38" r:id="rId8" xr:uid="{71FF0051-ABE5-4973-9ED9-91F5EC5E19E7}"/>
     <hyperlink ref="O40" r:id="rId9" xr:uid="{356432AE-63BD-45AD-AFAA-748A8876906A}"/>
     <hyperlink ref="O45" r:id="rId10" xr:uid="{4252AAA9-D643-4DFB-8757-57BF2C62AF79}"/>
+    <hyperlink ref="O43" r:id="rId11" xr:uid="{4252AAA9-D643-4DFB-8757-57BF2C62AF79}"/>
+    <hyperlink ref="O44" r:id="rId12" xr:uid="{4900D3BB-243B-40FF-9C55-6C4BFE9C0CFE}"/>
+    <hyperlink ref="O46" r:id="rId13" xr:uid="{25DCD23B-0B79-462D-8B8E-F58EC597A07D}"/>
+    <hyperlink ref="O47" r:id="rId14" xr:uid="{D25B6B7C-9BDB-4B88-A91C-C8F4749825FC}"/>
+    <hyperlink ref="O48" r:id="rId15" xr:uid="{3F61F8D5-D025-47EA-9E46-A33CD2A748C3}"/>
+    <hyperlink ref="O49" r:id="rId16" xr:uid="{7413B110-AA8C-4D1F-B232-EC9D2676EC03}"/>
+    <hyperlink ref="O50" r:id="rId17" xr:uid="{A8941504-CE22-4FFF-8C72-0C327A3F35E7}"/>
+    <hyperlink ref="O51" r:id="rId18" xr:uid="{4A006016-10C1-42ED-80E8-802F405B4AE4}"/>
+    <hyperlink ref="O52" r:id="rId19" xr:uid="{7E9F5DD0-1FF6-476A-A906-2A44F86A1D11}"/>
+    <hyperlink ref="O53" r:id="rId20" xr:uid="{1AD16DE8-1400-4B84-9B62-7205C096E12F}"/>
+    <hyperlink ref="O54" r:id="rId21" xr:uid="{C3A01C21-E8E2-417F-B950-130AACEE76C2}"/>
+    <hyperlink ref="O58" r:id="rId22" xr:uid="{76E42F68-0A71-40AC-B534-0BF58052A7AA}"/>
+    <hyperlink ref="O59" r:id="rId23" xr:uid="{32748E37-142E-4E11-B188-229CC5F68817}"/>
+    <hyperlink ref="O56" r:id="rId24" xr:uid="{9ED538C0-DBAB-4F32-B43E-BD185D1D322C}"/>
+    <hyperlink ref="O57" r:id="rId25" xr:uid="{57C56A3D-FC73-437B-BCB9-F35C624A7AC4}"/>
+    <hyperlink ref="O55" r:id="rId26" xr:uid="{D04C60CD-E9F0-40B2-BFF1-8E0AB7A9A0EF}"/>
+    <hyperlink ref="O61" r:id="rId27" xr:uid="{DD24637B-8A52-4477-BD1C-DE472004863A}"/>
+    <hyperlink ref="O62:O64" r:id="rId28" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/daily_aqi_nitrogen_dioxide/info.json" xr:uid="{955E32ED-9CFA-41A4-9D09-5B1D66C2A966}"/>
+    <hyperlink ref="O65" r:id="rId29" xr:uid="{039F5F3E-0910-4EE6-9FE0-7654E10CABAD}"/>
+    <hyperlink ref="O62" r:id="rId30" xr:uid="{373745D5-336B-46AD-BEF0-FF285433016E}"/>
+    <hyperlink ref="O63" r:id="rId31" xr:uid="{356CAD23-03AB-460F-AFCA-EC4BDE2D8AE0}"/>
+    <hyperlink ref="O64" r:id="rId32" xr:uid="{4F6B4081-E0D1-4EF1-825D-2153F4EE3414}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: fixed the broken urls from xml to json
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39287A48-5298-454A-A7BC-F539CE481AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DC6B3F-E098-4B35-A206-8FD8BC4483DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7299,54 +7299,6 @@
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/daily_aqi_nitrogen_dioxide/2011info.json</t>
   </si>
   <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2019info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2018info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2017info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2016info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2015info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2014info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2012info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2011info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2010info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2009info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2008info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2007info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2006info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2005info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2004info.xml</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2003info.xml</t>
-  </si>
-  <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/daily_aqi_nitrogen_dioxide/2010info.json</t>
   </si>
   <si>
@@ -8344,6 +8296,54 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL_BC/mc_pm2p5_dry_aerosol_in_air/2003info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2019info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2018info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2017info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2016info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2015info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2014info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2012info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2011info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2010info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2009info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2008info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2007info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2006info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2005info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2004info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/DSH/Annual/SL/daily_aqi_nitrogen_dioxide/2003info.json</t>
   </si>
 </sst>
 </file>
@@ -60348,7 +60348,7 @@
       </c>
       <c r="J1159" s="6"/>
       <c r="L1159" s="3" t="s">
-        <v>2423</v>
+        <v>2756</v>
       </c>
       <c r="M1159">
         <v>2</v>
@@ -60394,7 +60394,7 @@
       </c>
       <c r="J1160" s="6"/>
       <c r="L1160" s="3" t="s">
-        <v>2424</v>
+        <v>2757</v>
       </c>
       <c r="M1160">
         <v>2</v>
@@ -60440,7 +60440,7 @@
       </c>
       <c r="J1161" s="6"/>
       <c r="L1161" s="3" t="s">
-        <v>2425</v>
+        <v>2758</v>
       </c>
       <c r="M1161">
         <v>2</v>
@@ -60486,7 +60486,7 @@
       </c>
       <c r="J1162" s="6"/>
       <c r="L1162" s="3" t="s">
-        <v>2426</v>
+        <v>2759</v>
       </c>
       <c r="M1162">
         <v>2</v>
@@ -60532,7 +60532,7 @@
       </c>
       <c r="J1163" s="6"/>
       <c r="L1163" s="3" t="s">
-        <v>2427</v>
+        <v>2760</v>
       </c>
       <c r="M1163">
         <v>2</v>
@@ -60578,7 +60578,7 @@
       </c>
       <c r="J1164" s="6"/>
       <c r="L1164" s="3" t="s">
-        <v>2428</v>
+        <v>2761</v>
       </c>
       <c r="M1164">
         <v>2</v>
@@ -60624,7 +60624,7 @@
       </c>
       <c r="J1165" s="6"/>
       <c r="L1165" s="3" t="s">
-        <v>2429</v>
+        <v>2762</v>
       </c>
       <c r="M1165">
         <v>2</v>
@@ -60670,7 +60670,7 @@
       </c>
       <c r="J1166" s="6"/>
       <c r="L1166" s="3" t="s">
-        <v>2430</v>
+        <v>2763</v>
       </c>
       <c r="M1166">
         <v>2</v>
@@ -60716,7 +60716,7 @@
       </c>
       <c r="J1167" s="6"/>
       <c r="L1167" s="3" t="s">
-        <v>2431</v>
+        <v>2764</v>
       </c>
       <c r="M1167">
         <v>2</v>
@@ -60762,7 +60762,7 @@
       </c>
       <c r="J1168" s="6"/>
       <c r="L1168" s="3" t="s">
-        <v>2432</v>
+        <v>2765</v>
       </c>
       <c r="M1168">
         <v>2</v>
@@ -60808,7 +60808,7 @@
       </c>
       <c r="J1169" s="6"/>
       <c r="L1169" s="3" t="s">
-        <v>2433</v>
+        <v>2766</v>
       </c>
       <c r="M1169">
         <v>2</v>
@@ -60854,7 +60854,7 @@
       </c>
       <c r="J1170" s="6"/>
       <c r="L1170" s="3" t="s">
-        <v>2434</v>
+        <v>2767</v>
       </c>
       <c r="M1170">
         <v>2</v>
@@ -60900,7 +60900,7 @@
       </c>
       <c r="J1171" s="6"/>
       <c r="L1171" s="3" t="s">
-        <v>2435</v>
+        <v>2768</v>
       </c>
       <c r="M1171">
         <v>2</v>
@@ -60946,7 +60946,7 @@
       </c>
       <c r="J1172" s="6"/>
       <c r="L1172" s="3" t="s">
-        <v>2436</v>
+        <v>2769</v>
       </c>
       <c r="M1172">
         <v>2</v>
@@ -60992,7 +60992,7 @@
       </c>
       <c r="J1173" s="6"/>
       <c r="L1173" s="3" t="s">
-        <v>2437</v>
+        <v>2770</v>
       </c>
       <c r="M1173">
         <v>2</v>
@@ -61038,7 +61038,7 @@
       </c>
       <c r="J1174" s="6"/>
       <c r="L1174" s="3" t="s">
-        <v>2438</v>
+        <v>2771</v>
       </c>
       <c r="M1174">
         <v>2</v>
@@ -61452,7 +61452,7 @@
       </c>
       <c r="J1183" s="6"/>
       <c r="L1183" s="3" t="s">
-        <v>2439</v>
+        <v>2423</v>
       </c>
       <c r="M1183">
         <v>2</v>
@@ -61498,7 +61498,7 @@
       </c>
       <c r="J1184" s="6"/>
       <c r="L1184" s="3" t="s">
-        <v>2440</v>
+        <v>2424</v>
       </c>
       <c r="M1184">
         <v>2</v>
@@ -61544,7 +61544,7 @@
       </c>
       <c r="J1185" s="6"/>
       <c r="L1185" s="3" t="s">
-        <v>2441</v>
+        <v>2425</v>
       </c>
       <c r="M1185">
         <v>2</v>
@@ -61590,7 +61590,7 @@
       </c>
       <c r="J1186" s="6"/>
       <c r="L1186" s="3" t="s">
-        <v>2442</v>
+        <v>2426</v>
       </c>
       <c r="M1186">
         <v>2</v>
@@ -61636,7 +61636,7 @@
       </c>
       <c r="J1187" s="6"/>
       <c r="L1187" s="3" t="s">
-        <v>2443</v>
+        <v>2427</v>
       </c>
       <c r="M1187">
         <v>2</v>
@@ -61682,7 +61682,7 @@
       </c>
       <c r="J1188" s="6"/>
       <c r="L1188" s="3" t="s">
-        <v>2444</v>
+        <v>2428</v>
       </c>
       <c r="M1188">
         <v>2</v>
@@ -61728,7 +61728,7 @@
       </c>
       <c r="J1189" s="6"/>
       <c r="L1189" s="3" t="s">
-        <v>2445</v>
+        <v>2429</v>
       </c>
       <c r="M1189">
         <v>2</v>
@@ -61774,7 +61774,7 @@
       </c>
       <c r="J1190" s="6"/>
       <c r="L1190" s="3" t="s">
-        <v>2446</v>
+        <v>2430</v>
       </c>
       <c r="M1190">
         <v>2</v>
@@ -61820,7 +61820,7 @@
       </c>
       <c r="J1191" s="6"/>
       <c r="L1191" s="3" t="s">
-        <v>2447</v>
+        <v>2431</v>
       </c>
       <c r="M1191">
         <v>2</v>
@@ -61866,7 +61866,7 @@
       </c>
       <c r="J1192" s="6"/>
       <c r="L1192" s="3" t="s">
-        <v>2448</v>
+        <v>2432</v>
       </c>
       <c r="M1192">
         <v>2</v>
@@ -61912,7 +61912,7 @@
       </c>
       <c r="J1193" s="6"/>
       <c r="L1193" s="3" t="s">
-        <v>2449</v>
+        <v>2433</v>
       </c>
       <c r="M1193">
         <v>2</v>
@@ -61958,7 +61958,7 @@
       </c>
       <c r="J1194" s="6"/>
       <c r="L1194" s="3" t="s">
-        <v>2450</v>
+        <v>2434</v>
       </c>
       <c r="M1194">
         <v>2</v>
@@ -62004,7 +62004,7 @@
       </c>
       <c r="J1195" s="6"/>
       <c r="L1195" s="3" t="s">
-        <v>2451</v>
+        <v>2435</v>
       </c>
       <c r="M1195">
         <v>2</v>
@@ -62050,7 +62050,7 @@
       </c>
       <c r="J1196" s="6"/>
       <c r="L1196" s="3" t="s">
-        <v>2452</v>
+        <v>2436</v>
       </c>
       <c r="M1196">
         <v>2</v>
@@ -62096,7 +62096,7 @@
       </c>
       <c r="J1197" s="6"/>
       <c r="L1197" s="3" t="s">
-        <v>2453</v>
+        <v>2437</v>
       </c>
       <c r="M1197">
         <v>2</v>
@@ -62142,7 +62142,7 @@
       </c>
       <c r="J1198" s="6"/>
       <c r="L1198" s="3" t="s">
-        <v>2454</v>
+        <v>2438</v>
       </c>
       <c r="M1198">
         <v>2</v>
@@ -62188,7 +62188,7 @@
       </c>
       <c r="J1199" s="6"/>
       <c r="L1199" s="3" t="s">
-        <v>2455</v>
+        <v>2439</v>
       </c>
       <c r="M1199">
         <v>2</v>
@@ -62234,7 +62234,7 @@
       </c>
       <c r="J1200" s="6"/>
       <c r="L1200" s="3" t="s">
-        <v>2456</v>
+        <v>2440</v>
       </c>
       <c r="M1200">
         <v>2</v>
@@ -62280,7 +62280,7 @@
       </c>
       <c r="J1201" s="6"/>
       <c r="L1201" s="3" t="s">
-        <v>2457</v>
+        <v>2441</v>
       </c>
       <c r="M1201">
         <v>2</v>
@@ -62326,7 +62326,7 @@
       </c>
       <c r="J1202" s="6"/>
       <c r="L1202" s="3" t="s">
-        <v>2458</v>
+        <v>2442</v>
       </c>
       <c r="M1202">
         <v>2</v>
@@ -62372,7 +62372,7 @@
       </c>
       <c r="J1203" s="6"/>
       <c r="L1203" s="3" t="s">
-        <v>2459</v>
+        <v>2443</v>
       </c>
       <c r="M1203">
         <v>2</v>
@@ -62418,7 +62418,7 @@
       </c>
       <c r="J1204" s="6"/>
       <c r="L1204" s="3" t="s">
-        <v>2460</v>
+        <v>2444</v>
       </c>
       <c r="M1204">
         <v>2</v>
@@ -62464,7 +62464,7 @@
       </c>
       <c r="J1205" s="6"/>
       <c r="L1205" s="3" t="s">
-        <v>2461</v>
+        <v>2445</v>
       </c>
       <c r="M1205">
         <v>2</v>
@@ -62510,7 +62510,7 @@
       </c>
       <c r="J1206" s="6"/>
       <c r="L1206" s="3" t="s">
-        <v>2462</v>
+        <v>2446</v>
       </c>
       <c r="M1206">
         <v>2</v>
@@ -62556,7 +62556,7 @@
       </c>
       <c r="J1207" s="6"/>
       <c r="L1207" s="3" t="s">
-        <v>2463</v>
+        <v>2447</v>
       </c>
       <c r="M1207">
         <v>2</v>
@@ -62602,7 +62602,7 @@
       </c>
       <c r="J1208" s="6"/>
       <c r="L1208" s="3" t="s">
-        <v>2464</v>
+        <v>2448</v>
       </c>
       <c r="M1208">
         <v>2</v>
@@ -62648,7 +62648,7 @@
       </c>
       <c r="J1209" s="6"/>
       <c r="L1209" s="3" t="s">
-        <v>2465</v>
+        <v>2449</v>
       </c>
       <c r="M1209">
         <v>2</v>
@@ -62694,7 +62694,7 @@
       </c>
       <c r="J1210" s="6"/>
       <c r="L1210" s="3" t="s">
-        <v>2466</v>
+        <v>2450</v>
       </c>
       <c r="M1210">
         <v>2</v>
@@ -62740,7 +62740,7 @@
       </c>
       <c r="J1211" s="6"/>
       <c r="L1211" s="3" t="s">
-        <v>2467</v>
+        <v>2451</v>
       </c>
       <c r="M1211">
         <v>2</v>
@@ -62786,7 +62786,7 @@
       </c>
       <c r="J1212" s="6"/>
       <c r="L1212" s="3" t="s">
-        <v>2468</v>
+        <v>2452</v>
       </c>
       <c r="M1212">
         <v>2</v>
@@ -62832,7 +62832,7 @@
       </c>
       <c r="J1213" s="6"/>
       <c r="L1213" s="3" t="s">
-        <v>2469</v>
+        <v>2453</v>
       </c>
       <c r="M1213">
         <v>2</v>
@@ -62878,7 +62878,7 @@
       </c>
       <c r="J1214" s="6"/>
       <c r="L1214" s="3" t="s">
-        <v>2470</v>
+        <v>2454</v>
       </c>
       <c r="M1214">
         <v>2</v>
@@ -62924,7 +62924,7 @@
       </c>
       <c r="J1215" s="6"/>
       <c r="L1215" s="3" t="s">
-        <v>2471</v>
+        <v>2455</v>
       </c>
       <c r="M1215">
         <v>2</v>
@@ -62970,7 +62970,7 @@
       </c>
       <c r="J1216" s="6"/>
       <c r="L1216" s="3" t="s">
-        <v>2472</v>
+        <v>2456</v>
       </c>
       <c r="M1216">
         <v>2</v>
@@ -63016,7 +63016,7 @@
       </c>
       <c r="J1217" s="6"/>
       <c r="L1217" s="3" t="s">
-        <v>2473</v>
+        <v>2457</v>
       </c>
       <c r="M1217">
         <v>2</v>
@@ -63062,7 +63062,7 @@
       </c>
       <c r="J1218" s="6"/>
       <c r="L1218" s="3" t="s">
-        <v>2474</v>
+        <v>2458</v>
       </c>
       <c r="M1218">
         <v>2</v>
@@ -63108,7 +63108,7 @@
       </c>
       <c r="J1219" s="6"/>
       <c r="L1219" s="3" t="s">
-        <v>2475</v>
+        <v>2459</v>
       </c>
       <c r="M1219">
         <v>2</v>
@@ -63154,7 +63154,7 @@
       </c>
       <c r="J1220" s="6"/>
       <c r="L1220" s="3" t="s">
-        <v>2476</v>
+        <v>2460</v>
       </c>
       <c r="M1220">
         <v>2</v>
@@ -63200,7 +63200,7 @@
       </c>
       <c r="J1221" s="6"/>
       <c r="L1221" s="3" t="s">
-        <v>2477</v>
+        <v>2461</v>
       </c>
       <c r="M1221">
         <v>2</v>
@@ -63246,7 +63246,7 @@
       </c>
       <c r="J1222" s="6"/>
       <c r="L1222" s="3" t="s">
-        <v>2478</v>
+        <v>2462</v>
       </c>
       <c r="M1222">
         <v>2</v>
@@ -63292,7 +63292,7 @@
       </c>
       <c r="J1223" s="6"/>
       <c r="L1223" s="3" t="s">
-        <v>2479</v>
+        <v>2463</v>
       </c>
       <c r="M1223">
         <v>2</v>
@@ -63338,7 +63338,7 @@
       </c>
       <c r="J1224" s="6"/>
       <c r="L1224" s="3" t="s">
-        <v>2484</v>
+        <v>2468</v>
       </c>
       <c r="M1224">
         <v>2</v>
@@ -63384,7 +63384,7 @@
       </c>
       <c r="J1225" s="6"/>
       <c r="L1225" s="3" t="s">
-        <v>2485</v>
+        <v>2469</v>
       </c>
       <c r="M1225">
         <v>2</v>
@@ -63430,7 +63430,7 @@
       </c>
       <c r="J1226" s="6"/>
       <c r="L1226" s="3" t="s">
-        <v>2486</v>
+        <v>2470</v>
       </c>
       <c r="M1226">
         <v>2</v>
@@ -63476,7 +63476,7 @@
       </c>
       <c r="J1227" s="6"/>
       <c r="L1227" s="3" t="s">
-        <v>2487</v>
+        <v>2471</v>
       </c>
       <c r="M1227">
         <v>2</v>
@@ -63522,7 +63522,7 @@
       </c>
       <c r="J1228" s="6"/>
       <c r="L1228" s="3" t="s">
-        <v>2480</v>
+        <v>2464</v>
       </c>
       <c r="M1228">
         <v>2</v>
@@ -63568,7 +63568,7 @@
       </c>
       <c r="J1229" s="6"/>
       <c r="L1229" s="3" t="s">
-        <v>2481</v>
+        <v>2465</v>
       </c>
       <c r="M1229">
         <v>2</v>
@@ -63614,7 +63614,7 @@
       </c>
       <c r="J1230" s="6"/>
       <c r="L1230" s="3" t="s">
-        <v>2482</v>
+        <v>2466</v>
       </c>
       <c r="M1230">
         <v>2</v>
@@ -63660,7 +63660,7 @@
       </c>
       <c r="J1231" s="6"/>
       <c r="L1231" s="3" t="s">
-        <v>2483</v>
+        <v>2467</v>
       </c>
       <c r="M1231">
         <v>2</v>
@@ -63706,7 +63706,7 @@
       </c>
       <c r="J1232" s="6"/>
       <c r="L1232" s="3" t="s">
-        <v>2488</v>
+        <v>2472</v>
       </c>
       <c r="M1232">
         <v>2</v>
@@ -63752,7 +63752,7 @@
       </c>
       <c r="J1233" s="6"/>
       <c r="L1233" s="3" t="s">
-        <v>2489</v>
+        <v>2473</v>
       </c>
       <c r="M1233">
         <v>2</v>
@@ -63798,7 +63798,7 @@
       </c>
       <c r="J1234" s="6"/>
       <c r="L1234" s="3" t="s">
-        <v>2490</v>
+        <v>2474</v>
       </c>
       <c r="M1234">
         <v>2</v>
@@ -63844,7 +63844,7 @@
       </c>
       <c r="J1235" s="6"/>
       <c r="L1235" s="3" t="s">
-        <v>2491</v>
+        <v>2475</v>
       </c>
       <c r="M1235">
         <v>2</v>
@@ -63890,7 +63890,7 @@
       </c>
       <c r="J1236" s="6"/>
       <c r="L1236" s="3" t="s">
-        <v>2492</v>
+        <v>2476</v>
       </c>
       <c r="M1236">
         <v>2</v>
@@ -63936,7 +63936,7 @@
       </c>
       <c r="J1237" s="6"/>
       <c r="L1237" s="3" t="s">
-        <v>2493</v>
+        <v>2477</v>
       </c>
       <c r="M1237">
         <v>2</v>
@@ -63982,7 +63982,7 @@
       </c>
       <c r="J1238" s="6"/>
       <c r="L1238" s="3" t="s">
-        <v>2494</v>
+        <v>2478</v>
       </c>
       <c r="M1238">
         <v>2</v>
@@ -64028,7 +64028,7 @@
       </c>
       <c r="J1239" s="6"/>
       <c r="L1239" s="3" t="s">
-        <v>2495</v>
+        <v>2479</v>
       </c>
       <c r="M1239">
         <v>2</v>
@@ -64074,7 +64074,7 @@
       </c>
       <c r="J1240" s="6"/>
       <c r="L1240" s="3" t="s">
-        <v>2496</v>
+        <v>2480</v>
       </c>
       <c r="M1240">
         <v>2</v>
@@ -64120,7 +64120,7 @@
       </c>
       <c r="J1241" s="6"/>
       <c r="L1241" s="3" t="s">
-        <v>2499</v>
+        <v>2483</v>
       </c>
       <c r="M1241">
         <v>2</v>
@@ -64166,7 +64166,7 @@
       </c>
       <c r="J1242" s="6"/>
       <c r="L1242" s="3" t="s">
-        <v>2500</v>
+        <v>2484</v>
       </c>
       <c r="M1242">
         <v>2</v>
@@ -64212,7 +64212,7 @@
       </c>
       <c r="J1243" s="6"/>
       <c r="L1243" s="3" t="s">
-        <v>2501</v>
+        <v>2485</v>
       </c>
       <c r="M1243">
         <v>2</v>
@@ -64258,7 +64258,7 @@
       </c>
       <c r="J1244" s="6"/>
       <c r="L1244" s="3" t="s">
-        <v>2502</v>
+        <v>2486</v>
       </c>
       <c r="M1244">
         <v>2</v>
@@ -64304,7 +64304,7 @@
       </c>
       <c r="J1245" s="6"/>
       <c r="L1245" s="3" t="s">
-        <v>2503</v>
+        <v>2487</v>
       </c>
       <c r="M1245">
         <v>2</v>
@@ -64350,7 +64350,7 @@
       </c>
       <c r="J1246" s="6"/>
       <c r="L1246" s="3" t="s">
-        <v>2504</v>
+        <v>2488</v>
       </c>
       <c r="M1246">
         <v>2</v>
@@ -64396,7 +64396,7 @@
       </c>
       <c r="J1247" s="6"/>
       <c r="L1247" s="3" t="s">
-        <v>2505</v>
+        <v>2489</v>
       </c>
       <c r="M1247">
         <v>2</v>
@@ -64442,7 +64442,7 @@
       </c>
       <c r="J1248" s="6"/>
       <c r="L1248" s="3" t="s">
-        <v>2497</v>
+        <v>2481</v>
       </c>
       <c r="M1248">
         <v>2</v>
@@ -64488,7 +64488,7 @@
       </c>
       <c r="J1249" s="6"/>
       <c r="L1249" s="3" t="s">
-        <v>2498</v>
+        <v>2482</v>
       </c>
       <c r="M1249">
         <v>2</v>
@@ -64534,7 +64534,7 @@
       </c>
       <c r="J1250" s="6"/>
       <c r="L1250" s="3" t="s">
-        <v>2506</v>
+        <v>2490</v>
       </c>
       <c r="M1250">
         <v>2</v>
@@ -64580,7 +64580,7 @@
       </c>
       <c r="J1251" s="6"/>
       <c r="L1251" s="3" t="s">
-        <v>2507</v>
+        <v>2491</v>
       </c>
       <c r="M1251">
         <v>2</v>
@@ -64626,7 +64626,7 @@
       </c>
       <c r="J1252" s="6"/>
       <c r="L1252" s="3" t="s">
-        <v>2508</v>
+        <v>2492</v>
       </c>
       <c r="M1252">
         <v>2</v>
@@ -64672,7 +64672,7 @@
       </c>
       <c r="J1253" s="6"/>
       <c r="L1253" s="3" t="s">
-        <v>2509</v>
+        <v>2493</v>
       </c>
       <c r="M1253">
         <v>2</v>
@@ -64718,7 +64718,7 @@
       </c>
       <c r="J1254" s="6"/>
       <c r="L1254" s="3" t="s">
-        <v>2510</v>
+        <v>2494</v>
       </c>
       <c r="M1254">
         <v>2</v>
@@ -64764,7 +64764,7 @@
       </c>
       <c r="J1255" s="6"/>
       <c r="L1255" s="3" t="s">
-        <v>2511</v>
+        <v>2495</v>
       </c>
       <c r="M1255">
         <v>2</v>
@@ -64810,7 +64810,7 @@
       </c>
       <c r="J1256" s="6"/>
       <c r="L1256" s="3" t="s">
-        <v>2516</v>
+        <v>2500</v>
       </c>
       <c r="M1256">
         <v>2</v>
@@ -64856,7 +64856,7 @@
       </c>
       <c r="J1257" s="6"/>
       <c r="L1257" s="3" t="s">
-        <v>2517</v>
+        <v>2501</v>
       </c>
       <c r="M1257">
         <v>2</v>
@@ -64902,7 +64902,7 @@
       </c>
       <c r="J1258" s="6"/>
       <c r="L1258" s="3" t="s">
-        <v>2518</v>
+        <v>2502</v>
       </c>
       <c r="M1258">
         <v>2</v>
@@ -64948,7 +64948,7 @@
       </c>
       <c r="J1259" s="6"/>
       <c r="L1259" s="3" t="s">
-        <v>2519</v>
+        <v>2503</v>
       </c>
       <c r="M1259">
         <v>2</v>
@@ -64994,7 +64994,7 @@
       </c>
       <c r="J1260" s="6"/>
       <c r="L1260" s="3" t="s">
-        <v>2512</v>
+        <v>2496</v>
       </c>
       <c r="M1260">
         <v>2</v>
@@ -65040,7 +65040,7 @@
       </c>
       <c r="J1261" s="6"/>
       <c r="L1261" s="3" t="s">
-        <v>2513</v>
+        <v>2497</v>
       </c>
       <c r="M1261">
         <v>2</v>
@@ -65086,7 +65086,7 @@
       </c>
       <c r="J1262" s="6"/>
       <c r="L1262" s="3" t="s">
-        <v>2514</v>
+        <v>2498</v>
       </c>
       <c r="M1262">
         <v>2</v>
@@ -65132,7 +65132,7 @@
       </c>
       <c r="J1263" s="6"/>
       <c r="L1263" s="3" t="s">
-        <v>2515</v>
+        <v>2499</v>
       </c>
       <c r="M1263">
         <v>2</v>
@@ -65178,7 +65178,7 @@
       </c>
       <c r="J1264" s="6"/>
       <c r="L1264" s="3" t="s">
-        <v>2520</v>
+        <v>2504</v>
       </c>
       <c r="M1264">
         <v>2</v>
@@ -65224,7 +65224,7 @@
       </c>
       <c r="J1265" s="6"/>
       <c r="L1265" s="3" t="s">
-        <v>2521</v>
+        <v>2505</v>
       </c>
       <c r="M1265">
         <v>2</v>
@@ -65270,7 +65270,7 @@
       </c>
       <c r="J1266" s="6"/>
       <c r="L1266" s="3" t="s">
-        <v>2522</v>
+        <v>2506</v>
       </c>
       <c r="M1266">
         <v>2</v>
@@ -65316,7 +65316,7 @@
       </c>
       <c r="J1267" s="6"/>
       <c r="L1267" s="3" t="s">
-        <v>2523</v>
+        <v>2507</v>
       </c>
       <c r="M1267">
         <v>2</v>
@@ -65362,7 +65362,7 @@
       </c>
       <c r="J1268" s="6"/>
       <c r="L1268" s="3" t="s">
-        <v>2524</v>
+        <v>2508</v>
       </c>
       <c r="M1268">
         <v>2</v>
@@ -65408,7 +65408,7 @@
       </c>
       <c r="J1269" s="6"/>
       <c r="L1269" s="3" t="s">
-        <v>2525</v>
+        <v>2509</v>
       </c>
       <c r="M1269">
         <v>2</v>
@@ -65454,7 +65454,7 @@
       </c>
       <c r="J1270" s="6"/>
       <c r="L1270" s="3" t="s">
-        <v>2526</v>
+        <v>2510</v>
       </c>
       <c r="M1270">
         <v>2</v>
@@ -65500,7 +65500,7 @@
       </c>
       <c r="J1271" s="6"/>
       <c r="L1271" s="3" t="s">
-        <v>2527</v>
+        <v>2511</v>
       </c>
       <c r="M1271">
         <v>2</v>
@@ -65546,7 +65546,7 @@
       </c>
       <c r="J1272" s="6"/>
       <c r="L1272" s="3" t="s">
-        <v>2528</v>
+        <v>2512</v>
       </c>
       <c r="M1272">
         <v>2</v>
@@ -65592,7 +65592,7 @@
       </c>
       <c r="J1273" s="6"/>
       <c r="L1273" s="3" t="s">
-        <v>2529</v>
+        <v>2513</v>
       </c>
       <c r="M1273">
         <v>2</v>
@@ -65638,7 +65638,7 @@
       </c>
       <c r="J1274" s="6"/>
       <c r="L1274" s="3" t="s">
-        <v>2530</v>
+        <v>2514</v>
       </c>
       <c r="M1274">
         <v>2</v>
@@ -65684,7 +65684,7 @@
       </c>
       <c r="J1275" s="6"/>
       <c r="L1275" s="3" t="s">
-        <v>2531</v>
+        <v>2515</v>
       </c>
       <c r="M1275">
         <v>2</v>
@@ -65730,7 +65730,7 @@
       </c>
       <c r="J1276" s="6"/>
       <c r="L1276" s="3" t="s">
-        <v>2532</v>
+        <v>2516</v>
       </c>
       <c r="M1276">
         <v>2</v>
@@ -65776,7 +65776,7 @@
       </c>
       <c r="J1277" s="6"/>
       <c r="L1277" s="3" t="s">
-        <v>2533</v>
+        <v>2517</v>
       </c>
       <c r="M1277">
         <v>2</v>
@@ -65822,7 +65822,7 @@
       </c>
       <c r="J1278" s="6"/>
       <c r="L1278" s="3" t="s">
-        <v>2534</v>
+        <v>2518</v>
       </c>
       <c r="M1278">
         <v>2</v>
@@ -65868,7 +65868,7 @@
       </c>
       <c r="J1279" s="6"/>
       <c r="L1279" s="3" t="s">
-        <v>2535</v>
+        <v>2519</v>
       </c>
       <c r="M1279">
         <v>2</v>
@@ -65914,7 +65914,7 @@
       </c>
       <c r="J1280" s="6"/>
       <c r="L1280" s="3" t="s">
-        <v>2536</v>
+        <v>2520</v>
       </c>
       <c r="M1280">
         <v>2</v>
@@ -65960,7 +65960,7 @@
       </c>
       <c r="J1281" s="6"/>
       <c r="L1281" s="3" t="s">
-        <v>2537</v>
+        <v>2521</v>
       </c>
       <c r="M1281">
         <v>2</v>
@@ -66006,7 +66006,7 @@
       </c>
       <c r="J1282" s="6"/>
       <c r="L1282" s="3" t="s">
-        <v>2538</v>
+        <v>2522</v>
       </c>
       <c r="M1282">
         <v>2</v>
@@ -66052,7 +66052,7 @@
       </c>
       <c r="J1283" s="6"/>
       <c r="L1283" s="3" t="s">
-        <v>2539</v>
+        <v>2523</v>
       </c>
       <c r="M1283">
         <v>2</v>
@@ -66098,7 +66098,7 @@
       </c>
       <c r="J1284" s="6"/>
       <c r="L1284" s="3" t="s">
-        <v>2540</v>
+        <v>2524</v>
       </c>
       <c r="M1284">
         <v>2</v>
@@ -66144,7 +66144,7 @@
       </c>
       <c r="J1285" s="6"/>
       <c r="L1285" s="3" t="s">
-        <v>2541</v>
+        <v>2525</v>
       </c>
       <c r="M1285">
         <v>2</v>
@@ -66190,7 +66190,7 @@
       </c>
       <c r="J1286" s="6"/>
       <c r="L1286" s="3" t="s">
-        <v>2542</v>
+        <v>2526</v>
       </c>
       <c r="M1286">
         <v>2</v>
@@ -66236,7 +66236,7 @@
       </c>
       <c r="J1287" s="6"/>
       <c r="L1287" s="3" t="s">
-        <v>2543</v>
+        <v>2527</v>
       </c>
       <c r="M1287">
         <v>2</v>
@@ -66282,7 +66282,7 @@
       </c>
       <c r="J1288" s="6"/>
       <c r="L1288" s="3" t="s">
-        <v>2544</v>
+        <v>2528</v>
       </c>
       <c r="M1288">
         <v>2</v>
@@ -66328,7 +66328,7 @@
       </c>
       <c r="J1289" s="6"/>
       <c r="L1289" s="3" t="s">
-        <v>2545</v>
+        <v>2529</v>
       </c>
       <c r="M1289">
         <v>2</v>
@@ -66374,7 +66374,7 @@
       </c>
       <c r="J1290" s="6"/>
       <c r="L1290" s="3" t="s">
-        <v>2546</v>
+        <v>2530</v>
       </c>
       <c r="M1290">
         <v>2</v>
@@ -66420,7 +66420,7 @@
       </c>
       <c r="J1291" s="6"/>
       <c r="L1291" s="3" t="s">
-        <v>2547</v>
+        <v>2531</v>
       </c>
       <c r="M1291">
         <v>2</v>
@@ -66466,7 +66466,7 @@
       </c>
       <c r="J1292" s="6"/>
       <c r="L1292" s="3" t="s">
-        <v>2548</v>
+        <v>2532</v>
       </c>
       <c r="M1292">
         <v>2</v>
@@ -66512,7 +66512,7 @@
       </c>
       <c r="J1293" s="6"/>
       <c r="L1293" s="3" t="s">
-        <v>2549</v>
+        <v>2533</v>
       </c>
       <c r="M1293">
         <v>2</v>
@@ -66558,7 +66558,7 @@
       </c>
       <c r="J1294" s="6"/>
       <c r="L1294" s="3" t="s">
-        <v>2550</v>
+        <v>2534</v>
       </c>
       <c r="M1294">
         <v>2</v>
@@ -66604,7 +66604,7 @@
       </c>
       <c r="J1295" s="6"/>
       <c r="L1295" s="3" t="s">
-        <v>2558</v>
+        <v>2542</v>
       </c>
       <c r="M1295">
         <v>2</v>
@@ -66650,7 +66650,7 @@
       </c>
       <c r="J1296" s="6"/>
       <c r="L1296" s="3" t="s">
-        <v>2551</v>
+        <v>2535</v>
       </c>
       <c r="M1296">
         <v>2</v>
@@ -66696,7 +66696,7 @@
       </c>
       <c r="J1297" s="6"/>
       <c r="L1297" s="3" t="s">
-        <v>2552</v>
+        <v>2536</v>
       </c>
       <c r="M1297">
         <v>2</v>
@@ -66742,7 +66742,7 @@
       </c>
       <c r="J1298" s="6"/>
       <c r="L1298" s="3" t="s">
-        <v>2553</v>
+        <v>2537</v>
       </c>
       <c r="M1298">
         <v>2</v>
@@ -66788,7 +66788,7 @@
       </c>
       <c r="J1299" s="6"/>
       <c r="L1299" s="3" t="s">
-        <v>2554</v>
+        <v>2538</v>
       </c>
       <c r="M1299">
         <v>2</v>
@@ -66834,7 +66834,7 @@
       </c>
       <c r="J1300" s="6"/>
       <c r="L1300" s="3" t="s">
-        <v>2555</v>
+        <v>2539</v>
       </c>
       <c r="M1300">
         <v>2</v>
@@ -66880,7 +66880,7 @@
       </c>
       <c r="J1301" s="6"/>
       <c r="L1301" s="3" t="s">
-        <v>2556</v>
+        <v>2540</v>
       </c>
       <c r="M1301">
         <v>2</v>
@@ -66926,7 +66926,7 @@
       </c>
       <c r="J1302" s="6"/>
       <c r="L1302" s="3" t="s">
-        <v>2557</v>
+        <v>2541</v>
       </c>
       <c r="M1302">
         <v>2</v>
@@ -66972,7 +66972,7 @@
       </c>
       <c r="J1303" s="6"/>
       <c r="L1303" s="3" t="s">
-        <v>2559</v>
+        <v>2543</v>
       </c>
       <c r="M1303">
         <v>2</v>
@@ -67018,7 +67018,7 @@
       </c>
       <c r="J1304" s="6"/>
       <c r="L1304" s="3" t="s">
-        <v>2560</v>
+        <v>2544</v>
       </c>
       <c r="M1304">
         <v>2</v>
@@ -67064,7 +67064,7 @@
       </c>
       <c r="J1305" s="6"/>
       <c r="L1305" s="3" t="s">
-        <v>2561</v>
+        <v>2545</v>
       </c>
       <c r="M1305">
         <v>2</v>
@@ -67110,7 +67110,7 @@
       </c>
       <c r="J1306" s="6"/>
       <c r="L1306" s="3" t="s">
-        <v>2562</v>
+        <v>2546</v>
       </c>
       <c r="M1306">
         <v>2</v>
@@ -67156,7 +67156,7 @@
       </c>
       <c r="J1307" s="6"/>
       <c r="L1307" s="3" t="s">
-        <v>2563</v>
+        <v>2547</v>
       </c>
       <c r="M1307">
         <v>2</v>
@@ -67202,7 +67202,7 @@
       </c>
       <c r="J1308" s="6"/>
       <c r="L1308" s="3" t="s">
-        <v>2564</v>
+        <v>2548</v>
       </c>
       <c r="M1308">
         <v>2</v>
@@ -67248,7 +67248,7 @@
       </c>
       <c r="J1309" s="6"/>
       <c r="L1309" s="3" t="s">
-        <v>2565</v>
+        <v>2549</v>
       </c>
       <c r="M1309">
         <v>2</v>
@@ -67294,7 +67294,7 @@
       </c>
       <c r="J1310" s="6"/>
       <c r="L1310" s="3" t="s">
-        <v>2566</v>
+        <v>2550</v>
       </c>
       <c r="M1310">
         <v>2</v>
@@ -67340,7 +67340,7 @@
       </c>
       <c r="J1311" s="6"/>
       <c r="L1311" s="3" t="s">
-        <v>2567</v>
+        <v>2551</v>
       </c>
       <c r="M1311">
         <v>2</v>
@@ -67386,7 +67386,7 @@
       </c>
       <c r="J1312" s="6"/>
       <c r="L1312" s="3" t="s">
-        <v>2568</v>
+        <v>2552</v>
       </c>
       <c r="M1312">
         <v>2</v>
@@ -67432,7 +67432,7 @@
       </c>
       <c r="J1313" s="6"/>
       <c r="L1313" s="3" t="s">
-        <v>2569</v>
+        <v>2553</v>
       </c>
       <c r="M1313">
         <v>2</v>
@@ -67478,7 +67478,7 @@
       </c>
       <c r="J1314" s="6"/>
       <c r="L1314" s="3" t="s">
-        <v>2570</v>
+        <v>2554</v>
       </c>
       <c r="M1314">
         <v>2</v>
@@ -67524,7 +67524,7 @@
       </c>
       <c r="J1315" s="6"/>
       <c r="L1315" s="3" t="s">
-        <v>2571</v>
+        <v>2555</v>
       </c>
       <c r="M1315">
         <v>2</v>
@@ -67570,7 +67570,7 @@
       </c>
       <c r="J1316" s="6"/>
       <c r="L1316" s="3" t="s">
-        <v>2572</v>
+        <v>2556</v>
       </c>
       <c r="M1316">
         <v>2</v>
@@ -67616,7 +67616,7 @@
       </c>
       <c r="J1317" s="6"/>
       <c r="L1317" s="3" t="s">
-        <v>2573</v>
+        <v>2557</v>
       </c>
       <c r="M1317">
         <v>2</v>
@@ -67662,7 +67662,7 @@
       </c>
       <c r="J1318" s="6"/>
       <c r="L1318" s="3" t="s">
-        <v>2574</v>
+        <v>2558</v>
       </c>
       <c r="M1318">
         <v>2</v>
@@ -67708,7 +67708,7 @@
       </c>
       <c r="J1319" s="6"/>
       <c r="L1319" s="3" t="s">
-        <v>2575</v>
+        <v>2559</v>
       </c>
       <c r="M1319">
         <v>2</v>
@@ -67754,7 +67754,7 @@
       </c>
       <c r="J1320" s="6"/>
       <c r="L1320" s="3" t="s">
-        <v>2576</v>
+        <v>2560</v>
       </c>
       <c r="M1320">
         <v>2</v>
@@ -67800,7 +67800,7 @@
       </c>
       <c r="J1321" s="6"/>
       <c r="L1321" s="3" t="s">
-        <v>2577</v>
+        <v>2561</v>
       </c>
       <c r="M1321">
         <v>2</v>
@@ -67846,7 +67846,7 @@
       </c>
       <c r="J1322" s="6"/>
       <c r="L1322" s="3" t="s">
-        <v>2578</v>
+        <v>2562</v>
       </c>
       <c r="M1322">
         <v>2</v>
@@ -67892,7 +67892,7 @@
       </c>
       <c r="J1323" s="6"/>
       <c r="L1323" s="3" t="s">
-        <v>2579</v>
+        <v>2563</v>
       </c>
       <c r="M1323">
         <v>2</v>
@@ -67938,7 +67938,7 @@
       </c>
       <c r="J1324" s="6"/>
       <c r="L1324" s="3" t="s">
-        <v>2580</v>
+        <v>2564</v>
       </c>
       <c r="M1324">
         <v>2</v>
@@ -67984,7 +67984,7 @@
       </c>
       <c r="J1325" s="6"/>
       <c r="L1325" s="3" t="s">
-        <v>2581</v>
+        <v>2565</v>
       </c>
       <c r="M1325">
         <v>2</v>
@@ -68030,7 +68030,7 @@
       </c>
       <c r="J1326" s="6"/>
       <c r="L1326" s="3" t="s">
-        <v>2582</v>
+        <v>2566</v>
       </c>
       <c r="M1326">
         <v>2</v>
@@ -68076,7 +68076,7 @@
       </c>
       <c r="J1327" s="6"/>
       <c r="L1327" s="3" t="s">
-        <v>2588</v>
+        <v>2572</v>
       </c>
       <c r="M1327">
         <v>2</v>
@@ -68122,7 +68122,7 @@
       </c>
       <c r="J1328" s="6"/>
       <c r="L1328" s="3" t="s">
-        <v>2583</v>
+        <v>2567</v>
       </c>
       <c r="M1328">
         <v>2</v>
@@ -68168,7 +68168,7 @@
       </c>
       <c r="J1329" s="6"/>
       <c r="L1329" s="3" t="s">
-        <v>2584</v>
+        <v>2568</v>
       </c>
       <c r="M1329">
         <v>2</v>
@@ -68214,7 +68214,7 @@
       </c>
       <c r="J1330" s="6"/>
       <c r="L1330" s="3" t="s">
-        <v>2585</v>
+        <v>2569</v>
       </c>
       <c r="M1330">
         <v>2</v>
@@ -68260,7 +68260,7 @@
       </c>
       <c r="J1331" s="6"/>
       <c r="L1331" s="3" t="s">
-        <v>2586</v>
+        <v>2570</v>
       </c>
       <c r="M1331">
         <v>2</v>
@@ -68306,7 +68306,7 @@
       </c>
       <c r="J1332" s="6"/>
       <c r="L1332" s="3" t="s">
-        <v>2587</v>
+        <v>2571</v>
       </c>
       <c r="M1332">
         <v>2</v>
@@ -68352,7 +68352,7 @@
       </c>
       <c r="J1333" s="6"/>
       <c r="L1333" s="3" t="s">
-        <v>2589</v>
+        <v>2573</v>
       </c>
       <c r="M1333">
         <v>2</v>
@@ -68398,7 +68398,7 @@
       </c>
       <c r="J1334" s="6"/>
       <c r="L1334" s="3" t="s">
-        <v>2590</v>
+        <v>2574</v>
       </c>
       <c r="M1334">
         <v>2</v>
@@ -68444,7 +68444,7 @@
       </c>
       <c r="J1335" s="6"/>
       <c r="L1335" s="3" t="s">
-        <v>2591</v>
+        <v>2575</v>
       </c>
       <c r="M1335">
         <v>2</v>
@@ -68490,7 +68490,7 @@
       </c>
       <c r="J1336" s="6"/>
       <c r="L1336" s="3" t="s">
-        <v>2592</v>
+        <v>2576</v>
       </c>
       <c r="M1336">
         <v>2</v>
@@ -68536,7 +68536,7 @@
       </c>
       <c r="J1337" s="6"/>
       <c r="L1337" s="3" t="s">
-        <v>2601</v>
+        <v>2585</v>
       </c>
       <c r="M1337">
         <v>2</v>
@@ -68582,7 +68582,7 @@
       </c>
       <c r="J1338" s="6"/>
       <c r="L1338" s="3" t="s">
-        <v>2602</v>
+        <v>2586</v>
       </c>
       <c r="M1338">
         <v>2</v>
@@ -68628,7 +68628,7 @@
       </c>
       <c r="J1339" s="6"/>
       <c r="L1339" s="3" t="s">
-        <v>2603</v>
+        <v>2587</v>
       </c>
       <c r="M1339">
         <v>2</v>
@@ -68674,7 +68674,7 @@
       </c>
       <c r="J1340" s="6"/>
       <c r="L1340" s="3" t="s">
-        <v>2604</v>
+        <v>2588</v>
       </c>
       <c r="M1340">
         <v>2</v>
@@ -68720,7 +68720,7 @@
       </c>
       <c r="J1341" s="6"/>
       <c r="L1341" s="3" t="s">
-        <v>2605</v>
+        <v>2589</v>
       </c>
       <c r="M1341">
         <v>2</v>
@@ -68766,7 +68766,7 @@
       </c>
       <c r="J1342" s="6"/>
       <c r="L1342" s="3" t="s">
-        <v>2606</v>
+        <v>2590</v>
       </c>
       <c r="M1342">
         <v>2</v>
@@ -68812,7 +68812,7 @@
       </c>
       <c r="J1343" s="6"/>
       <c r="L1343" s="3" t="s">
-        <v>2593</v>
+        <v>2577</v>
       </c>
       <c r="M1343">
         <v>2</v>
@@ -68858,7 +68858,7 @@
       </c>
       <c r="J1344" s="6"/>
       <c r="L1344" s="3" t="s">
-        <v>2594</v>
+        <v>2578</v>
       </c>
       <c r="M1344">
         <v>2</v>
@@ -68904,7 +68904,7 @@
       </c>
       <c r="J1345" s="6"/>
       <c r="L1345" s="3" t="s">
-        <v>2595</v>
+        <v>2579</v>
       </c>
       <c r="M1345">
         <v>2</v>
@@ -68950,7 +68950,7 @@
       </c>
       <c r="J1346" s="6"/>
       <c r="L1346" s="3" t="s">
-        <v>2596</v>
+        <v>2580</v>
       </c>
       <c r="M1346">
         <v>2</v>
@@ -68996,7 +68996,7 @@
       </c>
       <c r="J1347" s="6"/>
       <c r="L1347" s="3" t="s">
-        <v>2597</v>
+        <v>2581</v>
       </c>
       <c r="M1347">
         <v>2</v>
@@ -69042,7 +69042,7 @@
       </c>
       <c r="J1348" s="6"/>
       <c r="L1348" s="3" t="s">
-        <v>2598</v>
+        <v>2582</v>
       </c>
       <c r="M1348">
         <v>2</v>
@@ -69088,7 +69088,7 @@
       </c>
       <c r="J1349" s="6"/>
       <c r="L1349" s="3" t="s">
-        <v>2599</v>
+        <v>2583</v>
       </c>
       <c r="M1349">
         <v>2</v>
@@ -69134,7 +69134,7 @@
       </c>
       <c r="J1350" s="6"/>
       <c r="L1350" s="3" t="s">
-        <v>2600</v>
+        <v>2584</v>
       </c>
       <c r="M1350">
         <v>2</v>
@@ -69180,7 +69180,7 @@
       </c>
       <c r="J1351" s="6"/>
       <c r="L1351" s="3" t="s">
-        <v>2607</v>
+        <v>2591</v>
       </c>
       <c r="M1351">
         <v>2</v>
@@ -69226,7 +69226,7 @@
       </c>
       <c r="J1352" s="6"/>
       <c r="L1352" s="3" t="s">
-        <v>2608</v>
+        <v>2592</v>
       </c>
       <c r="M1352">
         <v>2</v>
@@ -69272,7 +69272,7 @@
       </c>
       <c r="J1353" s="6"/>
       <c r="L1353" s="3" t="s">
-        <v>2611</v>
+        <v>2595</v>
       </c>
       <c r="M1353">
         <v>2</v>
@@ -69318,7 +69318,7 @@
       </c>
       <c r="J1354" s="6"/>
       <c r="L1354" s="3" t="s">
-        <v>2612</v>
+        <v>2596</v>
       </c>
       <c r="M1354">
         <v>2</v>
@@ -69364,7 +69364,7 @@
       </c>
       <c r="J1355" s="6"/>
       <c r="L1355" s="3" t="s">
-        <v>2613</v>
+        <v>2597</v>
       </c>
       <c r="M1355">
         <v>2</v>
@@ -69410,7 +69410,7 @@
       </c>
       <c r="J1356" s="6"/>
       <c r="L1356" s="3" t="s">
-        <v>2614</v>
+        <v>2598</v>
       </c>
       <c r="M1356">
         <v>2</v>
@@ -69456,7 +69456,7 @@
       </c>
       <c r="J1357" s="6"/>
       <c r="L1357" s="3" t="s">
-        <v>2615</v>
+        <v>2599</v>
       </c>
       <c r="M1357">
         <v>2</v>
@@ -69502,7 +69502,7 @@
       </c>
       <c r="J1358" s="6"/>
       <c r="L1358" s="3" t="s">
-        <v>2616</v>
+        <v>2600</v>
       </c>
       <c r="M1358">
         <v>2</v>
@@ -69548,7 +69548,7 @@
       </c>
       <c r="J1359" s="6"/>
       <c r="L1359" s="3" t="s">
-        <v>2609</v>
+        <v>2593</v>
       </c>
       <c r="M1359">
         <v>2</v>
@@ -69594,7 +69594,7 @@
       </c>
       <c r="J1360" s="6"/>
       <c r="L1360" s="3" t="s">
-        <v>2610</v>
+        <v>2594</v>
       </c>
       <c r="M1360">
         <v>2</v>
@@ -69640,7 +69640,7 @@
       </c>
       <c r="J1361" s="6"/>
       <c r="L1361" s="3" t="s">
-        <v>2617</v>
+        <v>2601</v>
       </c>
       <c r="M1361">
         <v>2</v>
@@ -69686,7 +69686,7 @@
       </c>
       <c r="J1362" s="6"/>
       <c r="L1362" s="3" t="s">
-        <v>2618</v>
+        <v>2602</v>
       </c>
       <c r="M1362">
         <v>2</v>
@@ -69732,7 +69732,7 @@
       </c>
       <c r="J1363" s="6"/>
       <c r="L1363" s="3" t="s">
-        <v>2619</v>
+        <v>2603</v>
       </c>
       <c r="M1363">
         <v>2</v>
@@ -69778,7 +69778,7 @@
       </c>
       <c r="J1364" s="6"/>
       <c r="L1364" s="3" t="s">
-        <v>2620</v>
+        <v>2604</v>
       </c>
       <c r="M1364">
         <v>2</v>
@@ -69824,7 +69824,7 @@
       </c>
       <c r="J1365" s="6"/>
       <c r="L1365" s="3" t="s">
-        <v>2621</v>
+        <v>2605</v>
       </c>
       <c r="M1365">
         <v>2</v>
@@ -69870,7 +69870,7 @@
       </c>
       <c r="J1366" s="6"/>
       <c r="L1366" s="3" t="s">
-        <v>2622</v>
+        <v>2606</v>
       </c>
       <c r="M1366">
         <v>2</v>
@@ -69916,7 +69916,7 @@
       </c>
       <c r="J1367" s="6"/>
       <c r="L1367" s="3" t="s">
-        <v>2623</v>
+        <v>2607</v>
       </c>
       <c r="M1367">
         <v>2</v>
@@ -69962,7 +69962,7 @@
       </c>
       <c r="J1368" s="6"/>
       <c r="L1368" s="3" t="s">
-        <v>2624</v>
+        <v>2608</v>
       </c>
       <c r="M1368">
         <v>2</v>
@@ -70008,7 +70008,7 @@
       </c>
       <c r="J1369" s="6"/>
       <c r="L1369" s="3" t="s">
-        <v>2625</v>
+        <v>2609</v>
       </c>
       <c r="M1369">
         <v>2</v>
@@ -70054,7 +70054,7 @@
       </c>
       <c r="J1370" s="6"/>
       <c r="L1370" s="3" t="s">
-        <v>2626</v>
+        <v>2610</v>
       </c>
       <c r="M1370">
         <v>2</v>
@@ -70100,7 +70100,7 @@
       </c>
       <c r="J1371" s="6"/>
       <c r="L1371" s="3" t="s">
-        <v>2627</v>
+        <v>2611</v>
       </c>
       <c r="M1371">
         <v>2</v>
@@ -70146,7 +70146,7 @@
       </c>
       <c r="J1372" s="6"/>
       <c r="L1372" s="3" t="s">
-        <v>2628</v>
+        <v>2612</v>
       </c>
       <c r="M1372">
         <v>2</v>
@@ -70192,7 +70192,7 @@
       </c>
       <c r="J1373" s="6"/>
       <c r="L1373" s="3" t="s">
-        <v>2629</v>
+        <v>2613</v>
       </c>
       <c r="M1373">
         <v>2</v>
@@ -70238,7 +70238,7 @@
       </c>
       <c r="J1374" s="6"/>
       <c r="L1374" s="3" t="s">
-        <v>2630</v>
+        <v>2614</v>
       </c>
       <c r="M1374">
         <v>2</v>
@@ -70284,7 +70284,7 @@
       </c>
       <c r="J1375" s="6"/>
       <c r="L1375" s="3" t="s">
-        <v>2631</v>
+        <v>2615</v>
       </c>
       <c r="M1375">
         <v>2</v>
@@ -70330,7 +70330,7 @@
       </c>
       <c r="J1376" s="6"/>
       <c r="L1376" s="3" t="s">
-        <v>2632</v>
+        <v>2616</v>
       </c>
       <c r="M1376">
         <v>2</v>
@@ -70376,7 +70376,7 @@
       </c>
       <c r="J1377" s="6"/>
       <c r="L1377" s="3" t="s">
-        <v>2633</v>
+        <v>2617</v>
       </c>
       <c r="M1377">
         <v>2</v>
@@ -70422,7 +70422,7 @@
       </c>
       <c r="J1378" s="6"/>
       <c r="L1378" s="3" t="s">
-        <v>2635</v>
+        <v>2619</v>
       </c>
       <c r="M1378">
         <v>2</v>
@@ -70468,7 +70468,7 @@
       </c>
       <c r="J1379" s="6"/>
       <c r="L1379" s="3" t="s">
-        <v>2636</v>
+        <v>2620</v>
       </c>
       <c r="M1379">
         <v>2</v>
@@ -70514,7 +70514,7 @@
       </c>
       <c r="J1380" s="6"/>
       <c r="L1380" s="3" t="s">
-        <v>2637</v>
+        <v>2621</v>
       </c>
       <c r="M1380">
         <v>2</v>
@@ -70560,7 +70560,7 @@
       </c>
       <c r="J1381" s="6"/>
       <c r="L1381" s="3" t="s">
-        <v>2638</v>
+        <v>2622</v>
       </c>
       <c r="M1381">
         <v>2</v>
@@ -70606,7 +70606,7 @@
       </c>
       <c r="J1382" s="6"/>
       <c r="L1382" s="3" t="s">
-        <v>2634</v>
+        <v>2618</v>
       </c>
       <c r="M1382">
         <v>2</v>
@@ -70652,7 +70652,7 @@
       </c>
       <c r="J1383" s="6"/>
       <c r="L1383" s="3" t="s">
-        <v>2639</v>
+        <v>2623</v>
       </c>
       <c r="M1383">
         <v>2</v>
@@ -70698,7 +70698,7 @@
       </c>
       <c r="J1384" s="6"/>
       <c r="L1384" s="3" t="s">
-        <v>2640</v>
+        <v>2624</v>
       </c>
       <c r="M1384">
         <v>2</v>
@@ -70744,7 +70744,7 @@
       </c>
       <c r="J1385" s="6"/>
       <c r="L1385" s="3" t="s">
-        <v>2649</v>
+        <v>2633</v>
       </c>
       <c r="M1385">
         <v>2</v>
@@ -70790,7 +70790,7 @@
       </c>
       <c r="J1386" s="6"/>
       <c r="L1386" s="3" t="s">
-        <v>2650</v>
+        <v>2634</v>
       </c>
       <c r="M1386">
         <v>2</v>
@@ -70836,7 +70836,7 @@
       </c>
       <c r="J1387" s="6"/>
       <c r="L1387" s="3" t="s">
-        <v>2651</v>
+        <v>2635</v>
       </c>
       <c r="M1387">
         <v>2</v>
@@ -70882,7 +70882,7 @@
       </c>
       <c r="J1388" s="6"/>
       <c r="L1388" s="3" t="s">
-        <v>2652</v>
+        <v>2636</v>
       </c>
       <c r="M1388">
         <v>2</v>
@@ -70928,7 +70928,7 @@
       </c>
       <c r="J1389" s="6"/>
       <c r="L1389" s="3" t="s">
-        <v>2653</v>
+        <v>2637</v>
       </c>
       <c r="M1389">
         <v>2</v>
@@ -70974,7 +70974,7 @@
       </c>
       <c r="J1390" s="6"/>
       <c r="L1390" s="3" t="s">
-        <v>2654</v>
+        <v>2638</v>
       </c>
       <c r="M1390">
         <v>2</v>
@@ -71020,7 +71020,7 @@
       </c>
       <c r="J1391" s="6"/>
       <c r="L1391" s="3" t="s">
-        <v>2641</v>
+        <v>2625</v>
       </c>
       <c r="M1391">
         <v>2</v>
@@ -71066,7 +71066,7 @@
       </c>
       <c r="J1392" s="6"/>
       <c r="L1392" s="3" t="s">
-        <v>2642</v>
+        <v>2626</v>
       </c>
       <c r="M1392">
         <v>2</v>
@@ -71112,7 +71112,7 @@
       </c>
       <c r="J1393" s="6"/>
       <c r="L1393" s="3" t="s">
-        <v>2643</v>
+        <v>2627</v>
       </c>
       <c r="M1393">
         <v>2</v>
@@ -71158,7 +71158,7 @@
       </c>
       <c r="J1394" s="6"/>
       <c r="L1394" s="3" t="s">
-        <v>2644</v>
+        <v>2628</v>
       </c>
       <c r="M1394">
         <v>2</v>
@@ -71204,7 +71204,7 @@
       </c>
       <c r="J1395" s="6"/>
       <c r="L1395" s="3" t="s">
-        <v>2645</v>
+        <v>2629</v>
       </c>
       <c r="M1395">
         <v>2</v>
@@ -71250,7 +71250,7 @@
       </c>
       <c r="J1396" s="6"/>
       <c r="L1396" s="3" t="s">
-        <v>2646</v>
+        <v>2630</v>
       </c>
       <c r="M1396">
         <v>2</v>
@@ -71296,7 +71296,7 @@
       </c>
       <c r="J1397" s="6"/>
       <c r="L1397" s="3" t="s">
-        <v>2647</v>
+        <v>2631</v>
       </c>
       <c r="M1397">
         <v>2</v>
@@ -71342,7 +71342,7 @@
       </c>
       <c r="J1398" s="6"/>
       <c r="L1398" s="3" t="s">
-        <v>2648</v>
+        <v>2632</v>
       </c>
       <c r="M1398">
         <v>2</v>
@@ -71388,7 +71388,7 @@
       </c>
       <c r="J1399" s="6"/>
       <c r="L1399" s="3" t="s">
-        <v>2655</v>
+        <v>2639</v>
       </c>
       <c r="M1399">
         <v>2</v>
@@ -71434,7 +71434,7 @@
       </c>
       <c r="J1400" s="6"/>
       <c r="L1400" s="3" t="s">
-        <v>2656</v>
+        <v>2640</v>
       </c>
       <c r="M1400">
         <v>2</v>
@@ -71480,7 +71480,7 @@
       </c>
       <c r="J1401" s="6"/>
       <c r="L1401" s="3" t="s">
-        <v>2657</v>
+        <v>2641</v>
       </c>
       <c r="M1401">
         <v>2</v>
@@ -71526,7 +71526,7 @@
       </c>
       <c r="J1402" s="6"/>
       <c r="L1402" s="3" t="s">
-        <v>2658</v>
+        <v>2642</v>
       </c>
       <c r="M1402">
         <v>2</v>
@@ -71572,7 +71572,7 @@
       </c>
       <c r="J1403" s="6"/>
       <c r="L1403" s="3" t="s">
-        <v>2659</v>
+        <v>2643</v>
       </c>
       <c r="M1403">
         <v>2</v>
@@ -71618,7 +71618,7 @@
       </c>
       <c r="J1404" s="6"/>
       <c r="L1404" s="3" t="s">
-        <v>2660</v>
+        <v>2644</v>
       </c>
       <c r="M1404">
         <v>2</v>
@@ -71664,7 +71664,7 @@
       </c>
       <c r="J1405" s="6"/>
       <c r="L1405" s="3" t="s">
-        <v>2664</v>
+        <v>2648</v>
       </c>
       <c r="M1405">
         <v>2</v>
@@ -71710,7 +71710,7 @@
       </c>
       <c r="J1406" s="6"/>
       <c r="L1406" s="3" t="s">
-        <v>2665</v>
+        <v>2649</v>
       </c>
       <c r="M1406">
         <v>2</v>
@@ -71756,7 +71756,7 @@
       </c>
       <c r="J1407" s="6"/>
       <c r="L1407" s="3" t="s">
-        <v>2666</v>
+        <v>2650</v>
       </c>
       <c r="M1407">
         <v>2</v>
@@ -71802,7 +71802,7 @@
       </c>
       <c r="J1408" s="6"/>
       <c r="L1408" s="3" t="s">
-        <v>2661</v>
+        <v>2645</v>
       </c>
       <c r="M1408">
         <v>2</v>
@@ -71848,7 +71848,7 @@
       </c>
       <c r="J1409" s="6"/>
       <c r="L1409" s="3" t="s">
-        <v>2662</v>
+        <v>2646</v>
       </c>
       <c r="M1409">
         <v>2</v>
@@ -71894,7 +71894,7 @@
       </c>
       <c r="J1410" s="6"/>
       <c r="L1410" s="3" t="s">
-        <v>2663</v>
+        <v>2647</v>
       </c>
       <c r="M1410">
         <v>2</v>
@@ -71940,7 +71940,7 @@
       </c>
       <c r="J1411" s="6"/>
       <c r="L1411" s="3" t="s">
-        <v>2668</v>
+        <v>2652</v>
       </c>
       <c r="M1411">
         <v>2</v>
@@ -71986,7 +71986,7 @@
       </c>
       <c r="J1412" s="6"/>
       <c r="L1412" s="3" t="s">
-        <v>2669</v>
+        <v>2653</v>
       </c>
       <c r="M1412">
         <v>2</v>
@@ -72032,7 +72032,7 @@
       </c>
       <c r="J1413" s="6"/>
       <c r="L1413" s="3" t="s">
-        <v>2670</v>
+        <v>2654</v>
       </c>
       <c r="M1413">
         <v>2</v>
@@ -72078,7 +72078,7 @@
       </c>
       <c r="J1414" s="6"/>
       <c r="L1414" s="3" t="s">
-        <v>2667</v>
+        <v>2651</v>
       </c>
       <c r="M1414">
         <v>2</v>
@@ -72124,7 +72124,7 @@
       </c>
       <c r="J1415" s="6"/>
       <c r="L1415" s="3" t="s">
-        <v>2671</v>
+        <v>2655</v>
       </c>
       <c r="M1415">
         <v>2</v>
@@ -72170,7 +72170,7 @@
       </c>
       <c r="J1416" s="6"/>
       <c r="L1416" s="3" t="s">
-        <v>2672</v>
+        <v>2656</v>
       </c>
       <c r="M1416">
         <v>2</v>
@@ -72216,7 +72216,7 @@
       </c>
       <c r="J1417" s="6"/>
       <c r="L1417" s="3" t="s">
-        <v>2677</v>
+        <v>2661</v>
       </c>
       <c r="M1417">
         <v>2</v>
@@ -72262,7 +72262,7 @@
       </c>
       <c r="J1418" s="6"/>
       <c r="L1418" s="3" t="s">
-        <v>2678</v>
+        <v>2662</v>
       </c>
       <c r="M1418">
         <v>2</v>
@@ -72308,7 +72308,7 @@
       </c>
       <c r="J1419" s="6"/>
       <c r="L1419" s="3" t="s">
-        <v>2679</v>
+        <v>2663</v>
       </c>
       <c r="M1419">
         <v>2</v>
@@ -72354,7 +72354,7 @@
       </c>
       <c r="J1420" s="6"/>
       <c r="L1420" s="3" t="s">
-        <v>2680</v>
+        <v>2664</v>
       </c>
       <c r="M1420">
         <v>2</v>
@@ -72400,7 +72400,7 @@
       </c>
       <c r="J1421" s="6"/>
       <c r="L1421" s="3" t="s">
-        <v>2681</v>
+        <v>2665</v>
       </c>
       <c r="M1421">
         <v>2</v>
@@ -72446,7 +72446,7 @@
       </c>
       <c r="J1422" s="6"/>
       <c r="L1422" s="3" t="s">
-        <v>2673</v>
+        <v>2657</v>
       </c>
       <c r="M1422">
         <v>2</v>
@@ -72492,7 +72492,7 @@
       </c>
       <c r="J1423" s="6"/>
       <c r="L1423" s="3" t="s">
-        <v>2674</v>
+        <v>2658</v>
       </c>
       <c r="M1423">
         <v>2</v>
@@ -72538,7 +72538,7 @@
       </c>
       <c r="J1424" s="6"/>
       <c r="L1424" s="3" t="s">
-        <v>2675</v>
+        <v>2659</v>
       </c>
       <c r="M1424">
         <v>2</v>
@@ -72584,7 +72584,7 @@
       </c>
       <c r="J1425" s="6"/>
       <c r="L1425" s="3" t="s">
-        <v>2676</v>
+        <v>2660</v>
       </c>
       <c r="M1425">
         <v>2</v>
@@ -72630,7 +72630,7 @@
       </c>
       <c r="J1426" s="6"/>
       <c r="L1426" s="3" t="s">
-        <v>2684</v>
+        <v>2668</v>
       </c>
       <c r="M1426">
         <v>2</v>
@@ -72676,7 +72676,7 @@
       </c>
       <c r="J1427" s="6"/>
       <c r="L1427" s="3" t="s">
-        <v>2685</v>
+        <v>2669</v>
       </c>
       <c r="M1427">
         <v>2</v>
@@ -72722,7 +72722,7 @@
       </c>
       <c r="J1428" s="6"/>
       <c r="L1428" s="3" t="s">
-        <v>2686</v>
+        <v>2670</v>
       </c>
       <c r="M1428">
         <v>2</v>
@@ -72768,7 +72768,7 @@
       </c>
       <c r="J1429" s="6"/>
       <c r="L1429" s="3" t="s">
-        <v>2682</v>
+        <v>2666</v>
       </c>
       <c r="M1429">
         <v>2</v>
@@ -72814,7 +72814,7 @@
       </c>
       <c r="J1430" s="6"/>
       <c r="L1430" s="3" t="s">
-        <v>2683</v>
+        <v>2667</v>
       </c>
       <c r="M1430">
         <v>2</v>
@@ -72860,7 +72860,7 @@
       </c>
       <c r="J1431" s="6"/>
       <c r="L1431" s="3" t="s">
-        <v>2687</v>
+        <v>2671</v>
       </c>
       <c r="M1431">
         <v>2</v>
@@ -72906,7 +72906,7 @@
       </c>
       <c r="J1432" s="6"/>
       <c r="L1432" s="3" t="s">
-        <v>2688</v>
+        <v>2672</v>
       </c>
       <c r="M1432">
         <v>2</v>
@@ -72952,7 +72952,7 @@
       </c>
       <c r="J1433" s="6"/>
       <c r="L1433" s="3" t="s">
-        <v>2689</v>
+        <v>2673</v>
       </c>
       <c r="M1433">
         <v>2</v>
@@ -72998,7 +72998,7 @@
       </c>
       <c r="J1434" s="6"/>
       <c r="L1434" s="3" t="s">
-        <v>2690</v>
+        <v>2674</v>
       </c>
       <c r="M1434">
         <v>2</v>
@@ -73044,7 +73044,7 @@
       </c>
       <c r="J1435" s="6"/>
       <c r="L1435" s="3" t="s">
-        <v>2691</v>
+        <v>2675</v>
       </c>
       <c r="M1435">
         <v>2</v>
@@ -73090,7 +73090,7 @@
       </c>
       <c r="J1436" s="6"/>
       <c r="L1436" s="3" t="s">
-        <v>2692</v>
+        <v>2676</v>
       </c>
       <c r="M1436">
         <v>2</v>
@@ -73136,7 +73136,7 @@
       </c>
       <c r="J1437" s="6"/>
       <c r="L1437" s="3" t="s">
-        <v>2693</v>
+        <v>2677</v>
       </c>
       <c r="M1437">
         <v>2</v>
@@ -73182,7 +73182,7 @@
       </c>
       <c r="J1438" s="6"/>
       <c r="L1438" s="3" t="s">
-        <v>2694</v>
+        <v>2678</v>
       </c>
       <c r="M1438">
         <v>2</v>
@@ -73228,7 +73228,7 @@
       </c>
       <c r="J1439" s="6"/>
       <c r="L1439" s="3" t="s">
-        <v>2695</v>
+        <v>2679</v>
       </c>
       <c r="M1439">
         <v>2</v>
@@ -73274,7 +73274,7 @@
       </c>
       <c r="J1440" s="6"/>
       <c r="L1440" s="3" t="s">
-        <v>2696</v>
+        <v>2680</v>
       </c>
       <c r="M1440">
         <v>2</v>
@@ -73320,7 +73320,7 @@
       </c>
       <c r="J1441" s="6"/>
       <c r="L1441" s="3" t="s">
-        <v>2697</v>
+        <v>2681</v>
       </c>
       <c r="M1441">
         <v>2</v>
@@ -73366,7 +73366,7 @@
       </c>
       <c r="J1442" s="6"/>
       <c r="L1442" s="3" t="s">
-        <v>2698</v>
+        <v>2682</v>
       </c>
       <c r="M1442">
         <v>2</v>
@@ -73412,7 +73412,7 @@
       </c>
       <c r="J1443" s="6"/>
       <c r="L1443" s="3" t="s">
-        <v>2699</v>
+        <v>2683</v>
       </c>
       <c r="M1443">
         <v>2</v>
@@ -73458,7 +73458,7 @@
       </c>
       <c r="J1444" s="6"/>
       <c r="L1444" s="3" t="s">
-        <v>2700</v>
+        <v>2684</v>
       </c>
       <c r="M1444">
         <v>2</v>
@@ -73504,7 +73504,7 @@
       </c>
       <c r="J1445" s="6"/>
       <c r="L1445" s="3" t="s">
-        <v>2701</v>
+        <v>2685</v>
       </c>
       <c r="M1445">
         <v>2</v>
@@ -73550,7 +73550,7 @@
       </c>
       <c r="J1446" s="6"/>
       <c r="L1446" s="3" t="s">
-        <v>2702</v>
+        <v>2686</v>
       </c>
       <c r="M1446">
         <v>2</v>
@@ -73596,7 +73596,7 @@
       </c>
       <c r="J1447" s="6"/>
       <c r="L1447" s="3" t="s">
-        <v>2703</v>
+        <v>2687</v>
       </c>
       <c r="M1447">
         <v>2</v>
@@ -73642,7 +73642,7 @@
       </c>
       <c r="J1448" s="6"/>
       <c r="L1448" s="3" t="s">
-        <v>2704</v>
+        <v>2688</v>
       </c>
       <c r="M1448">
         <v>2</v>
@@ -73688,7 +73688,7 @@
       </c>
       <c r="J1449" s="6"/>
       <c r="L1449" s="3" t="s">
-        <v>2705</v>
+        <v>2689</v>
       </c>
       <c r="M1449">
         <v>2</v>
@@ -73734,7 +73734,7 @@
       </c>
       <c r="J1450" s="6"/>
       <c r="L1450" s="3" t="s">
-        <v>2706</v>
+        <v>2690</v>
       </c>
       <c r="M1450">
         <v>2</v>
@@ -73780,7 +73780,7 @@
       </c>
       <c r="J1451" s="6"/>
       <c r="L1451" s="3" t="s">
-        <v>2707</v>
+        <v>2691</v>
       </c>
       <c r="M1451">
         <v>2</v>
@@ -73826,7 +73826,7 @@
       </c>
       <c r="J1452" s="6"/>
       <c r="L1452" s="3" t="s">
-        <v>2708</v>
+        <v>2692</v>
       </c>
       <c r="M1452">
         <v>2</v>
@@ -73872,7 +73872,7 @@
       </c>
       <c r="J1453" s="6"/>
       <c r="L1453" s="3" t="s">
-        <v>2709</v>
+        <v>2693</v>
       </c>
       <c r="M1453">
         <v>2</v>
@@ -73918,7 +73918,7 @@
       </c>
       <c r="J1454" s="6"/>
       <c r="L1454" s="3" t="s">
-        <v>2710</v>
+        <v>2694</v>
       </c>
       <c r="M1454">
         <v>2</v>
@@ -73964,7 +73964,7 @@
       </c>
       <c r="J1455" s="6"/>
       <c r="L1455" s="3" t="s">
-        <v>2711</v>
+        <v>2695</v>
       </c>
       <c r="M1455">
         <v>2</v>
@@ -74010,7 +74010,7 @@
       </c>
       <c r="J1456" s="6"/>
       <c r="L1456" s="3" t="s">
-        <v>2712</v>
+        <v>2696</v>
       </c>
       <c r="M1456">
         <v>2</v>
@@ -74056,7 +74056,7 @@
       </c>
       <c r="J1457" s="6"/>
       <c r="L1457" s="3" t="s">
-        <v>2713</v>
+        <v>2697</v>
       </c>
       <c r="M1457">
         <v>2</v>
@@ -74102,7 +74102,7 @@
       </c>
       <c r="J1458" s="6"/>
       <c r="L1458" s="3" t="s">
-        <v>2714</v>
+        <v>2698</v>
       </c>
       <c r="M1458">
         <v>2</v>
@@ -74148,7 +74148,7 @@
       </c>
       <c r="J1459" s="6"/>
       <c r="L1459" s="3" t="s">
-        <v>2715</v>
+        <v>2699</v>
       </c>
       <c r="M1459">
         <v>2</v>
@@ -74194,7 +74194,7 @@
       </c>
       <c r="J1460" s="6"/>
       <c r="L1460" s="3" t="s">
-        <v>2716</v>
+        <v>2700</v>
       </c>
       <c r="M1460">
         <v>2</v>
@@ -74240,7 +74240,7 @@
       </c>
       <c r="J1461" s="6"/>
       <c r="L1461" s="3" t="s">
-        <v>2717</v>
+        <v>2701</v>
       </c>
       <c r="M1461">
         <v>2</v>
@@ -74286,7 +74286,7 @@
       </c>
       <c r="J1462" s="6"/>
       <c r="L1462" s="3" t="s">
-        <v>2718</v>
+        <v>2702</v>
       </c>
       <c r="M1462">
         <v>2</v>
@@ -74332,7 +74332,7 @@
       </c>
       <c r="J1463" s="6"/>
       <c r="L1463" s="3" t="s">
-        <v>2719</v>
+        <v>2703</v>
       </c>
       <c r="M1463">
         <v>2</v>
@@ -74378,7 +74378,7 @@
       </c>
       <c r="J1464" s="6"/>
       <c r="L1464" s="3" t="s">
-        <v>2720</v>
+        <v>2704</v>
       </c>
       <c r="M1464">
         <v>2</v>
@@ -74424,7 +74424,7 @@
       </c>
       <c r="J1465" s="6"/>
       <c r="L1465" s="3" t="s">
-        <v>2721</v>
+        <v>2705</v>
       </c>
       <c r="M1465">
         <v>2</v>
@@ -74470,7 +74470,7 @@
       </c>
       <c r="J1466" s="6"/>
       <c r="L1466" s="3" t="s">
-        <v>2722</v>
+        <v>2706</v>
       </c>
       <c r="M1466">
         <v>2</v>
@@ -74516,7 +74516,7 @@
       </c>
       <c r="J1467" s="6"/>
       <c r="L1467" s="3" t="s">
-        <v>2726</v>
+        <v>2710</v>
       </c>
       <c r="M1467">
         <v>2</v>
@@ -74562,7 +74562,7 @@
       </c>
       <c r="J1468" s="6"/>
       <c r="L1468" s="3" t="s">
-        <v>2727</v>
+        <v>2711</v>
       </c>
       <c r="M1468">
         <v>2</v>
@@ -74608,7 +74608,7 @@
       </c>
       <c r="J1469" s="6"/>
       <c r="L1469" s="3" t="s">
-        <v>2728</v>
+        <v>2712</v>
       </c>
       <c r="M1469">
         <v>2</v>
@@ -74654,7 +74654,7 @@
       </c>
       <c r="J1470" s="6"/>
       <c r="L1470" s="3" t="s">
-        <v>2723</v>
+        <v>2707</v>
       </c>
       <c r="M1470">
         <v>2</v>
@@ -74700,7 +74700,7 @@
       </c>
       <c r="J1471" s="6"/>
       <c r="L1471" s="3" t="s">
-        <v>2724</v>
+        <v>2708</v>
       </c>
       <c r="M1471">
         <v>2</v>
@@ -74746,7 +74746,7 @@
       </c>
       <c r="J1472" s="6"/>
       <c r="L1472" s="3" t="s">
-        <v>2725</v>
+        <v>2709</v>
       </c>
       <c r="M1472">
         <v>2</v>
@@ -74792,7 +74792,7 @@
       </c>
       <c r="J1473" s="6"/>
       <c r="L1473" s="3" t="s">
-        <v>2729</v>
+        <v>2713</v>
       </c>
       <c r="M1473">
         <v>2</v>
@@ -74838,7 +74838,7 @@
       </c>
       <c r="J1474" s="6"/>
       <c r="L1474" s="3" t="s">
-        <v>2730</v>
+        <v>2714</v>
       </c>
       <c r="M1474">
         <v>2</v>
@@ -74884,7 +74884,7 @@
       </c>
       <c r="J1475" s="6"/>
       <c r="L1475" s="3" t="s">
-        <v>2731</v>
+        <v>2715</v>
       </c>
       <c r="M1475">
         <v>2</v>
@@ -74930,7 +74930,7 @@
       </c>
       <c r="J1476" s="6"/>
       <c r="L1476" s="3" t="s">
-        <v>2732</v>
+        <v>2716</v>
       </c>
       <c r="M1476">
         <v>2</v>
@@ -74976,7 +74976,7 @@
       </c>
       <c r="J1477" s="6"/>
       <c r="L1477" s="3" t="s">
-        <v>2733</v>
+        <v>2717</v>
       </c>
       <c r="M1477">
         <v>2</v>
@@ -75022,7 +75022,7 @@
       </c>
       <c r="J1478" s="6"/>
       <c r="L1478" s="3" t="s">
-        <v>2734</v>
+        <v>2718</v>
       </c>
       <c r="M1478">
         <v>2</v>
@@ -75068,7 +75068,7 @@
       </c>
       <c r="J1479" s="6"/>
       <c r="L1479" s="3" t="s">
-        <v>2735</v>
+        <v>2719</v>
       </c>
       <c r="M1479">
         <v>2</v>
@@ -75114,7 +75114,7 @@
       </c>
       <c r="J1480" s="6"/>
       <c r="L1480" s="3" t="s">
-        <v>2736</v>
+        <v>2720</v>
       </c>
       <c r="M1480">
         <v>2</v>
@@ -75160,7 +75160,7 @@
       </c>
       <c r="J1481" s="6"/>
       <c r="L1481" s="3" t="s">
-        <v>2737</v>
+        <v>2721</v>
       </c>
       <c r="M1481">
         <v>2</v>
@@ -75206,7 +75206,7 @@
       </c>
       <c r="J1482" s="6"/>
       <c r="L1482" s="3" t="s">
-        <v>2738</v>
+        <v>2722</v>
       </c>
       <c r="M1482">
         <v>2</v>
@@ -75252,7 +75252,7 @@
       </c>
       <c r="J1483" s="6"/>
       <c r="L1483" s="3" t="s">
-        <v>2739</v>
+        <v>2723</v>
       </c>
       <c r="M1483">
         <v>2</v>
@@ -75298,7 +75298,7 @@
       </c>
       <c r="J1484" s="6"/>
       <c r="L1484" s="3" t="s">
-        <v>2740</v>
+        <v>2724</v>
       </c>
       <c r="M1484">
         <v>2</v>
@@ -75344,7 +75344,7 @@
       </c>
       <c r="J1485" s="6"/>
       <c r="L1485" s="3" t="s">
-        <v>2741</v>
+        <v>2725</v>
       </c>
       <c r="M1485">
         <v>2</v>
@@ -75390,7 +75390,7 @@
       </c>
       <c r="J1486" s="6"/>
       <c r="L1486" s="3" t="s">
-        <v>2742</v>
+        <v>2726</v>
       </c>
       <c r="M1486">
         <v>2</v>
@@ -75436,7 +75436,7 @@
       </c>
       <c r="J1487" s="6"/>
       <c r="L1487" s="3" t="s">
-        <v>2743</v>
+        <v>2727</v>
       </c>
       <c r="M1487">
         <v>2</v>
@@ -75482,7 +75482,7 @@
       </c>
       <c r="J1488" s="6"/>
       <c r="L1488" s="3" t="s">
-        <v>2744</v>
+        <v>2728</v>
       </c>
       <c r="M1488">
         <v>2</v>
@@ -75528,7 +75528,7 @@
       </c>
       <c r="J1489" s="6"/>
       <c r="L1489" s="3" t="s">
-        <v>2745</v>
+        <v>2729</v>
       </c>
       <c r="M1489">
         <v>2</v>
@@ -75574,7 +75574,7 @@
       </c>
       <c r="J1490" s="6"/>
       <c r="L1490" s="3" t="s">
-        <v>2746</v>
+        <v>2730</v>
       </c>
       <c r="M1490">
         <v>2</v>
@@ -75620,7 +75620,7 @@
       </c>
       <c r="J1491" s="6"/>
       <c r="L1491" s="3" t="s">
-        <v>2747</v>
+        <v>2731</v>
       </c>
       <c r="M1491">
         <v>2</v>
@@ -75666,7 +75666,7 @@
       </c>
       <c r="J1492" s="6"/>
       <c r="L1492" s="3" t="s">
-        <v>2748</v>
+        <v>2732</v>
       </c>
       <c r="M1492">
         <v>2</v>
@@ -75712,7 +75712,7 @@
       </c>
       <c r="J1493" s="6"/>
       <c r="L1493" s="3" t="s">
-        <v>2749</v>
+        <v>2733</v>
       </c>
       <c r="M1493">
         <v>2</v>
@@ -75758,7 +75758,7 @@
       </c>
       <c r="J1494" s="6"/>
       <c r="L1494" s="3" t="s">
-        <v>2750</v>
+        <v>2734</v>
       </c>
       <c r="M1494">
         <v>2</v>
@@ -75804,7 +75804,7 @@
       </c>
       <c r="J1495" s="6"/>
       <c r="L1495" s="3" t="s">
-        <v>2751</v>
+        <v>2735</v>
       </c>
       <c r="M1495">
         <v>2</v>
@@ -75850,7 +75850,7 @@
       </c>
       <c r="J1496" s="6"/>
       <c r="L1496" s="3" t="s">
-        <v>2752</v>
+        <v>2736</v>
       </c>
       <c r="M1496">
         <v>2</v>
@@ -75896,7 +75896,7 @@
       </c>
       <c r="J1497" s="6"/>
       <c r="L1497" s="3" t="s">
-        <v>2753</v>
+        <v>2737</v>
       </c>
       <c r="M1497">
         <v>2</v>
@@ -75942,7 +75942,7 @@
       </c>
       <c r="J1498" s="6"/>
       <c r="L1498" s="3" t="s">
-        <v>2754</v>
+        <v>2738</v>
       </c>
       <c r="M1498">
         <v>2</v>
@@ -75988,7 +75988,7 @@
       </c>
       <c r="J1499" s="6"/>
       <c r="L1499" s="3" t="s">
-        <v>2755</v>
+        <v>2739</v>
       </c>
       <c r="M1499">
         <v>2</v>
@@ -76034,7 +76034,7 @@
       </c>
       <c r="J1500" s="6"/>
       <c r="L1500" s="3" t="s">
-        <v>2756</v>
+        <v>2740</v>
       </c>
       <c r="M1500">
         <v>2</v>
@@ -76080,7 +76080,7 @@
       </c>
       <c r="J1501" s="6"/>
       <c r="L1501" s="3" t="s">
-        <v>2757</v>
+        <v>2741</v>
       </c>
       <c r="M1501">
         <v>2</v>
@@ -76126,7 +76126,7 @@
       </c>
       <c r="J1502" s="6"/>
       <c r="L1502" s="3" t="s">
-        <v>2758</v>
+        <v>2742</v>
       </c>
       <c r="M1502">
         <v>2</v>
@@ -76172,7 +76172,7 @@
       </c>
       <c r="J1503" s="6"/>
       <c r="L1503" s="3" t="s">
-        <v>2759</v>
+        <v>2743</v>
       </c>
       <c r="M1503">
         <v>2</v>
@@ -76218,7 +76218,7 @@
       </c>
       <c r="J1504" s="6"/>
       <c r="L1504" s="3" t="s">
-        <v>2760</v>
+        <v>2744</v>
       </c>
       <c r="M1504">
         <v>2</v>
@@ -76264,7 +76264,7 @@
       </c>
       <c r="J1505" s="6"/>
       <c r="L1505" s="3" t="s">
-        <v>2761</v>
+        <v>2745</v>
       </c>
       <c r="M1505">
         <v>2</v>
@@ -76310,7 +76310,7 @@
       </c>
       <c r="J1506" s="6"/>
       <c r="L1506" s="3" t="s">
-        <v>2764</v>
+        <v>2748</v>
       </c>
       <c r="M1506">
         <v>2</v>
@@ -76356,7 +76356,7 @@
       </c>
       <c r="J1507" s="6"/>
       <c r="L1507" s="3" t="s">
-        <v>2762</v>
+        <v>2746</v>
       </c>
       <c r="M1507">
         <v>2</v>
@@ -76402,7 +76402,7 @@
       </c>
       <c r="J1508" s="6"/>
       <c r="L1508" s="3" t="s">
-        <v>2763</v>
+        <v>2747</v>
       </c>
       <c r="M1508">
         <v>2</v>
@@ -76448,7 +76448,7 @@
       </c>
       <c r="J1509" s="6"/>
       <c r="L1509" s="3" t="s">
-        <v>2765</v>
+        <v>2749</v>
       </c>
       <c r="M1509">
         <v>2</v>
@@ -76494,7 +76494,7 @@
       </c>
       <c r="J1510" s="6"/>
       <c r="L1510" s="3" t="s">
-        <v>2766</v>
+        <v>2750</v>
       </c>
       <c r="M1510">
         <v>2</v>
@@ -76540,7 +76540,7 @@
       </c>
       <c r="J1511" s="6"/>
       <c r="L1511" s="3" t="s">
-        <v>2767</v>
+        <v>2751</v>
       </c>
       <c r="M1511">
         <v>2</v>
@@ -76586,7 +76586,7 @@
       </c>
       <c r="J1512" s="6"/>
       <c r="L1512" s="3" t="s">
-        <v>2768</v>
+        <v>2752</v>
       </c>
       <c r="M1512">
         <v>2</v>
@@ -76632,7 +76632,7 @@
       </c>
       <c r="J1513" s="6"/>
       <c r="L1513" s="3" t="s">
-        <v>2769</v>
+        <v>2753</v>
       </c>
       <c r="M1513">
         <v>2</v>
@@ -76678,7 +76678,7 @@
       </c>
       <c r="J1514" s="6"/>
       <c r="L1514" s="3" t="s">
-        <v>2770</v>
+        <v>2754</v>
       </c>
       <c r="M1514">
         <v>2</v>
@@ -76724,7 +76724,7 @@
       </c>
       <c r="J1515" s="6"/>
       <c r="L1515" s="3" t="s">
-        <v>2771</v>
+        <v>2755</v>
       </c>
       <c r="M1515">
         <v>2</v>

</xml_diff>

<commit_message>
fix: changed type for biomass burning aerosol and corrected paths in surface level folder
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA40EF4-E13E-46B0-8E19-04844816C4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA961C0-5E0B-4119-B651-FCC3AFC21B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -9063,6 +9063,12 @@
       <c r="G8">
         <v>0</v>
       </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
@@ -9106,6 +9112,12 @@
       <c r="F10" t="s">
         <v>2772</v>
       </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
@@ -9123,6 +9135,12 @@
       <c r="F11" t="s">
         <v>2772</v>
       </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
@@ -9140,6 +9158,12 @@
       <c r="F12" t="s">
         <v>2773</v>
       </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
@@ -9156,6 +9180,12 @@
       </c>
       <c r="F13" t="s">
         <v>2773</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
@@ -11659,7 +11689,7 @@
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>2777</v>
+        <v>2774</v>
       </c>
       <c r="L45" t="s">
         <v>219</v>
@@ -11892,7 +11922,7 @@
         <v>1</v>
       </c>
       <c r="J49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
         <v>2777</v>
@@ -12249,7 +12279,7 @@
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>2776</v>
+        <v>2774</v>
       </c>
       <c r="L55" t="s">
         <v>269</v>

</xml_diff>

<commit_message>
chore: added all created json links to the datasets and variables tabs
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577D8B87-A935-4E2E-BF9C-D8B5CFECCBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EC4F1E-F6BB-44F4-9C2E-4936F42FDC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,25 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">datasets!$A$1:$T$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">variables!$A$1:$S$1515</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6490" uniqueCount="3200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6591" uniqueCount="3301">
   <si>
     <t>DbId</t>
   </si>
@@ -9628,6 +9641,309 @@
   </si>
   <si>
     <t>19b02dc323e-layer-276-0</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__anuual_mean__ug_m3_timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/co__annual_mean__mg_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/co__2010__mil.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__timeseries.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2022.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2021.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2020.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2019.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2018.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2017.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2016.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2015.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2014.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2013.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2012.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2011.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/co__max_8hr_mean__mg_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2022.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2021.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2020.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2019.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2018.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2017.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2016.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2015.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2014.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2011.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2013.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2012.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2022.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2021.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2020.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2019.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2018.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2017.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2016.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2015.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2014.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2013.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2012.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2011.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/nox__annual_mean__ug_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2022.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2021.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2020.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2019.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2018.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2017.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2016.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2015.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2014.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2013.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2012.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2011.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2022_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2021_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2020_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2019_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2018_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2017_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2016_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2015_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2014_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2013_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2012_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2011_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2010_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2022_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2021_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2020_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2019_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2018_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2017_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2016_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2015_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2014_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2013_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2012_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2011_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm10__annual_mean__ug_m3__2010_g.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2022.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2021.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2020.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2019.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2018.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2017.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2016.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2015.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2014.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2013.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2012.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2011.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2010.json</t>
   </si>
 </sst>
 </file>
@@ -12183,6 +12499,9 @@
       <c r="M30">
         <v>4002</v>
       </c>
+      <c r="O30" s="3" t="s">
+        <v>3208</v>
+      </c>
       <c r="P30">
         <v>2</v>
       </c>
@@ -12239,6 +12558,9 @@
       <c r="M31">
         <v>4003</v>
       </c>
+      <c r="O31" s="3" t="s">
+        <v>3207</v>
+      </c>
       <c r="P31">
         <v>2</v>
       </c>
@@ -12295,6 +12617,9 @@
       <c r="M32">
         <v>4004</v>
       </c>
+      <c r="O32" s="3" t="s">
+        <v>3205</v>
+      </c>
       <c r="P32">
         <v>2</v>
       </c>
@@ -12351,6 +12676,9 @@
       <c r="M33">
         <v>4005</v>
       </c>
+      <c r="O33" s="3" t="s">
+        <v>3203</v>
+      </c>
       <c r="P33">
         <v>2</v>
       </c>
@@ -12407,6 +12735,9 @@
       <c r="M34">
         <v>4006</v>
       </c>
+      <c r="O34" s="3" t="s">
+        <v>3204</v>
+      </c>
       <c r="P34">
         <v>2</v>
       </c>
@@ -12463,6 +12794,9 @@
       <c r="M35">
         <v>4007</v>
       </c>
+      <c r="O35" s="3" t="s">
+        <v>3201</v>
+      </c>
       <c r="P35">
         <v>2</v>
       </c>
@@ -12519,6 +12853,9 @@
       <c r="M36">
         <v>4008</v>
       </c>
+      <c r="O36" s="3" t="s">
+        <v>3202</v>
+      </c>
       <c r="P36">
         <v>2</v>
       </c>
@@ -12574,6 +12911,9 @@
       </c>
       <c r="M37">
         <v>4009</v>
+      </c>
+      <c r="O37" s="3" t="s">
+        <v>3200</v>
       </c>
       <c r="P37">
         <v>2</v>
@@ -14325,6 +14665,14 @@
     <hyperlink ref="O63" r:id="rId31" xr:uid="{356CAD23-03AB-460F-AFCA-EC4BDE2D8AE0}"/>
     <hyperlink ref="O64" r:id="rId32" xr:uid="{4F6B4081-E0D1-4EF1-825D-2153F4EE3414}"/>
     <hyperlink ref="E40" r:id="rId33" xr:uid="{FD826172-87CB-45B3-A0FC-D8B3114ACB40}"/>
+    <hyperlink ref="O37" r:id="rId34" xr:uid="{140F4408-E7AA-44B6-A18E-360C0D67CD7D}"/>
+    <hyperlink ref="O35" r:id="rId35" xr:uid="{808E1FD3-625F-468F-B5CE-C7D46AEC377C}"/>
+    <hyperlink ref="O36" r:id="rId36" xr:uid="{EEDF3432-B070-4FF4-BC80-348F20F284B0}"/>
+    <hyperlink ref="O34" r:id="rId37" xr:uid="{92BB371E-C739-4E6E-90A8-536B8C7ABAAB}"/>
+    <hyperlink ref="O33" r:id="rId38" xr:uid="{28DFF9D9-D4E7-49F3-9FF8-53AEB03F1132}"/>
+    <hyperlink ref="O32" r:id="rId39" xr:uid="{B0A928E1-5A9D-4904-925C-B849C701CBE6}"/>
+    <hyperlink ref="O31" r:id="rId40" xr:uid="{DE66E62C-23D8-409B-8828-A2B1F7104694}"/>
+    <hyperlink ref="O30" r:id="rId41" xr:uid="{7F69EBA1-2661-4784-B19E-BB4CCA00E309}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -55736,6 +56084,9 @@
         <v>0</v>
       </c>
       <c r="J1018" s="6"/>
+      <c r="L1018" s="3" t="s">
+        <v>3209</v>
+      </c>
       <c r="M1018">
         <v>2</v>
       </c>
@@ -55781,6 +56132,9 @@
         <v>0</v>
       </c>
       <c r="J1019" s="6"/>
+      <c r="L1019" s="3" t="s">
+        <v>3210</v>
+      </c>
       <c r="M1019">
         <v>2</v>
       </c>
@@ -55826,6 +56180,9 @@
         <v>0</v>
       </c>
       <c r="J1020" s="6"/>
+      <c r="L1020" s="3" t="s">
+        <v>3211</v>
+      </c>
       <c r="M1020">
         <v>2</v>
       </c>
@@ -55871,6 +56228,9 @@
         <v>0</v>
       </c>
       <c r="J1021" s="6"/>
+      <c r="L1021" s="3" t="s">
+        <v>3212</v>
+      </c>
       <c r="M1021">
         <v>2</v>
       </c>
@@ -55916,6 +56276,9 @@
         <v>0</v>
       </c>
       <c r="J1022" s="6"/>
+      <c r="L1022" s="3" t="s">
+        <v>3213</v>
+      </c>
       <c r="M1022">
         <v>2</v>
       </c>
@@ -55961,6 +56324,9 @@
         <v>0</v>
       </c>
       <c r="J1023" s="6"/>
+      <c r="L1023" s="3" t="s">
+        <v>3214</v>
+      </c>
       <c r="M1023">
         <v>2</v>
       </c>
@@ -56006,6 +56372,9 @@
         <v>0</v>
       </c>
       <c r="J1024" s="6"/>
+      <c r="L1024" s="3" t="s">
+        <v>3215</v>
+      </c>
       <c r="M1024">
         <v>2</v>
       </c>
@@ -56051,6 +56420,9 @@
         <v>0</v>
       </c>
       <c r="J1025" s="6"/>
+      <c r="L1025" s="3" t="s">
+        <v>3216</v>
+      </c>
       <c r="M1025">
         <v>2</v>
       </c>
@@ -56096,6 +56468,9 @@
         <v>0</v>
       </c>
       <c r="J1026" s="6"/>
+      <c r="L1026" s="3" t="s">
+        <v>3217</v>
+      </c>
       <c r="M1026">
         <v>2</v>
       </c>
@@ -56141,6 +56516,9 @@
         <v>0</v>
       </c>
       <c r="J1027" s="6"/>
+      <c r="L1027" s="3" t="s">
+        <v>3218</v>
+      </c>
       <c r="M1027">
         <v>2</v>
       </c>
@@ -56186,6 +56564,9 @@
         <v>0</v>
       </c>
       <c r="J1028" s="6"/>
+      <c r="L1028" s="3" t="s">
+        <v>3219</v>
+      </c>
       <c r="M1028">
         <v>2</v>
       </c>
@@ -56231,6 +56612,9 @@
         <v>0</v>
       </c>
       <c r="J1029" s="6"/>
+      <c r="L1029" s="3" t="s">
+        <v>3220</v>
+      </c>
       <c r="M1029">
         <v>2</v>
       </c>
@@ -56276,6 +56660,9 @@
         <v>0</v>
       </c>
       <c r="J1030" s="6"/>
+      <c r="L1030" s="3" t="s">
+        <v>3221</v>
+      </c>
       <c r="M1030">
         <v>2</v>
       </c>
@@ -56321,6 +56708,9 @@
         <v>0</v>
       </c>
       <c r="J1031" s="6"/>
+      <c r="L1031" s="3" t="s">
+        <v>3206</v>
+      </c>
       <c r="M1031">
         <v>2</v>
       </c>
@@ -56366,6 +56756,9 @@
         <v>0</v>
       </c>
       <c r="J1032" s="6"/>
+      <c r="L1032" s="3" t="s">
+        <v>3222</v>
+      </c>
       <c r="M1032">
         <v>2</v>
       </c>
@@ -56411,6 +56804,9 @@
         <v>0</v>
       </c>
       <c r="J1033" s="6"/>
+      <c r="L1033" s="3" t="s">
+        <v>3223</v>
+      </c>
       <c r="M1033">
         <v>2</v>
       </c>
@@ -56456,6 +56852,9 @@
         <v>0</v>
       </c>
       <c r="J1034" s="6"/>
+      <c r="L1034" s="3" t="s">
+        <v>3224</v>
+      </c>
       <c r="M1034">
         <v>2</v>
       </c>
@@ -56501,6 +56900,9 @@
         <v>0</v>
       </c>
       <c r="J1035" s="6"/>
+      <c r="L1035" s="3" t="s">
+        <v>3225</v>
+      </c>
       <c r="M1035">
         <v>2</v>
       </c>
@@ -56546,6 +56948,9 @@
         <v>0</v>
       </c>
       <c r="J1036" s="6"/>
+      <c r="L1036" s="3" t="s">
+        <v>3226</v>
+      </c>
       <c r="M1036">
         <v>2</v>
       </c>
@@ -56591,6 +56996,9 @@
         <v>0</v>
       </c>
       <c r="J1037" s="6"/>
+      <c r="L1037" s="3" t="s">
+        <v>3227</v>
+      </c>
       <c r="M1037">
         <v>2</v>
       </c>
@@ -56636,6 +57044,9 @@
         <v>0</v>
       </c>
       <c r="J1038" s="6"/>
+      <c r="L1038" s="3" t="s">
+        <v>3228</v>
+      </c>
       <c r="M1038">
         <v>2</v>
       </c>
@@ -56681,6 +57092,9 @@
         <v>0</v>
       </c>
       <c r="J1039" s="6"/>
+      <c r="L1039" s="3" t="s">
+        <v>3229</v>
+      </c>
       <c r="M1039">
         <v>2</v>
       </c>
@@ -56726,6 +57140,9 @@
         <v>0</v>
       </c>
       <c r="J1040" s="6"/>
+      <c r="L1040" s="3" t="s">
+        <v>3230</v>
+      </c>
       <c r="M1040">
         <v>2</v>
       </c>
@@ -56771,6 +57188,9 @@
         <v>0</v>
       </c>
       <c r="J1041" s="6"/>
+      <c r="L1041" s="3" t="s">
+        <v>3231</v>
+      </c>
       <c r="M1041">
         <v>2</v>
       </c>
@@ -56816,6 +57236,9 @@
         <v>0</v>
       </c>
       <c r="J1042" s="6"/>
+      <c r="L1042" s="3" t="s">
+        <v>3234</v>
+      </c>
       <c r="M1042">
         <v>2</v>
       </c>
@@ -56861,6 +57284,9 @@
         <v>0</v>
       </c>
       <c r="J1043" s="6"/>
+      <c r="L1043" s="3" t="s">
+        <v>3235</v>
+      </c>
       <c r="M1043">
         <v>2</v>
       </c>
@@ -56906,6 +57332,9 @@
         <v>0</v>
       </c>
       <c r="J1044" s="6"/>
+      <c r="L1044" s="3" t="s">
+        <v>3232</v>
+      </c>
       <c r="M1044">
         <v>2</v>
       </c>
@@ -56951,6 +57380,9 @@
         <v>0</v>
       </c>
       <c r="J1045" s="6"/>
+      <c r="L1045" s="3" t="s">
+        <v>3233</v>
+      </c>
       <c r="M1045">
         <v>2</v>
       </c>
@@ -56996,6 +57428,9 @@
         <v>0</v>
       </c>
       <c r="J1046" s="6"/>
+      <c r="L1046" s="3" t="s">
+        <v>3236</v>
+      </c>
       <c r="M1046">
         <v>2</v>
       </c>
@@ -57041,6 +57476,9 @@
         <v>0</v>
       </c>
       <c r="J1047" s="6"/>
+      <c r="L1047" s="3" t="s">
+        <v>3237</v>
+      </c>
       <c r="M1047">
         <v>2</v>
       </c>
@@ -57086,6 +57524,9 @@
         <v>0</v>
       </c>
       <c r="J1048" s="6"/>
+      <c r="L1048" s="3" t="s">
+        <v>3238</v>
+      </c>
       <c r="M1048">
         <v>2</v>
       </c>
@@ -57131,6 +57572,9 @@
         <v>0</v>
       </c>
       <c r="J1049" s="6"/>
+      <c r="L1049" s="3" t="s">
+        <v>3239</v>
+      </c>
       <c r="M1049">
         <v>2</v>
       </c>
@@ -57176,6 +57620,9 @@
         <v>0</v>
       </c>
       <c r="J1050" s="6"/>
+      <c r="L1050" s="3" t="s">
+        <v>3240</v>
+      </c>
       <c r="M1050">
         <v>2</v>
       </c>
@@ -57221,6 +57668,9 @@
         <v>0</v>
       </c>
       <c r="J1051" s="6"/>
+      <c r="L1051" s="3" t="s">
+        <v>3241</v>
+      </c>
       <c r="M1051">
         <v>2</v>
       </c>
@@ -57266,6 +57716,9 @@
         <v>0</v>
       </c>
       <c r="J1052" s="6"/>
+      <c r="L1052" s="3" t="s">
+        <v>3242</v>
+      </c>
       <c r="M1052">
         <v>2</v>
       </c>
@@ -57311,6 +57764,9 @@
         <v>0</v>
       </c>
       <c r="J1053" s="6"/>
+      <c r="L1053" s="3" t="s">
+        <v>3243</v>
+      </c>
       <c r="M1053">
         <v>2</v>
       </c>
@@ -57356,6 +57812,9 @@
         <v>0</v>
       </c>
       <c r="J1054" s="6"/>
+      <c r="L1054" s="3" t="s">
+        <v>3244</v>
+      </c>
       <c r="M1054">
         <v>2</v>
       </c>
@@ -57401,6 +57860,9 @@
         <v>0</v>
       </c>
       <c r="J1055" s="6"/>
+      <c r="L1055" s="3" t="s">
+        <v>3245</v>
+      </c>
       <c r="M1055">
         <v>2</v>
       </c>
@@ -57446,6 +57908,9 @@
         <v>0</v>
       </c>
       <c r="J1056" s="6"/>
+      <c r="L1056" s="3" t="s">
+        <v>3246</v>
+      </c>
       <c r="M1056">
         <v>2</v>
       </c>
@@ -57491,6 +57956,9 @@
         <v>0</v>
       </c>
       <c r="J1057" s="6"/>
+      <c r="L1057" s="3" t="s">
+        <v>3247</v>
+      </c>
       <c r="M1057">
         <v>2</v>
       </c>
@@ -57536,6 +58004,9 @@
         <v>0</v>
       </c>
       <c r="J1058" s="6"/>
+      <c r="L1058" s="3" t="s">
+        <v>3248</v>
+      </c>
       <c r="M1058">
         <v>2</v>
       </c>
@@ -57581,6 +58052,9 @@
         <v>0</v>
       </c>
       <c r="J1059" s="6"/>
+      <c r="L1059" s="3" t="s">
+        <v>3249</v>
+      </c>
       <c r="M1059">
         <v>2</v>
       </c>
@@ -57626,6 +58100,9 @@
         <v>0</v>
       </c>
       <c r="J1060" s="6"/>
+      <c r="L1060" s="3" t="s">
+        <v>3250</v>
+      </c>
       <c r="M1060">
         <v>2</v>
       </c>
@@ -57671,6 +58148,9 @@
         <v>0</v>
       </c>
       <c r="J1061" s="6"/>
+      <c r="L1061" s="3" t="s">
+        <v>3251</v>
+      </c>
       <c r="M1061">
         <v>2</v>
       </c>
@@ -57716,6 +58196,9 @@
         <v>0</v>
       </c>
       <c r="J1062" s="6"/>
+      <c r="L1062" s="3" t="s">
+        <v>3252</v>
+      </c>
       <c r="M1062">
         <v>2</v>
       </c>
@@ -57761,6 +58244,9 @@
         <v>0</v>
       </c>
       <c r="J1063" s="6"/>
+      <c r="L1063" s="3" t="s">
+        <v>3253</v>
+      </c>
       <c r="M1063">
         <v>2</v>
       </c>
@@ -57806,6 +58292,9 @@
         <v>0</v>
       </c>
       <c r="J1064" s="6"/>
+      <c r="L1064" s="3" t="s">
+        <v>3254</v>
+      </c>
       <c r="M1064">
         <v>2</v>
       </c>
@@ -57851,6 +58340,9 @@
         <v>0</v>
       </c>
       <c r="J1065" s="6"/>
+      <c r="L1065" s="3" t="s">
+        <v>3255</v>
+      </c>
       <c r="M1065">
         <v>2</v>
       </c>
@@ -57896,6 +58388,9 @@
         <v>0</v>
       </c>
       <c r="J1066" s="6"/>
+      <c r="L1066" s="3" t="s">
+        <v>3256</v>
+      </c>
       <c r="M1066">
         <v>2</v>
       </c>
@@ -57941,6 +58436,9 @@
         <v>0</v>
       </c>
       <c r="J1067" s="6"/>
+      <c r="L1067" s="3" t="s">
+        <v>3257</v>
+      </c>
       <c r="M1067">
         <v>2</v>
       </c>
@@ -57986,6 +58484,9 @@
         <v>0</v>
       </c>
       <c r="J1068" s="6"/>
+      <c r="L1068" s="3" t="s">
+        <v>3258</v>
+      </c>
       <c r="M1068">
         <v>2</v>
       </c>
@@ -58031,6 +58532,9 @@
         <v>0</v>
       </c>
       <c r="J1069" s="6"/>
+      <c r="L1069" s="3" t="s">
+        <v>3259</v>
+      </c>
       <c r="M1069">
         <v>2</v>
       </c>
@@ -58076,6 +58580,9 @@
         <v>0</v>
       </c>
       <c r="J1070" s="6"/>
+      <c r="L1070" s="3" t="s">
+        <v>3260</v>
+      </c>
       <c r="M1070">
         <v>2</v>
       </c>
@@ -58121,6 +58628,9 @@
         <v>0</v>
       </c>
       <c r="J1071" s="6"/>
+      <c r="L1071" s="3" t="s">
+        <v>3261</v>
+      </c>
       <c r="M1071">
         <v>2</v>
       </c>
@@ -58166,6 +58676,9 @@
         <v>0</v>
       </c>
       <c r="J1072" s="6"/>
+      <c r="L1072" s="3" t="s">
+        <v>3262</v>
+      </c>
       <c r="M1072">
         <v>2</v>
       </c>
@@ -58211,6 +58724,9 @@
         <v>0</v>
       </c>
       <c r="J1073" s="6"/>
+      <c r="L1073" s="3" t="s">
+        <v>3263</v>
+      </c>
       <c r="M1073">
         <v>2</v>
       </c>
@@ -58256,6 +58772,9 @@
         <v>0</v>
       </c>
       <c r="J1074" s="6"/>
+      <c r="L1074" s="3" t="s">
+        <v>3264</v>
+      </c>
       <c r="M1074">
         <v>2</v>
       </c>
@@ -58301,6 +58820,9 @@
         <v>0</v>
       </c>
       <c r="J1075" s="6"/>
+      <c r="L1075" s="3" t="s">
+        <v>3265</v>
+      </c>
       <c r="M1075">
         <v>2</v>
       </c>
@@ -58346,6 +58868,9 @@
         <v>0</v>
       </c>
       <c r="J1076" s="6"/>
+      <c r="L1076" s="3" t="s">
+        <v>3266</v>
+      </c>
       <c r="M1076">
         <v>2</v>
       </c>
@@ -58391,6 +58916,9 @@
         <v>0</v>
       </c>
       <c r="J1077" s="6"/>
+      <c r="L1077" s="3" t="s">
+        <v>3267</v>
+      </c>
       <c r="M1077">
         <v>2</v>
       </c>
@@ -58436,6 +58964,9 @@
         <v>0</v>
       </c>
       <c r="J1078" s="6"/>
+      <c r="L1078" s="3" t="s">
+        <v>3268</v>
+      </c>
       <c r="M1078">
         <v>2</v>
       </c>
@@ -58481,6 +59012,9 @@
         <v>0</v>
       </c>
       <c r="J1079" s="6"/>
+      <c r="L1079" s="3" t="s">
+        <v>3269</v>
+      </c>
       <c r="M1079">
         <v>2</v>
       </c>
@@ -58526,6 +59060,9 @@
         <v>0</v>
       </c>
       <c r="J1080" s="6"/>
+      <c r="L1080" s="3" t="s">
+        <v>3270</v>
+      </c>
       <c r="M1080">
         <v>2</v>
       </c>
@@ -58571,6 +59108,9 @@
         <v>0</v>
       </c>
       <c r="J1081" s="6"/>
+      <c r="L1081" s="3" t="s">
+        <v>3271</v>
+      </c>
       <c r="M1081">
         <v>2</v>
       </c>
@@ -58616,6 +59156,9 @@
         <v>0</v>
       </c>
       <c r="J1082" s="6"/>
+      <c r="L1082" s="3" t="s">
+        <v>3272</v>
+      </c>
       <c r="M1082">
         <v>2</v>
       </c>
@@ -58661,6 +59204,9 @@
         <v>0</v>
       </c>
       <c r="J1083" s="6"/>
+      <c r="L1083" s="3" t="s">
+        <v>3273</v>
+      </c>
       <c r="M1083">
         <v>2</v>
       </c>
@@ -58706,6 +59252,9 @@
         <v>0</v>
       </c>
       <c r="J1084" s="6"/>
+      <c r="L1084" s="3" t="s">
+        <v>3274</v>
+      </c>
       <c r="M1084">
         <v>2</v>
       </c>
@@ -58751,6 +59300,9 @@
         <v>0</v>
       </c>
       <c r="J1085" s="6"/>
+      <c r="L1085" s="3" t="s">
+        <v>3275</v>
+      </c>
       <c r="M1085">
         <v>2</v>
       </c>
@@ -58796,6 +59348,9 @@
         <v>0</v>
       </c>
       <c r="J1086" s="6"/>
+      <c r="L1086" s="3" t="s">
+        <v>3276</v>
+      </c>
       <c r="M1086">
         <v>2</v>
       </c>
@@ -58841,6 +59396,9 @@
         <v>0</v>
       </c>
       <c r="J1087" s="6"/>
+      <c r="L1087" s="3" t="s">
+        <v>3277</v>
+      </c>
       <c r="M1087">
         <v>2</v>
       </c>
@@ -58886,6 +59444,9 @@
         <v>0</v>
       </c>
       <c r="J1088" s="6"/>
+      <c r="L1088" s="3" t="s">
+        <v>3278</v>
+      </c>
       <c r="M1088">
         <v>2</v>
       </c>
@@ -58931,6 +59492,9 @@
         <v>0</v>
       </c>
       <c r="J1089" s="6"/>
+      <c r="L1089" s="3" t="s">
+        <v>3279</v>
+      </c>
       <c r="M1089">
         <v>2</v>
       </c>
@@ -58976,6 +59540,9 @@
         <v>0</v>
       </c>
       <c r="J1090" s="6"/>
+      <c r="L1090" s="3" t="s">
+        <v>3280</v>
+      </c>
       <c r="M1090">
         <v>2</v>
       </c>
@@ -59021,6 +59588,9 @@
         <v>0</v>
       </c>
       <c r="J1091" s="6"/>
+      <c r="L1091" s="3" t="s">
+        <v>3281</v>
+      </c>
       <c r="M1091">
         <v>2</v>
       </c>
@@ -59066,6 +59636,9 @@
         <v>0</v>
       </c>
       <c r="J1092" s="6"/>
+      <c r="L1092" s="3" t="s">
+        <v>3282</v>
+      </c>
       <c r="M1092">
         <v>2</v>
       </c>
@@ -59111,6 +59684,9 @@
         <v>0</v>
       </c>
       <c r="J1093" s="6"/>
+      <c r="L1093" s="3" t="s">
+        <v>3283</v>
+      </c>
       <c r="M1093">
         <v>2</v>
       </c>
@@ -59156,6 +59732,9 @@
         <v>0</v>
       </c>
       <c r="J1094" s="6"/>
+      <c r="L1094" s="3" t="s">
+        <v>3284</v>
+      </c>
       <c r="M1094">
         <v>2</v>
       </c>
@@ -59201,6 +59780,9 @@
         <v>0</v>
       </c>
       <c r="J1095" s="6"/>
+      <c r="L1095" s="3" t="s">
+        <v>3285</v>
+      </c>
       <c r="M1095">
         <v>2</v>
       </c>
@@ -59246,6 +59828,9 @@
         <v>0</v>
       </c>
       <c r="J1096" s="6"/>
+      <c r="L1096" s="3" t="s">
+        <v>3286</v>
+      </c>
       <c r="M1096">
         <v>2</v>
       </c>
@@ -59291,6 +59876,9 @@
         <v>0</v>
       </c>
       <c r="J1097" s="6"/>
+      <c r="L1097" s="3" t="s">
+        <v>3287</v>
+      </c>
       <c r="M1097">
         <v>2</v>
       </c>
@@ -59336,6 +59924,9 @@
         <v>0</v>
       </c>
       <c r="J1098" s="6"/>
+      <c r="L1098" s="3" t="s">
+        <v>3288</v>
+      </c>
       <c r="M1098">
         <v>2</v>
       </c>
@@ -59381,6 +59972,9 @@
         <v>0</v>
       </c>
       <c r="J1099" s="6"/>
+      <c r="L1099" s="3" t="s">
+        <v>3289</v>
+      </c>
       <c r="M1099">
         <v>2</v>
       </c>
@@ -59426,6 +60020,9 @@
         <v>0</v>
       </c>
       <c r="J1100" s="6"/>
+      <c r="L1100" s="3" t="s">
+        <v>3290</v>
+      </c>
       <c r="M1100">
         <v>2</v>
       </c>
@@ -59471,6 +60068,9 @@
         <v>0</v>
       </c>
       <c r="J1101" s="6"/>
+      <c r="L1101" s="3" t="s">
+        <v>3291</v>
+      </c>
       <c r="M1101">
         <v>2</v>
       </c>
@@ -59516,6 +60116,9 @@
         <v>0</v>
       </c>
       <c r="J1102" s="6"/>
+      <c r="L1102" s="3" t="s">
+        <v>3292</v>
+      </c>
       <c r="M1102">
         <v>2</v>
       </c>
@@ -59561,6 +60164,9 @@
         <v>0</v>
       </c>
       <c r="J1103" s="6"/>
+      <c r="L1103" s="3" t="s">
+        <v>3293</v>
+      </c>
       <c r="M1103">
         <v>2</v>
       </c>
@@ -59606,6 +60212,9 @@
         <v>0</v>
       </c>
       <c r="J1104" s="6"/>
+      <c r="L1104" s="3" t="s">
+        <v>3294</v>
+      </c>
       <c r="M1104">
         <v>2</v>
       </c>
@@ -59651,6 +60260,9 @@
         <v>0</v>
       </c>
       <c r="J1105" s="6"/>
+      <c r="L1105" s="3" t="s">
+        <v>3295</v>
+      </c>
       <c r="M1105">
         <v>2</v>
       </c>
@@ -59696,6 +60308,9 @@
         <v>0</v>
       </c>
       <c r="J1106" s="6"/>
+      <c r="L1106" s="3" t="s">
+        <v>3296</v>
+      </c>
       <c r="M1106">
         <v>2</v>
       </c>
@@ -59741,6 +60356,9 @@
         <v>0</v>
       </c>
       <c r="J1107" s="6"/>
+      <c r="L1107" s="3" t="s">
+        <v>3297</v>
+      </c>
       <c r="M1107">
         <v>2</v>
       </c>
@@ -59786,6 +60404,9 @@
         <v>0</v>
       </c>
       <c r="J1108" s="6"/>
+      <c r="L1108" s="3" t="s">
+        <v>3298</v>
+      </c>
       <c r="M1108">
         <v>2</v>
       </c>
@@ -59831,6 +60452,9 @@
         <v>0</v>
       </c>
       <c r="J1109" s="6"/>
+      <c r="L1109" s="3" t="s">
+        <v>3299</v>
+      </c>
       <c r="M1109">
         <v>2</v>
       </c>
@@ -59876,6 +60500,9 @@
         <v>0</v>
       </c>
       <c r="J1110" s="6"/>
+      <c r="L1110" s="3" t="s">
+        <v>3300</v>
+      </c>
       <c r="M1110">
         <v>2</v>
       </c>
@@ -79726,9 +80353,112 @@
     <hyperlink ref="L1156" r:id="rId445" xr:uid="{4C737807-DA25-4B3C-BE08-C21879564672}"/>
     <hyperlink ref="L1157" r:id="rId446" xr:uid="{CF680533-4ABC-4AF1-9F1F-0B7829E3B08A}"/>
     <hyperlink ref="L1158" r:id="rId447" xr:uid="{C936BFF0-FD22-47E0-B892-5339F7C0D628}"/>
+    <hyperlink ref="L1018" r:id="rId448" xr:uid="{85A9131B-5685-4F66-A9AE-F88E00539263}"/>
+    <hyperlink ref="L1019" r:id="rId449" xr:uid="{FFDB8E7D-8448-41B7-B8D9-574230F80D22}"/>
+    <hyperlink ref="L1020" r:id="rId450" xr:uid="{407FCB5E-F7B8-458A-AA59-FF58FE33EFF2}"/>
+    <hyperlink ref="L1021" r:id="rId451" xr:uid="{7D6D60AB-D5F7-497F-8AB8-F8FBB2FFBFB0}"/>
+    <hyperlink ref="L1022:L1028" r:id="rId452" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2019.json" xr:uid="{EE5EAAD9-E0E8-4D74-BC25-D631DF31423F}"/>
+    <hyperlink ref="L1022" r:id="rId453" xr:uid="{11588CAA-AE84-4313-AE8B-F0F7AC07E497}"/>
+    <hyperlink ref="L1023" r:id="rId454" xr:uid="{599FDDAA-7684-45EB-8D92-92CD220EB07E}"/>
+    <hyperlink ref="L1024" r:id="rId455" xr:uid="{7A91ACA0-C608-4C23-AD9B-5E81DFD76D4E}"/>
+    <hyperlink ref="L1025" r:id="rId456" xr:uid="{394CF502-435F-419B-ABEF-855604B512BA}"/>
+    <hyperlink ref="L1026" r:id="rId457" xr:uid="{CFD80DA1-C7BE-4F10-805C-25F385386C51}"/>
+    <hyperlink ref="L1027" r:id="rId458" xr:uid="{610ABCFF-4278-48A9-8382-D1BF24F836C0}"/>
+    <hyperlink ref="L1028" r:id="rId459" xr:uid="{6910793A-7FAE-49A0-B25F-537B9449E24B}"/>
+    <hyperlink ref="L1029:L1030" r:id="rId460" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2019.json" xr:uid="{9D6EBF13-D381-4C67-8782-E91760BAE8A0}"/>
+    <hyperlink ref="L1029" r:id="rId461" xr:uid="{30FE3909-1222-46CC-B07E-D2442EEE8D50}"/>
+    <hyperlink ref="L1030" r:id="rId462" xr:uid="{A678B830-F250-4875-9F60-B6D13E095343}"/>
+    <hyperlink ref="L1031:L1032" r:id="rId463" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/bz__annual_mean__ug_m3__2019.json" xr:uid="{CC3B9A7E-E372-459E-AE6A-7D0263E98CE5}"/>
+    <hyperlink ref="L1031" r:id="rId464" xr:uid="{2A6F2134-A328-4F79-A361-B26927210E5D}"/>
+    <hyperlink ref="L1032" r:id="rId465" xr:uid="{82AA3813-0653-4BEF-912A-6784B2B832D3}"/>
+    <hyperlink ref="L1033" r:id="rId466" xr:uid="{794F9753-A2D0-43B7-B13F-5F18E937DB6B}"/>
+    <hyperlink ref="L1034" r:id="rId467" xr:uid="{F65A3A07-83B7-404F-B557-1921BF9E3D7C}"/>
+    <hyperlink ref="L1035" r:id="rId468" xr:uid="{9EBCA301-F149-47E6-9BA7-8E4C3E4056D9}"/>
+    <hyperlink ref="L1036" r:id="rId469" xr:uid="{2DCBD81D-AD47-46BE-94FA-DAC719864412}"/>
+    <hyperlink ref="L1037:L1043" r:id="rId470" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2019.json" xr:uid="{786091A8-46C0-46D3-AFA5-100E2A097C6E}"/>
+    <hyperlink ref="L1037" r:id="rId471" xr:uid="{8F4183DC-5003-435C-97A8-776D5CBBD281}"/>
+    <hyperlink ref="L1038" r:id="rId472" xr:uid="{32C36E27-8E82-4EEE-8C8B-DE96B59E0EE3}"/>
+    <hyperlink ref="L1039" r:id="rId473" xr:uid="{EBE9F38A-8A86-4A60-A621-F650B99C78E9}"/>
+    <hyperlink ref="L1040" r:id="rId474" xr:uid="{327BAF9C-4998-42B6-A04C-4CA76B0E33B0}"/>
+    <hyperlink ref="L1041" r:id="rId475" xr:uid="{B65AE598-CF59-4D7A-9A99-CE077F2F8578}"/>
+    <hyperlink ref="L1042" r:id="rId476" xr:uid="{0FDB2EDD-80D2-4D0F-9C46-B5F3027580A3}"/>
+    <hyperlink ref="L1043" r:id="rId477" xr:uid="{BA717DC7-5CB2-4B75-8AF1-6D2F12816342}"/>
+    <hyperlink ref="L1044:L1045" r:id="rId478" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/no2__annual_mean__ug_m3__2019.json" xr:uid="{5F8285EC-E7E9-4D6D-85FA-028031A19235}"/>
+    <hyperlink ref="L1044" r:id="rId479" xr:uid="{1AC75627-89E4-4F6B-8C77-21EF99664C3F}"/>
+    <hyperlink ref="L1045" r:id="rId480" xr:uid="{0A6B3F44-E3EC-4848-AD11-8C2AE2F8CC63}"/>
+    <hyperlink ref="L1046" r:id="rId481" xr:uid="{2AD4BFCD-F484-4234-89EA-C38B1622829F}"/>
+    <hyperlink ref="L1047" r:id="rId482" xr:uid="{BBD37B84-6F8B-4379-841C-A9638C23DAD1}"/>
+    <hyperlink ref="L1048" r:id="rId483" xr:uid="{6842A1D5-36E9-41AC-BABB-59D170A5ECA7}"/>
+    <hyperlink ref="L1049" r:id="rId484" xr:uid="{5B844D9A-A5DB-4ADF-82B1-08E8D86A63AA}"/>
+    <hyperlink ref="L1050" r:id="rId485" xr:uid="{C3B3AC69-894A-44DC-B4B5-CE50C4E3A23E}"/>
+    <hyperlink ref="L1051" r:id="rId486" xr:uid="{52834128-7E33-4EC4-90C2-51970485CD54}"/>
+    <hyperlink ref="L1052" r:id="rId487" xr:uid="{B25D4069-9248-4FE4-9374-BD7EB5B9D2B1}"/>
+    <hyperlink ref="L1053" r:id="rId488" xr:uid="{5EE1E688-0519-4484-8D67-CE819FD710F7}"/>
+    <hyperlink ref="L1054" r:id="rId489" xr:uid="{6799419C-DBBB-48D8-B1C0-84E22C5ECFD7}"/>
+    <hyperlink ref="L1055" r:id="rId490" xr:uid="{C46E2A92-79E2-4DAD-B0C6-A7437DCD2562}"/>
+    <hyperlink ref="L1056" r:id="rId491" xr:uid="{5C2BBE2E-AAF7-4C58-8444-4FB22846ABDB}"/>
+    <hyperlink ref="L1057" r:id="rId492" xr:uid="{0BE1D659-C84A-401F-A9B6-18064BF9C049}"/>
+    <hyperlink ref="L1058" r:id="rId493" xr:uid="{AB0A5D1B-129A-4656-AA8A-16C9ED7853D0}"/>
+    <hyperlink ref="L1059" r:id="rId494" xr:uid="{7D3FF192-8C44-47F4-9877-1D1F8A769EAC}"/>
+    <hyperlink ref="L1060:L1061" r:id="rId495" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2022.json" xr:uid="{A5612EE1-5A69-405E-A095-2A7F21480433}"/>
+    <hyperlink ref="L1060" r:id="rId496" xr:uid="{D912D51A-19C0-4ED0-A352-B396D744541E}"/>
+    <hyperlink ref="L1061" r:id="rId497" xr:uid="{17D0AEA5-4458-4129-B962-7F2F825A293A}"/>
+    <hyperlink ref="L1062" r:id="rId498" xr:uid="{A2166901-E5BD-4EC2-B11F-9924B8A8A854}"/>
+    <hyperlink ref="L1063:L1067" r:id="rId499" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2019.json" xr:uid="{634B0DE9-1685-4B7E-A8F9-F418159FEE38}"/>
+    <hyperlink ref="L1063" r:id="rId500" xr:uid="{42DCC152-1EFF-4C84-B2D6-1E890299B126}"/>
+    <hyperlink ref="L1064" r:id="rId501" xr:uid="{AD4F091C-FC4B-402A-BE71-153611DB887F}"/>
+    <hyperlink ref="L1065" r:id="rId502" xr:uid="{A238315C-A63D-436A-BC23-14B881A8EFE6}"/>
+    <hyperlink ref="L1066" r:id="rId503" xr:uid="{940BB13F-28F8-4BAD-9EF7-B170307C33F1}"/>
+    <hyperlink ref="L1067" r:id="rId504" xr:uid="{F5D534C1-3C36-4505-BEBE-EE3CA5DBBD3F}"/>
+    <hyperlink ref="L1068:L1070" r:id="rId505" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/dgt_120__2019.json" xr:uid="{2C235762-42FD-46AB-A15B-8A758808E074}"/>
+    <hyperlink ref="L1068" r:id="rId506" xr:uid="{6A636136-01E6-4A27-8427-2B8A02EAF8E1}"/>
+    <hyperlink ref="L1069" r:id="rId507" xr:uid="{142DB99F-2B8C-4D04-B4F1-59B094CB000A}"/>
+    <hyperlink ref="L1070" r:id="rId508" xr:uid="{98B44F81-3257-44E9-93EF-2D2680FA9B3F}"/>
+    <hyperlink ref="L1071" r:id="rId509" xr:uid="{F757E6D9-A83F-44BF-866D-E97914A0EEF1}"/>
+    <hyperlink ref="L1072" r:id="rId510" xr:uid="{B7D236C4-CF76-4D9D-8B10-A4537334B2F1}"/>
+    <hyperlink ref="L1073:L1075" r:id="rId511" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2022_g.json" xr:uid="{34FDA581-4BE9-49A9-86AC-29340E2AD4FC}"/>
+    <hyperlink ref="L1073" r:id="rId512" xr:uid="{467FFD2A-0E33-4ABA-A371-4AB2E2D36928}"/>
+    <hyperlink ref="L1074" r:id="rId513" xr:uid="{CF3F3CA1-D8EF-4553-A7D3-38BD4A5CED26}"/>
+    <hyperlink ref="L1075" r:id="rId514" xr:uid="{2E3E4A4D-B041-4900-863F-889B3B496BBB}"/>
+    <hyperlink ref="L1076:L1082" r:id="rId515" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2022_g.json" xr:uid="{D84A3343-37F7-4E63-AED2-FCC9826E5414}"/>
+    <hyperlink ref="L1076" r:id="rId516" xr:uid="{CD9226FC-CCDB-4E10-AD81-EC70F1B66AEB}"/>
+    <hyperlink ref="L1077" r:id="rId517" xr:uid="{6EDE82E7-6307-45A1-89C1-DA43099D65FA}"/>
+    <hyperlink ref="L1078" r:id="rId518" xr:uid="{D0FCA14E-C91D-4152-8401-3958F74B0B87}"/>
+    <hyperlink ref="L1079" r:id="rId519" xr:uid="{0134FAB6-97AD-4F55-8977-9C308F82728B}"/>
+    <hyperlink ref="L1080" r:id="rId520" xr:uid="{F14A7EF9-9F16-463B-898D-E472DEB26252}"/>
+    <hyperlink ref="L1082" r:id="rId521" xr:uid="{102C6100-0479-4C7D-A0B0-153497B43490}"/>
+    <hyperlink ref="L1083:L1084" r:id="rId522" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/pm25__annual_mean__ug_m3__2022_g.json" xr:uid="{5679949B-8FDA-4151-B4B8-6B88F85CA6ED}"/>
+    <hyperlink ref="L1083" r:id="rId523" xr:uid="{AD625A51-2630-4F28-A865-A633B39BA3EF}"/>
+    <hyperlink ref="L1084" r:id="rId524" xr:uid="{FB2C70E0-B553-4430-9F1B-3F16E11E6620}"/>
+    <hyperlink ref="L1085" r:id="rId525" xr:uid="{25885C4B-DDF7-4C70-86D3-B661FC0B9DDE}"/>
+    <hyperlink ref="L1086" r:id="rId526" xr:uid="{05BE2495-501F-40B6-903E-76C754CBFB2D}"/>
+    <hyperlink ref="L1087" r:id="rId527" xr:uid="{AC7022D2-1D7A-4809-B08A-E04C8728D455}"/>
+    <hyperlink ref="L1088" r:id="rId528" xr:uid="{AE7ED104-43A5-4E9C-9FAC-AB5C9B0F282C}"/>
+    <hyperlink ref="L1089" r:id="rId529" xr:uid="{AA81A0A3-AB0B-4966-90A8-C1E5E7CF6FDC}"/>
+    <hyperlink ref="L1090" r:id="rId530" xr:uid="{12DF25B9-5061-4991-9983-7C22A4585FCF}"/>
+    <hyperlink ref="L1091" r:id="rId531" xr:uid="{92E3397B-2C32-4D0C-87CA-8FCAAB9E648E}"/>
+    <hyperlink ref="L1092" r:id="rId532" xr:uid="{6DF878FC-48D0-4F5C-BBBB-F13B3DBECBC9}"/>
+    <hyperlink ref="L1093" r:id="rId533" xr:uid="{6DFB5BF9-BD00-4915-ACA9-D2C3FA96FF1B}"/>
+    <hyperlink ref="L1094" r:id="rId534" xr:uid="{180F5927-0FB7-4F96-ADAC-799B08A16116}"/>
+    <hyperlink ref="L1095" r:id="rId535" xr:uid="{E264D8FB-9808-4B94-9903-732C2582D462}"/>
+    <hyperlink ref="L1096" r:id="rId536" xr:uid="{C9A0B431-D3C8-4633-A6AA-23793FB626AF}"/>
+    <hyperlink ref="L1097" r:id="rId537" xr:uid="{E229DE6F-F669-48EA-A941-887D2A8598DE}"/>
+    <hyperlink ref="L1098" r:id="rId538" xr:uid="{1B96A0A3-7FAF-4F7E-9ABB-6541AFE105EA}"/>
+    <hyperlink ref="L1099" r:id="rId539" xr:uid="{EF5701F3-C866-4F17-9579-AB7E0A801BD3}"/>
+    <hyperlink ref="L1100" r:id="rId540" xr:uid="{DD46443B-1D37-497B-AF17-921EEBF6D131}"/>
+    <hyperlink ref="L1101" r:id="rId541" xr:uid="{2418AE7C-D9E2-4B53-B8E8-00A491BD6B24}"/>
+    <hyperlink ref="L1102" r:id="rId542" xr:uid="{80531937-158B-4D00-8E5D-CFA976C15507}"/>
+    <hyperlink ref="L1103" r:id="rId543" xr:uid="{75720B30-AF9A-48E1-9AB7-0997661F0FA2}"/>
+    <hyperlink ref="L1104" r:id="rId544" xr:uid="{7E3A8FDB-C601-4A66-B837-10A7361BA702}"/>
+    <hyperlink ref="L1105" r:id="rId545" xr:uid="{BF518131-581B-4316-B777-487A583CEFC9}"/>
+    <hyperlink ref="L1106" r:id="rId546" xr:uid="{21150F5A-3051-413A-9A15-92361F513FB5}"/>
+    <hyperlink ref="L1107" r:id="rId547" xr:uid="{643ABB3E-A671-475F-BA65-2247B7CFBF4A}"/>
+    <hyperlink ref="L1108" r:id="rId548" xr:uid="{156E5320-324A-46A9-83F8-B4EFDEECD6C8}"/>
+    <hyperlink ref="L1109" r:id="rId549" xr:uid="{665C61A8-134F-442F-98D5-81FFD9A3B965}"/>
+    <hyperlink ref="L1110" r:id="rId550" xr:uid="{9372FBA2-CD81-4F9B-B049-5FD85AD034A7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId448"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId551"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: noise level urls added
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EC4F1E-F6BB-44F4-9C2E-4936F42FDC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA96BF9-5874-49A0-8939-464E075D85B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6591" uniqueCount="3301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6599" uniqueCount="3309">
   <si>
     <t>DbId</t>
   </si>
@@ -9944,6 +9944,30 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/ModelledBackgroundPollution/so2__annual_mean__ug_m3__2010.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Environmental_Noise_Directive_Noise_Mapping_Agglomerations_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Road_Noise_Lnight_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Road_Noise_Lden_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Road_Noise_LAeq_16h_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Rail_Noise_Lnight_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Rail_Noise_Lden_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Rail_Noise_LAeq_16h_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Noise_Action_Planning_Important_Areas_Round_3.json</t>
   </si>
 </sst>
 </file>
@@ -10564,6 +10588,9 @@
       <c r="G5">
         <v>3000</v>
       </c>
+      <c r="H5" s="3" t="s">
+        <v>3308</v>
+      </c>
       <c r="I5">
         <v>2</v>
       </c>
@@ -10835,6 +10862,7 @@
     <hyperlink ref="H7" r:id="rId2" xr:uid="{D75E7FAE-D953-4BAD-9FB5-353B5789F8AB}"/>
     <hyperlink ref="H8" r:id="rId3" xr:uid="{B1632C55-A38E-4D56-A2E2-F9D7C9F4331A}"/>
     <hyperlink ref="H9" r:id="rId4" xr:uid="{8C4ADDA5-96A2-4CD2-9BE8-8E08E00E0EE1}"/>
+    <hyperlink ref="H5" r:id="rId5" xr:uid="{FF63FA53-105B-4DCF-9427-D386BFA3F0E8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -12019,6 +12047,7 @@
       <c r="M21">
         <v>2006</v>
       </c>
+      <c r="O21" s="3"/>
       <c r="P21">
         <v>2</v>
       </c>
@@ -12072,6 +12101,9 @@
       <c r="M22">
         <v>3001</v>
       </c>
+      <c r="O22" s="3" t="s">
+        <v>3302</v>
+      </c>
       <c r="P22">
         <v>2</v>
       </c>
@@ -12125,6 +12157,9 @@
       <c r="M23">
         <v>3002</v>
       </c>
+      <c r="O23" s="3" t="s">
+        <v>3303</v>
+      </c>
       <c r="P23">
         <v>2</v>
       </c>
@@ -12178,6 +12213,9 @@
       <c r="M24">
         <v>3003</v>
       </c>
+      <c r="O24" s="3" t="s">
+        <v>3304</v>
+      </c>
       <c r="P24">
         <v>2</v>
       </c>
@@ -12231,6 +12269,9 @@
       <c r="M25">
         <v>3004</v>
       </c>
+      <c r="O25" s="3" t="s">
+        <v>3305</v>
+      </c>
       <c r="P25">
         <v>2</v>
       </c>
@@ -12284,6 +12325,9 @@
       <c r="M26">
         <v>3005</v>
       </c>
+      <c r="O26" s="3" t="s">
+        <v>3306</v>
+      </c>
       <c r="P26">
         <v>2</v>
       </c>
@@ -12337,6 +12381,9 @@
       <c r="M27">
         <v>3006</v>
       </c>
+      <c r="O27" s="3" t="s">
+        <v>3307</v>
+      </c>
       <c r="P27">
         <v>2</v>
       </c>
@@ -12390,6 +12437,9 @@
       <c r="M28">
         <v>3007</v>
       </c>
+      <c r="O28" s="3" t="s">
+        <v>3301</v>
+      </c>
       <c r="P28">
         <v>2</v>
       </c>
@@ -12443,6 +12493,7 @@
       <c r="M29">
         <v>4001</v>
       </c>
+      <c r="O29" s="3"/>
       <c r="P29">
         <v>2</v>
       </c>
@@ -14673,6 +14724,12 @@
     <hyperlink ref="O32" r:id="rId39" xr:uid="{B0A928E1-5A9D-4904-925C-B849C701CBE6}"/>
     <hyperlink ref="O31" r:id="rId40" xr:uid="{DE66E62C-23D8-409B-8828-A2B1F7104694}"/>
     <hyperlink ref="O30" r:id="rId41" xr:uid="{7F69EBA1-2661-4784-B19E-BB4CCA00E309}"/>
+    <hyperlink ref="O28" r:id="rId42" xr:uid="{CF6A1E08-AF38-4E47-BDD3-65A0F83099E2}"/>
+    <hyperlink ref="O23" r:id="rId43" xr:uid="{AB2AEF75-2B89-4336-A0E7-2603A34E2C13}"/>
+    <hyperlink ref="O24" r:id="rId44" xr:uid="{64F05A85-03DC-45CF-8143-21651CEB6A98}"/>
+    <hyperlink ref="O25" r:id="rId45" xr:uid="{E5D04D95-49C3-477F-A7E3-1A8B51774504}"/>
+    <hyperlink ref="O26" r:id="rId46" xr:uid="{2FED63F0-811E-4A6F-9493-69C015A2AC1D}"/>
+    <hyperlink ref="O27" r:id="rId47" xr:uid="{72F2FDFB-8D42-449F-BDA1-2EF6464AB23C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: added links for climatejust variables
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA96BF9-5874-49A0-8939-464E075D85B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A5F052-D4F1-4D37-AAE6-C2AB9E342E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6599" uniqueCount="3309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6605" uniqueCount="3315">
   <si>
     <t>DbId</t>
   </si>
@@ -9968,6 +9968,24 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise /Level3/EN_Noise_Action_Planning_Important_Areas_Round_3.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/EN_Grid_Heat.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/EN_LSOA_2011_BFC_V3_2022_CJ.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/WA_LSOA_2011_BFC_V3_2022_CJ.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/EN_MSOA_2011_SHVI_CJ.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/UK_Grid_UKCP18_CJ.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/UK_LSOA_2011_Flood_Data_CJ.json</t>
   </si>
 </sst>
 </file>
@@ -11782,6 +11800,9 @@
       <c r="M16">
         <v>2001</v>
       </c>
+      <c r="O16" s="3" t="s">
+        <v>3309</v>
+      </c>
       <c r="P16">
         <v>2</v>
       </c>
@@ -11835,6 +11856,9 @@
       <c r="M17">
         <v>2002</v>
       </c>
+      <c r="O17" s="3" t="s">
+        <v>3310</v>
+      </c>
       <c r="P17">
         <v>2</v>
       </c>
@@ -11888,6 +11912,9 @@
       <c r="M18">
         <v>2003</v>
       </c>
+      <c r="O18" s="3" t="s">
+        <v>3312</v>
+      </c>
       <c r="P18">
         <v>2</v>
       </c>
@@ -11941,6 +11968,9 @@
       <c r="M19">
         <v>2004</v>
       </c>
+      <c r="O19" s="3" t="s">
+        <v>3313</v>
+      </c>
       <c r="P19">
         <v>2</v>
       </c>
@@ -11994,6 +12024,9 @@
       <c r="M20">
         <v>2005</v>
       </c>
+      <c r="O20" s="3" t="s">
+        <v>3314</v>
+      </c>
       <c r="P20">
         <v>2</v>
       </c>
@@ -12047,7 +12080,9 @@
       <c r="M21">
         <v>2006</v>
       </c>
-      <c r="O21" s="3"/>
+      <c r="O21" s="3" t="s">
+        <v>3311</v>
+      </c>
       <c r="P21">
         <v>2</v>
       </c>
@@ -14730,6 +14765,12 @@
     <hyperlink ref="O25" r:id="rId45" xr:uid="{E5D04D95-49C3-477F-A7E3-1A8B51774504}"/>
     <hyperlink ref="O26" r:id="rId46" xr:uid="{2FED63F0-811E-4A6F-9493-69C015A2AC1D}"/>
     <hyperlink ref="O27" r:id="rId47" xr:uid="{72F2FDFB-8D42-449F-BDA1-2EF6464AB23C}"/>
+    <hyperlink ref="O16" r:id="rId48" xr:uid="{3817A9EF-DEC2-42F4-BC65-6C8B01E3147F}"/>
+    <hyperlink ref="O17" r:id="rId49" xr:uid="{0BB7BCDC-3B19-4AD9-ABC8-5F927DB382BD}"/>
+    <hyperlink ref="O18" r:id="rId50" xr:uid="{D43D9927-3B4E-405E-8C05-78E889C82752}"/>
+    <hyperlink ref="O19" r:id="rId51" xr:uid="{D537EB9A-51DD-48F7-9457-FD32A5E9864B}"/>
+    <hyperlink ref="O20" r:id="rId52" xr:uid="{521DDBB9-66B8-4124-AF2F-E5E8F789B155}"/>
+    <hyperlink ref="O21" r:id="rId53" xr:uid="{74B2F229-A063-45D4-8571-63C642C1E2BC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: added urls to climatejust variables of the config and highlighted some issues in the info-descriptions one
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE60840-B9A9-4942-B697-92D766CE6589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D2EFF0-C3AF-4CD9-A13F-86E15B06AE01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6606" uniqueCount="3316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6635" uniqueCount="3345">
   <si>
     <t>DbId</t>
   </si>
@@ -9989,6 +9989,93 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-101.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-102.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-103.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-104.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-105.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-106.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-107.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-108.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-109.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-110.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-111.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-112.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-113.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-114.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-115.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-116.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-117.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-118.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-119.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-120.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-122.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-123.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-130.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-131.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-132.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-201.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-202.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-203.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-204.json</t>
   </si>
 </sst>
 </file>
@@ -23987,6 +24074,9 @@
         <v>0</v>
       </c>
       <c r="J231" s="6"/>
+      <c r="L231" s="3" t="s">
+        <v>3341</v>
+      </c>
       <c r="M231">
         <v>2</v>
       </c>
@@ -28187,6 +28277,9 @@
         <v>0</v>
       </c>
       <c r="J336" s="6"/>
+      <c r="L336" s="3" t="s">
+        <v>3343</v>
+      </c>
       <c r="M336">
         <v>2</v>
       </c>
@@ -46947,6 +47040,9 @@
         <v>0</v>
       </c>
       <c r="J787" s="6"/>
+      <c r="L787" s="3" t="s">
+        <v>3327</v>
+      </c>
       <c r="M787">
         <v>2</v>
       </c>
@@ -46987,6 +47083,9 @@
         <v>0</v>
       </c>
       <c r="J788" s="6"/>
+      <c r="L788" s="3" t="s">
+        <v>3338</v>
+      </c>
       <c r="M788">
         <v>2</v>
       </c>
@@ -47027,6 +47126,7 @@
         <v>0</v>
       </c>
       <c r="J789" s="6"/>
+      <c r="L789" s="3"/>
       <c r="M789">
         <v>2</v>
       </c>
@@ -47067,6 +47167,7 @@
         <v>0</v>
       </c>
       <c r="J790" s="6"/>
+      <c r="L790" s="3"/>
       <c r="M790">
         <v>2</v>
       </c>
@@ -47107,6 +47208,9 @@
         <v>0</v>
       </c>
       <c r="J791" s="6"/>
+      <c r="L791" s="3" t="s">
+        <v>3325</v>
+      </c>
       <c r="M791">
         <v>2</v>
       </c>
@@ -47267,6 +47371,9 @@
         <v>0</v>
       </c>
       <c r="J795" s="6"/>
+      <c r="L795" s="3" t="s">
+        <v>3337</v>
+      </c>
       <c r="M795">
         <v>2</v>
       </c>
@@ -47307,6 +47414,7 @@
         <v>0</v>
       </c>
       <c r="J796" s="6"/>
+      <c r="L796" s="3"/>
       <c r="M796">
         <v>2</v>
       </c>
@@ -47347,6 +47455,9 @@
         <v>0</v>
       </c>
       <c r="J797" s="6"/>
+      <c r="L797" s="3" t="s">
+        <v>3336</v>
+      </c>
       <c r="M797">
         <v>2</v>
       </c>
@@ -47387,6 +47498,9 @@
         <v>0</v>
       </c>
       <c r="J798" s="6"/>
+      <c r="L798" s="3" t="s">
+        <v>3340</v>
+      </c>
       <c r="M798">
         <v>2</v>
       </c>
@@ -47427,6 +47541,9 @@
         <v>0</v>
       </c>
       <c r="J799" s="6"/>
+      <c r="L799" s="3" t="s">
+        <v>3320</v>
+      </c>
       <c r="M799">
         <v>2</v>
       </c>
@@ -47467,6 +47584,9 @@
         <v>0</v>
       </c>
       <c r="J800" s="6"/>
+      <c r="L800" s="3" t="s">
+        <v>3323</v>
+      </c>
       <c r="M800">
         <v>2</v>
       </c>
@@ -47507,6 +47627,9 @@
         <v>0</v>
       </c>
       <c r="J801" s="6"/>
+      <c r="L801" s="3" t="s">
+        <v>3324</v>
+      </c>
       <c r="M801">
         <v>2</v>
       </c>
@@ -47547,6 +47670,7 @@
         <v>0</v>
       </c>
       <c r="J802" s="6"/>
+      <c r="L802" s="3"/>
       <c r="M802">
         <v>2</v>
       </c>
@@ -47587,6 +47711,9 @@
         <v>0</v>
       </c>
       <c r="J803" s="6"/>
+      <c r="L803" s="3" t="s">
+        <v>3316</v>
+      </c>
       <c r="M803">
         <v>2</v>
       </c>
@@ -47827,6 +47954,9 @@
         <v>0</v>
       </c>
       <c r="J809" s="6"/>
+      <c r="L809" s="3" t="s">
+        <v>3334</v>
+      </c>
       <c r="M809">
         <v>2</v>
       </c>
@@ -47867,6 +47997,9 @@
         <v>0</v>
       </c>
       <c r="J810" s="6"/>
+      <c r="L810" s="3" t="s">
+        <v>3318</v>
+      </c>
       <c r="M810">
         <v>2</v>
       </c>
@@ -47907,6 +48040,9 @@
         <v>0</v>
       </c>
       <c r="J811" s="6"/>
+      <c r="L811" s="3" t="s">
+        <v>3319</v>
+      </c>
       <c r="M811">
         <v>2</v>
       </c>
@@ -47947,6 +48083,9 @@
         <v>0</v>
       </c>
       <c r="J812" s="6"/>
+      <c r="L812" s="3" t="s">
+        <v>3333</v>
+      </c>
       <c r="M812">
         <v>2</v>
       </c>
@@ -47987,6 +48126,9 @@
         <v>0</v>
       </c>
       <c r="J813" s="6"/>
+      <c r="L813" s="3" t="s">
+        <v>3330</v>
+      </c>
       <c r="M813">
         <v>2</v>
       </c>
@@ -48627,6 +48769,9 @@
         <v>0</v>
       </c>
       <c r="J829" s="6"/>
+      <c r="L829" s="3" t="s">
+        <v>3339</v>
+      </c>
       <c r="M829">
         <v>2</v>
       </c>
@@ -48667,6 +48812,9 @@
         <v>0</v>
       </c>
       <c r="J830" s="6"/>
+      <c r="L830" s="3" t="s">
+        <v>3331</v>
+      </c>
       <c r="M830">
         <v>2</v>
       </c>
@@ -48707,6 +48855,9 @@
         <v>0</v>
       </c>
       <c r="J831" s="6"/>
+      <c r="L831" s="3" t="s">
+        <v>3322</v>
+      </c>
       <c r="M831">
         <v>2</v>
       </c>
@@ -48747,6 +48898,7 @@
         <v>0</v>
       </c>
       <c r="J832" s="6"/>
+      <c r="L832" s="3"/>
       <c r="M832">
         <v>2</v>
       </c>
@@ -48787,6 +48939,9 @@
         <v>0</v>
       </c>
       <c r="J833" s="6"/>
+      <c r="L833" s="3" t="s">
+        <v>3335</v>
+      </c>
       <c r="M833">
         <v>2</v>
       </c>
@@ -48827,6 +48982,7 @@
         <v>0</v>
       </c>
       <c r="J834" s="6"/>
+      <c r="L834" s="3"/>
       <c r="M834">
         <v>2</v>
       </c>
@@ -48867,6 +49023,7 @@
         <v>0</v>
       </c>
       <c r="J835" s="6"/>
+      <c r="L835" s="3"/>
       <c r="M835">
         <v>2</v>
       </c>
@@ -48907,6 +49064,9 @@
         <v>0</v>
       </c>
       <c r="J836" s="6"/>
+      <c r="L836" s="3" t="s">
+        <v>3321</v>
+      </c>
       <c r="M836">
         <v>2</v>
       </c>
@@ -48947,6 +49107,9 @@
         <v>0</v>
       </c>
       <c r="J837" s="6"/>
+      <c r="L837" s="3" t="s">
+        <v>3326</v>
+      </c>
       <c r="M837">
         <v>2</v>
       </c>
@@ -48987,6 +49150,9 @@
         <v>0</v>
       </c>
       <c r="J838" s="6"/>
+      <c r="L838" s="3" t="s">
+        <v>3328</v>
+      </c>
       <c r="M838">
         <v>2</v>
       </c>
@@ -49027,6 +49193,9 @@
         <v>0</v>
       </c>
       <c r="J839" s="6"/>
+      <c r="L839" s="3" t="s">
+        <v>3332</v>
+      </c>
       <c r="M839">
         <v>2</v>
       </c>
@@ -49067,6 +49236,7 @@
         <v>0</v>
       </c>
       <c r="J840" s="6"/>
+      <c r="L840" s="3"/>
       <c r="M840">
         <v>2</v>
       </c>
@@ -49107,6 +49277,9 @@
         <v>0</v>
       </c>
       <c r="J841" s="6"/>
+      <c r="L841" s="3" t="s">
+        <v>3329</v>
+      </c>
       <c r="M841">
         <v>2</v>
       </c>
@@ -49147,6 +49320,9 @@
         <v>0</v>
       </c>
       <c r="J842" s="6"/>
+      <c r="L842" s="3" t="s">
+        <v>3317</v>
+      </c>
       <c r="M842">
         <v>2</v>
       </c>
@@ -49667,6 +49843,9 @@
         <v>0</v>
       </c>
       <c r="J855" s="6"/>
+      <c r="L855" s="3" t="s">
+        <v>3342</v>
+      </c>
       <c r="M855">
         <v>2</v>
       </c>
@@ -53787,6 +53966,9 @@
         <v>0</v>
       </c>
       <c r="J958" s="6"/>
+      <c r="L958" s="3" t="s">
+        <v>3344</v>
+      </c>
       <c r="M958">
         <v>2</v>
       </c>
@@ -80562,9 +80744,38 @@
     <hyperlink ref="L1108" r:id="rId548" xr:uid="{156E5320-324A-46A9-83F8-B4EFDEECD6C8}"/>
     <hyperlink ref="L1109" r:id="rId549" xr:uid="{665C61A8-134F-442F-98D5-81FFD9A3B965}"/>
     <hyperlink ref="L1110" r:id="rId550" xr:uid="{9372FBA2-CD81-4F9B-B049-5FD85AD034A7}"/>
+    <hyperlink ref="L803" r:id="rId551" xr:uid="{E7A4C19A-12C2-42A2-8673-C3768AB93009}"/>
+    <hyperlink ref="L842" r:id="rId552" xr:uid="{B8D06407-52A3-45EC-A1F9-1DDB45EC101B}"/>
+    <hyperlink ref="L810" r:id="rId553" xr:uid="{F5708804-9705-46D4-801C-EBD036F5B411}"/>
+    <hyperlink ref="L811" r:id="rId554" xr:uid="{0D29EF0B-288E-49B1-A739-6002748759CF}"/>
+    <hyperlink ref="L799" r:id="rId555" xr:uid="{C51CC765-CEBD-4790-930E-BDA5930D873C}"/>
+    <hyperlink ref="L836" r:id="rId556" xr:uid="{FF818180-4BE8-43AD-9049-CEF4C8939E30}"/>
+    <hyperlink ref="L831" r:id="rId557" xr:uid="{37EFB9A7-9147-4734-932A-83C2E1C2B9EF}"/>
+    <hyperlink ref="L800" r:id="rId558" xr:uid="{5DF17578-F967-4E0A-A51F-BE78DB0DF4B2}"/>
+    <hyperlink ref="L801" r:id="rId559" xr:uid="{DDE2A222-0F0C-419E-B63C-BDBEF7F8CFFA}"/>
+    <hyperlink ref="L791" r:id="rId560" xr:uid="{754831BB-AFEC-4FE4-8452-E6FCE5C23A4C}"/>
+    <hyperlink ref="L837" r:id="rId561" xr:uid="{209779CC-9626-4546-B819-F9AFCB5083C2}"/>
+    <hyperlink ref="L787" r:id="rId562" xr:uid="{B699DB45-A67A-4A59-B809-DE414AB48D14}"/>
+    <hyperlink ref="L838" r:id="rId563" xr:uid="{8177588D-2302-429A-BB6A-86BE04DC90A6}"/>
+    <hyperlink ref="L841" r:id="rId564" xr:uid="{51CAE882-65BC-4394-8F1C-60E1E7C02EBB}"/>
+    <hyperlink ref="L813" r:id="rId565" xr:uid="{7BE4653C-D870-4126-AAA9-23C1DD74403D}"/>
+    <hyperlink ref="L830" r:id="rId566" xr:uid="{10E6B9B1-5D76-4184-8740-7EA70231C735}"/>
+    <hyperlink ref="L839" r:id="rId567" xr:uid="{696BFE12-510C-4CD3-9E47-D0481FD901B7}"/>
+    <hyperlink ref="L812" r:id="rId568" xr:uid="{5ED1529A-5F4E-4308-ACAF-7642BC1D2868}"/>
+    <hyperlink ref="L809" r:id="rId569" xr:uid="{38C05E39-F010-4D1A-8CAC-1699A9C2E280}"/>
+    <hyperlink ref="L833" r:id="rId570" xr:uid="{393D38E2-36D6-4C37-87D8-808AF1F52D0C}"/>
+    <hyperlink ref="L797" r:id="rId571" xr:uid="{F363A484-A9E6-4FD3-BB2F-1C8FA1B9D51E}"/>
+    <hyperlink ref="L795" r:id="rId572" xr:uid="{5F8BD157-A5B0-4DBE-93EA-4FB22CE4C48B}"/>
+    <hyperlink ref="L788" r:id="rId573" xr:uid="{9E44EAF8-5BED-4C0F-A89E-0B6ECD0F06A5}"/>
+    <hyperlink ref="L829" r:id="rId574" xr:uid="{039F1AB2-B467-43C7-A3E2-59F9C5AE09D9}"/>
+    <hyperlink ref="L798" r:id="rId575" xr:uid="{0ED5745A-50E4-49C0-ABDD-4DF7772E2247}"/>
+    <hyperlink ref="L231" r:id="rId576" xr:uid="{5A72733D-5117-4137-87AD-536B0CE04DFF}"/>
+    <hyperlink ref="L855" r:id="rId577" xr:uid="{0EFB5B1D-0695-4F20-8AE2-DE5269E5D19E}"/>
+    <hyperlink ref="L336" r:id="rId578" xr:uid="{D6D10C65-F36A-489A-8707-F63B4D121DEE}"/>
+    <hyperlink ref="L958" r:id="rId579" display="https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-203.json" xr:uid="{121C0C2E-817E-4E76-92E4-761664ADBCCC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId551"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId580"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: corrected defra noise levels configuration source
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D2EFF0-C3AF-4CD9-A13F-86E15B06AE01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4BBED3-E913-4E5B-BEE5-C236757592E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">datasets!$A$1:$T$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">variables!$A$1:$S$1515</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -9985,9 +9985,6 @@
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise/Level3/EN_Environmental_Noise_Directive_Noise_Mapping_Agglomerations_Round_3.json</t>
   </si>
   <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise/Level3/EN_Noise_Action_Planning_Important_Areas_Round_3.json</t>
-  </si>
-  <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info.json</t>
   </si>
   <si>
@@ -10076,6 +10073,9 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/info-204.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/DEFRA/Noise/Level3/info.json</t>
   </si>
 </sst>
 </file>
@@ -10671,7 +10671,7 @@
         <v>2000</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>3315</v>
+        <v>3314</v>
       </c>
       <c r="I4">
         <v>2</v>
@@ -10700,7 +10700,7 @@
         <v>3000</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>3314</v>
+        <v>3344</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -24075,7 +24075,7 @@
       </c>
       <c r="J231" s="6"/>
       <c r="L231" s="3" t="s">
-        <v>3341</v>
+        <v>3340</v>
       </c>
       <c r="M231">
         <v>2</v>
@@ -28278,7 +28278,7 @@
       </c>
       <c r="J336" s="6"/>
       <c r="L336" s="3" t="s">
-        <v>3343</v>
+        <v>3342</v>
       </c>
       <c r="M336">
         <v>2</v>
@@ -47041,7 +47041,7 @@
       </c>
       <c r="J787" s="6"/>
       <c r="L787" s="3" t="s">
-        <v>3327</v>
+        <v>3326</v>
       </c>
       <c r="M787">
         <v>2</v>
@@ -47084,7 +47084,7 @@
       </c>
       <c r="J788" s="6"/>
       <c r="L788" s="3" t="s">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="M788">
         <v>2</v>
@@ -47209,7 +47209,7 @@
       </c>
       <c r="J791" s="6"/>
       <c r="L791" s="3" t="s">
-        <v>3325</v>
+        <v>3324</v>
       </c>
       <c r="M791">
         <v>2</v>
@@ -47372,7 +47372,7 @@
       </c>
       <c r="J795" s="6"/>
       <c r="L795" s="3" t="s">
-        <v>3337</v>
+        <v>3336</v>
       </c>
       <c r="M795">
         <v>2</v>
@@ -47456,7 +47456,7 @@
       </c>
       <c r="J797" s="6"/>
       <c r="L797" s="3" t="s">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="M797">
         <v>2</v>
@@ -47499,7 +47499,7 @@
       </c>
       <c r="J798" s="6"/>
       <c r="L798" s="3" t="s">
-        <v>3340</v>
+        <v>3339</v>
       </c>
       <c r="M798">
         <v>2</v>
@@ -47542,7 +47542,7 @@
       </c>
       <c r="J799" s="6"/>
       <c r="L799" s="3" t="s">
-        <v>3320</v>
+        <v>3319</v>
       </c>
       <c r="M799">
         <v>2</v>
@@ -47585,7 +47585,7 @@
       </c>
       <c r="J800" s="6"/>
       <c r="L800" s="3" t="s">
-        <v>3323</v>
+        <v>3322</v>
       </c>
       <c r="M800">
         <v>2</v>
@@ -47628,7 +47628,7 @@
       </c>
       <c r="J801" s="6"/>
       <c r="L801" s="3" t="s">
-        <v>3324</v>
+        <v>3323</v>
       </c>
       <c r="M801">
         <v>2</v>
@@ -47712,7 +47712,7 @@
       </c>
       <c r="J803" s="6"/>
       <c r="L803" s="3" t="s">
-        <v>3316</v>
+        <v>3315</v>
       </c>
       <c r="M803">
         <v>2</v>
@@ -47955,7 +47955,7 @@
       </c>
       <c r="J809" s="6"/>
       <c r="L809" s="3" t="s">
-        <v>3334</v>
+        <v>3333</v>
       </c>
       <c r="M809">
         <v>2</v>
@@ -47998,7 +47998,7 @@
       </c>
       <c r="J810" s="6"/>
       <c r="L810" s="3" t="s">
-        <v>3318</v>
+        <v>3317</v>
       </c>
       <c r="M810">
         <v>2</v>
@@ -48041,7 +48041,7 @@
       </c>
       <c r="J811" s="6"/>
       <c r="L811" s="3" t="s">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="M811">
         <v>2</v>
@@ -48084,7 +48084,7 @@
       </c>
       <c r="J812" s="6"/>
       <c r="L812" s="3" t="s">
-        <v>3333</v>
+        <v>3332</v>
       </c>
       <c r="M812">
         <v>2</v>
@@ -48127,7 +48127,7 @@
       </c>
       <c r="J813" s="6"/>
       <c r="L813" s="3" t="s">
-        <v>3330</v>
+        <v>3329</v>
       </c>
       <c r="M813">
         <v>2</v>
@@ -48770,7 +48770,7 @@
       </c>
       <c r="J829" s="6"/>
       <c r="L829" s="3" t="s">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="M829">
         <v>2</v>
@@ -48813,7 +48813,7 @@
       </c>
       <c r="J830" s="6"/>
       <c r="L830" s="3" t="s">
-        <v>3331</v>
+        <v>3330</v>
       </c>
       <c r="M830">
         <v>2</v>
@@ -48856,7 +48856,7 @@
       </c>
       <c r="J831" s="6"/>
       <c r="L831" s="3" t="s">
-        <v>3322</v>
+        <v>3321</v>
       </c>
       <c r="M831">
         <v>2</v>
@@ -48940,7 +48940,7 @@
       </c>
       <c r="J833" s="6"/>
       <c r="L833" s="3" t="s">
-        <v>3335</v>
+        <v>3334</v>
       </c>
       <c r="M833">
         <v>2</v>
@@ -49065,7 +49065,7 @@
       </c>
       <c r="J836" s="6"/>
       <c r="L836" s="3" t="s">
-        <v>3321</v>
+        <v>3320</v>
       </c>
       <c r="M836">
         <v>2</v>
@@ -49108,7 +49108,7 @@
       </c>
       <c r="J837" s="6"/>
       <c r="L837" s="3" t="s">
-        <v>3326</v>
+        <v>3325</v>
       </c>
       <c r="M837">
         <v>2</v>
@@ -49151,7 +49151,7 @@
       </c>
       <c r="J838" s="6"/>
       <c r="L838" s="3" t="s">
-        <v>3328</v>
+        <v>3327</v>
       </c>
       <c r="M838">
         <v>2</v>
@@ -49194,7 +49194,7 @@
       </c>
       <c r="J839" s="6"/>
       <c r="L839" s="3" t="s">
-        <v>3332</v>
+        <v>3331</v>
       </c>
       <c r="M839">
         <v>2</v>
@@ -49278,7 +49278,7 @@
       </c>
       <c r="J841" s="6"/>
       <c r="L841" s="3" t="s">
-        <v>3329</v>
+        <v>3328</v>
       </c>
       <c r="M841">
         <v>2</v>
@@ -49321,7 +49321,7 @@
       </c>
       <c r="J842" s="6"/>
       <c r="L842" s="3" t="s">
-        <v>3317</v>
+        <v>3316</v>
       </c>
       <c r="M842">
         <v>2</v>
@@ -49844,7 +49844,7 @@
       </c>
       <c r="J855" s="6"/>
       <c r="L855" s="3" t="s">
-        <v>3342</v>
+        <v>3341</v>
       </c>
       <c r="M855">
         <v>2</v>
@@ -53967,7 +53967,7 @@
       </c>
       <c r="J958" s="6"/>
       <c r="L958" s="3" t="s">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="M958">
         <v>2</v>

</xml_diff>

<commit_message>
fix: corrected the daily_aqi_pm2p5_dry_aerosol infographic
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0CCFC3-2063-43A3-8B70-6E86C613614C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2303545A-85F1-4CB0-9ACE-771DAF2666CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6639" uniqueCount="3349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6639" uniqueCount="3350">
   <si>
     <t>DbId</t>
   </si>
@@ -10088,6 +10088,9 @@
   </si>
   <si>
     <t>The field '% no. of care homes exposed to flooding' measures the percentage of care home facilities within a neighborhood that are physically located in areas identified as prone to flooding. Within the Climate Just framework, this metric serves as an indicator of enhanced exposure. It identifies institutional settings where highly sensitive populations (such as the elderly or those with chronic health conditions) are at direct risk of contact with floodwaters. The physical exposure of these buildings is a critical factor because it can severely undermine a community's ability to respond and recover, as the residents often rely on complex institutional care regimes and may have limited personal mobility during an emergency.</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/MetOffice/AQREAN/Annual/SL/daily_aqi_pm2p5_dry_aerosol/info.json</t>
   </si>
 </sst>
 </file>
@@ -13503,7 +13506,7 @@
         <v>7003</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>1853</v>
+        <v>3349</v>
       </c>
       <c r="P44">
         <v>2</v>

</xml_diff>

<commit_message>
chore: deleted two variable description rows from the config.xlsx
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2303545A-85F1-4CB0-9ACE-771DAF2666CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8C1CE2-BE9B-4E53-A41F-2A843AFD1520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6639" uniqueCount="3350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6637" uniqueCount="3348">
   <si>
     <t>DbId</t>
   </si>
@@ -10079,12 +10079,6 @@
   </si>
   <si>
     <t>The field 'All pensioner households (%)' (internal field name AllPensioner_HH) represents the percentage of households within a neighborhood (LSOA, Data Zone, or SOA) where all residents are of pensionable age.This metric is a core indicator used to calculate the Neighbourhood Flood Vulnerability Index (NFVI). Within the Climate Just framework, it serves as a measure of sensitivity, identifying populations that may be more susceptible to negative health and welfare impacts during a flood event due to age-related biophysical characteristics</t>
-  </si>
-  <si>
-    <t>The field 'Recent arrivals to UK (% people with &lt;1 yr residency coming from outside UK)' (internal name ArrivalsInUK) represents the percentage of a neighborhood's population that has been resident in the UK for less than one year after arriving from a foreign country. Within the Climate Just framework, this metric is used as an indicator of social vulnerability. It identifies groups that may have a reduced ability to prepare for, respond to, and recover from flooding due to a lack of local knowledge, limited community networks, or unfamiliarity with how to access essential information and public services during an extreme weather event.</t>
-  </si>
-  <si>
-    <t>The field '% caravan or other mobile or temporary structures in all households' (internal name Caravan_HH) represents the percentage of households within a neighborhood (LSOA, Data Zone, or SOA) that reside in non-permanent dwellings. Within the Climate Just framework, this metric is used as an indicator of enhanced exposure related to housing characteristics. Because caravans and temporary structures are typically less resilient to the physical force of water than permanent brick-and-mortar buildings, this indicator identifies areas here the physical environment is likely to accentuate the severity of a flood event's impact on residents.</t>
   </si>
   <si>
     <t>The field '% no. of care homes exposed to flooding' measures the percentage of care home facilities within a neighborhood that are physically located in areas identified as prone to flooding. Within the Climate Just framework, this metric serves as an indicator of enhanced exposure. It identifies institutional settings where highly sensitive populations (such as the elderly or those with chronic health conditions) are at direct risk of contact with floodwaters. The physical exposure of these buildings is a critical factor because it can severely undermine a community's ability to respond and recover, as the residents often rely on complex institutional care regimes and may have limited personal mobility during an emergency.</t>
@@ -13506,7 +13500,7 @@
         <v>7003</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>3349</v>
+        <v>3347</v>
       </c>
       <c r="P44">
         <v>2</v>
@@ -47072,9 +47066,7 @@
       <c r="P787" t="b">
         <v>0</v>
       </c>
-      <c r="R787" t="s">
-        <v>3346</v>
-      </c>
+      <c r="R787"/>
     </row>
     <row r="788" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A788">
@@ -47117,9 +47109,7 @@
       <c r="P788" t="b">
         <v>0</v>
       </c>
-      <c r="R788" t="s">
-        <v>3347</v>
-      </c>
+      <c r="R788"/>
     </row>
     <row r="789" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A789">
@@ -47161,7 +47151,7 @@
         <v>0</v>
       </c>
       <c r="R789" t="s">
-        <v>3348</v>
+        <v>3346</v>
       </c>
     </row>
     <row r="790" spans="1:18" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
chore: removed filters from config.xlsx
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F129AA7B-BAB6-4325-B2AF-1D5607336F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832DAB5F-559B-4301-8222-09AB1D2FEAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11483,7 +11483,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:W65"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -11583,7 +11582,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -11642,7 +11641,7 @@
         <v>2274</v>
       </c>
     </row>
-    <row r="3" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>101</v>
       </c>
@@ -11701,7 +11700,7 @@
         <v>2275</v>
       </c>
     </row>
-    <row r="4" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>201</v>
       </c>
@@ -11760,7 +11759,7 @@
         <v>2276</v>
       </c>
     </row>
-    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>301</v>
       </c>
@@ -11816,7 +11815,7 @@
         <v>2277</v>
       </c>
     </row>
-    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>401</v>
       </c>
@@ -11872,7 +11871,7 @@
         <v>2278</v>
       </c>
     </row>
-    <row r="7" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>501</v>
       </c>
@@ -11928,7 +11927,7 @@
         <v>2279</v>
       </c>
     </row>
-    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>601</v>
       </c>
@@ -11984,7 +11983,7 @@
         <v>2280</v>
       </c>
     </row>
-    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>701</v>
       </c>
@@ -12037,7 +12036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>801</v>
       </c>
@@ -12090,7 +12089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>901</v>
       </c>
@@ -12143,7 +12142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1001</v>
       </c>
@@ -12196,7 +12195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1101</v>
       </c>
@@ -12249,7 +12248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1201</v>
       </c>
@@ -12302,7 +12301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>1301</v>
       </c>
@@ -12358,7 +12357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1401</v>
       </c>
@@ -12414,7 +12413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1501</v>
       </c>
@@ -12470,7 +12469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1601</v>
       </c>
@@ -12526,7 +12525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1701</v>
       </c>
@@ -12638,7 +12637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1901</v>
       </c>
@@ -12694,7 +12693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2001</v>
       </c>
@@ -12750,7 +12749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2101</v>
       </c>
@@ -12806,7 +12805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2201</v>
       </c>
@@ -12862,7 +12861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2301</v>
       </c>
@@ -12918,7 +12917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2401</v>
       </c>
@@ -12974,7 +12973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2501</v>
       </c>
@@ -13030,7 +13029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2601</v>
       </c>
@@ -13086,7 +13085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2701</v>
       </c>
@@ -13143,7 +13142,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="30" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2801</v>
       </c>
@@ -13202,7 +13201,7 @@
         <v>2266</v>
       </c>
     </row>
-    <row r="31" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2901</v>
       </c>
@@ -13261,7 +13260,7 @@
         <v>2267</v>
       </c>
     </row>
-    <row r="32" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>3001</v>
       </c>
@@ -13320,7 +13319,7 @@
         <v>2268</v>
       </c>
     </row>
-    <row r="33" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>3101</v>
       </c>
@@ -13379,7 +13378,7 @@
         <v>2269</v>
       </c>
     </row>
-    <row r="34" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3201</v>
       </c>
@@ -13438,7 +13437,7 @@
         <v>2270</v>
       </c>
     </row>
-    <row r="35" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>3301</v>
       </c>
@@ -13497,7 +13496,7 @@
         <v>2271</v>
       </c>
     </row>
-    <row r="36" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3401</v>
       </c>
@@ -13556,7 +13555,7 @@
         <v>2272</v>
       </c>
     </row>
-    <row r="37" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>3501</v>
       </c>
@@ -13615,7 +13614,7 @@
         <v>2273</v>
       </c>
     </row>
-    <row r="38" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>3601</v>
       </c>
@@ -13674,7 +13673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:22" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>3701</v>
       </c>
@@ -13724,7 +13723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>3801</v>
       </c>
@@ -13783,7 +13782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:22" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>3901</v>
       </c>
@@ -13833,7 +13832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>4001</v>
       </c>
@@ -13889,7 +13888,7 @@
         <v>2224</v>
       </c>
     </row>
-    <row r="43" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>4101</v>
       </c>
@@ -13951,7 +13950,7 @@
         <v>2225</v>
       </c>
     </row>
-    <row r="44" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>4201</v>
       </c>
@@ -14013,7 +14012,7 @@
         <v>2226</v>
       </c>
     </row>
-    <row r="45" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>4301</v>
       </c>
@@ -14075,7 +14074,7 @@
         <v>2227</v>
       </c>
     </row>
-    <row r="46" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>4401</v>
       </c>
@@ -14137,7 +14136,7 @@
         <v>2228</v>
       </c>
     </row>
-    <row r="47" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>4501</v>
       </c>
@@ -14199,7 +14198,7 @@
         <v>2229</v>
       </c>
     </row>
-    <row r="48" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>4601</v>
       </c>
@@ -14261,7 +14260,7 @@
         <v>2230</v>
       </c>
     </row>
-    <row r="49" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>4701</v>
       </c>
@@ -14323,7 +14322,7 @@
         <v>2231</v>
       </c>
     </row>
-    <row r="50" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>4801</v>
       </c>
@@ -14385,7 +14384,7 @@
         <v>2232</v>
       </c>
     </row>
-    <row r="51" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>4901</v>
       </c>
@@ -14447,7 +14446,7 @@
         <v>2233</v>
       </c>
     </row>
-    <row r="52" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>5001</v>
       </c>
@@ -14509,7 +14508,7 @@
         <v>2234</v>
       </c>
     </row>
-    <row r="53" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>5101</v>
       </c>
@@ -14571,7 +14570,7 @@
         <v>2235</v>
       </c>
     </row>
-    <row r="54" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>5201</v>
       </c>
@@ -14633,7 +14632,7 @@
         <v>2236</v>
       </c>
     </row>
-    <row r="55" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>5301</v>
       </c>
@@ -14695,7 +14694,7 @@
         <v>2237</v>
       </c>
     </row>
-    <row r="56" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>5401</v>
       </c>
@@ -14757,7 +14756,7 @@
         <v>2238</v>
       </c>
     </row>
-    <row r="57" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>5501</v>
       </c>
@@ -14819,7 +14818,7 @@
         <v>2239</v>
       </c>
     </row>
-    <row r="58" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>5601</v>
       </c>
@@ -14881,7 +14880,7 @@
         <v>2240</v>
       </c>
     </row>
-    <row r="59" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>5701</v>
       </c>
@@ -14943,7 +14942,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="60" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>5801</v>
       </c>
@@ -15000,7 +14999,7 @@
         <v>2223</v>
       </c>
     </row>
-    <row r="61" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>5901</v>
       </c>
@@ -15062,7 +15061,7 @@
         <v>2242</v>
       </c>
     </row>
-    <row r="62" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>6001</v>
       </c>
@@ -15124,7 +15123,7 @@
         <v>2243</v>
       </c>
     </row>
-    <row r="63" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>6101</v>
       </c>
@@ -15186,7 +15185,7 @@
         <v>2244</v>
       </c>
     </row>
-    <row r="64" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>6201</v>
       </c>
@@ -15248,7 +15247,7 @@
         <v>2245</v>
       </c>
     </row>
-    <row r="65" spans="1:22" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>6301</v>
       </c>
@@ -15311,13 +15310,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T65" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="climatejust_lsoas_uk_2011_flood_data"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:T65" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <hyperlinks>
     <hyperlink ref="E22" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
     <hyperlink ref="E29" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>

</xml_diff>

<commit_message>
chore: added two new records in the config.xlsx
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF108D0-0F52-4A62-97DF-B770A20FB2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B8C49A-55BD-48CA-8E28-69C220089573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6971" uniqueCount="3664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6973" uniqueCount="3666">
   <si>
     <t>DbId</t>
   </si>
@@ -11033,6 +11033,12 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_lsoas_wa_2011_2022_v3_2022_data/128_housingheatvulnerability.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/001_r_hzz_cv1.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/002_r_hzz_cv2.json</t>
   </si>
 </sst>
 </file>
@@ -19985,6 +19991,9 @@
       <c r="J110" s="6" t="s">
         <v>369</v>
       </c>
+      <c r="L110" t="s">
+        <v>3664</v>
+      </c>
       <c r="M110">
         <v>2</v>
       </c>
@@ -20027,6 +20036,9 @@
       <c r="J111" s="6" t="s">
         <v>369</v>
       </c>
+      <c r="L111" t="s">
+        <v>3665</v>
+      </c>
       <c r="M111">
         <v>2</v>
       </c>
@@ -24841,7 +24853,7 @@
         <v>0</v>
       </c>
       <c r="J226" s="6"/>
-      <c r="L226" t="s">
+      <c r="L226" s="3" t="s">
         <v>3354</v>
       </c>
       <c r="M226">
@@ -82716,9 +82728,10 @@
     <hyperlink ref="L1109" r:id="rId549" xr:uid="{665C61A8-134F-442F-98D5-81FFD9A3B965}"/>
     <hyperlink ref="L1110" r:id="rId550" xr:uid="{9372FBA2-CD81-4F9B-B049-5FD85AD034A7}"/>
     <hyperlink ref="L842" r:id="rId551" xr:uid="{888B8DBF-54D3-48FC-BBCE-D30D8A5C2EF7}"/>
+    <hyperlink ref="L226" r:id="rId552" xr:uid="{17799A3C-A04C-4D45-BE2E-BCC0D0D59AB1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId552"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId553"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
chore: added two example config references
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B8C49A-55BD-48CA-8E28-69C220089573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F758F3-6073-4109-9B2C-EAC641AC834F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6973" uniqueCount="3666">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6975" uniqueCount="3668">
   <si>
     <t>DbId</t>
   </si>
@@ -11039,6 +11039,12 @@
   </si>
   <si>
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/002_r_hzz_cv2.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/aa.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/bb.json</t>
   </si>
 </sst>
 </file>
@@ -20081,6 +20087,9 @@
       <c r="J112" s="6" t="s">
         <v>369</v>
       </c>
+      <c r="L112" t="s">
+        <v>3666</v>
+      </c>
       <c r="M112">
         <v>2</v>
       </c>
@@ -20122,6 +20131,9 @@
       </c>
       <c r="J113" s="6" t="s">
         <v>375</v>
+      </c>
+      <c r="L113" t="s">
+        <v>3667</v>
       </c>
       <c r="M113">
         <v>2</v>

</xml_diff>

<commit_message>
fix: corrected json config paths for the climatejust ukcp18 dataset in the config.xlsx file
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980BD46C-E886-4206-ABE6-CDFC613FCEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB49CA5-E29E-4081-AA1A-12C2CC466862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11359,1084 +11359,1084 @@
     <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_england_heat/108_zchm90wn.json</t>
   </si>
   <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/001_tas_rcp26_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/002_tas_rcp26_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/003_tas_rcp26_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/004_tas_rcp26_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/005_tas_rcp26_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/006_tas_rcp26_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/007_tas_rcp26_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/008_tas_rcp26_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/009_tas_rcp26_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/010_tas_rcp45_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/011_tas_rcp45_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/012_tas_rcp45_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/013_tas_rcp45_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/014_tas_rcp45_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/015_tas_rcp45_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/016_tas_rcp45_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/017_tas_rcp45_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/018_tas_rcp45_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/019_tas_rcp60_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/020_tas_rcp60_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/021_tas_rcp60_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/022_tas_rcp60_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/023_tas_rcp60_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/024_tas_rcp60_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/025_tas_rcp60_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/026_tas_rcp60_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/027_tas_rcp60_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/028_tas_rcp85_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/029_tas_rcp85_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/030_tas_rcp85_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/031_tas_rcp85_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/032_tas_rcp85_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/033_tas_rcp85_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/034_tas_rcp85_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/035_tas_rcp85_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/036_tas_rcp85_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/037_tasmax_rcp26_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/038_tasmax_rcp26_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/039_tasmax_rcp26_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/040_tasmax_rcp26_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/041_tasmax_rcp26_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/042_tasmax_rcp26_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/043_tasmax_rcp26_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/044_tasmax_rcp26_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/045_tasmax_rcp26_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/046_tasmax_rcp45_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/047_tasmax_rcp45_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/048_tasmax_rcp45_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/049_tasmax_rcp45_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/050_tasmax_rcp45_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/051_tasmax_rcp45_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/052_tasmax_rcp45_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/053_tasmax_rcp45_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/054_tasmax_rcp45_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/055_tasmax_rcp60_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/056_tasmax_rcp60_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/057_tasmax_rcp60_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/058_tasmax_rcp60_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/059_tasmax_rcp60_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/060_tasmax_rcp60_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/061_tasmax_rcp60_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/062_tasmax_rcp60_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/063_tasmax_rcp60_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/064_tasmax_rcp85_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/065_tasmax_rcp85_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/066_tasmax_rcp85_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/067_tasmax_rcp85_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/068_tasmax_rcp85_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/069_tasmax_rcp85_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/070_tasmax_rcp85_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/071_tasmax_rcp85_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/072_tasmax_rcp85_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/073_z_all_rel_tas_rcp26_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/074_z_all_rel_tas_rcp26_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/075_z_all_rel_tas_rcp26_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/076_z_all_rel_tas_rcp26_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/077_z_all_rel_tas_rcp26_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/078_z_all_rel_tas_rcp26_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/079_z_all_rel_tas_rcp26_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/080_z_all_rel_tas_rcp26_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/081_z_all_rel_tas_rcp26_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/082_z_all_rel_tas_rcp45_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/083_z_all_rel_tas_rcp45_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/084_z_all_rel_tas_rcp45_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/085_z_all_rel_tas_rcp45_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/086_z_all_rel_tas_rcp45_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/087_z_all_rel_tas_rcp45_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/088_z_all_rel_tas_rcp45_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/089_z_all_rel_tas_rcp45_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/090_z_all_rel_tas_rcp45_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/091_z_all_rel_tas_rcp60_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/092_z_all_rel_tas_rcp60_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/093_z_all_rel_tas_rcp60_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/094_z_all_rel_tas_rcp60_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/095_z_all_rel_tas_rcp60_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/096_z_all_rel_tas_rcp60_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/097_z_all_rel_tas_rcp60_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/098_z_all_rel_tas_rcp60_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/099_z_all_rel_tas_rcp60_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/100_z_all_rel_tas_rcp85_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/101_z_all_rel_tas_rcp85_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/102_z_all_rel_tas_rcp85_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/103_z_all_rel_tas_rcp85_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/104_z_all_rel_tas_rcp85_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/105_z_all_rel_tas_rcp85_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/106_z_all_rel_tas_rcp85_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/107_z_all_rel_tas_rcp85_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/108_z_all_rel_tas_rcp85_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/109_z_all_rel_tasmax_rcp26_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/110_z_all_rel_tasmax_rcp26_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/111_z_all_rel_tasmax_rcp26_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/112_z_all_rel_tasmax_rcp26_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/113_z_all_rel_tasmax_rcp26_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/114_z_all_rel_tasmax_rcp26_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/115_z_all_rel_tasmax_rcp26_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/116_z_all_rel_tasmax_rcp26_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/117_z_all_rel_tasmax_rcp26_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/118_z_all_rel_tasmax_rcp45_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/119_z_all_rel_tasmax_rcp45_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/120_z_all_rel_tasmax_rcp45_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/121_z_all_rel_tasmax_rcp45_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/122_z_all_rel_tasmax_rcp45_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/123_z_all_rel_tasmax_rcp45_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/124_z_all_rel_tasmax_rcp45_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/125_z_all_rel_tasmax_rcp45_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/126_z_all_rel_tasmax_rcp45_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/127_z_all_rel_tasmax_rcp60_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/128_z_all_rel_tasmax_rcp60_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/129_z_all_rel_tasmax_rcp60_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/130_z_all_rel_tasmax_rcp60_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/131_z_all_rel_tasmax_rcp60_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/132_z_all_rel_tasmax_rcp60_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/133_z_all_rel_tasmax_rcp60_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/134_z_all_rel_tasmax_rcp60_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/135_z_all_rel_tasmax_rcp60_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/136_z_all_rel_tasmax_rcp85_2019_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/137_z_all_rel_tasmax_rcp85_2019_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/138_z_all_rel_tasmax_rcp85_2019_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/139_z_all_rel_tasmax_rcp85_2049_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/140_z_all_rel_tasmax_rcp85_2049_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/141_z_all_rel_tasmax_rcp85_2049_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/142_z_all_rel_tasmax_rcp85_2079_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/143_z_all_rel_tasmax_rcp85_2079_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/144_z_all_rel_tasmax_rcp85_2079_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/145_tasmax_rcp26_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/146_tasmax_rcp26_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/147_tasmax_rcp26_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/148_tasmax_rcp26_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/149_tasmax_rcp26_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/150_tasmax_rcp26_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/151_tasmax_rcp26_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/152_tasmax_rcp26_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/153_tasmax_rcp26_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/154_tasmax_rcp26_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/155_tasmax_rcp26_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/156_tasmax_rcp26_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/157_tasmax_rcp26_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/158_tasmax_rcp26_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/159_tasmax_rcp26_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/160_tasmax_rcp26_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/161_tasmax_rcp26_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/162_tasmax_rcp26_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/163_tasmax_rcp26_rp100_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/164_tasmax_rcp26_rp100_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/165_tasmax_rcp26_rp100_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/166_tasmax_rcp26_rp100_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/167_tasmax_rcp26_rp100_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/168_tasmax_rcp26_rp100_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/169_tasmax_rcp26_rp100_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/170_tasmax_rcp26_rp100_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/171_tasmax_rcp26_rp100_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/172_tasmax_rcp45_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/173_tasmax_rcp45_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/174_tasmax_rcp45_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/175_tasmax_rcp45_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/176_tasmax_rcp45_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/177_tasmax_rcp45_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/178_tasmax_rcp45_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/179_tasmax_rcp45_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/180_tasmax_rcp45_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/181_tasmax_rcp45_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/182_tasmax_rcp45_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/183_tasmax_rcp45_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/184_tasmax_rcp45_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/185_tasmax_rcp45_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/186_tasmax_rcp45_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/187_tasmax_rcp45_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/188_tasmax_rcp45_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/189_tasmax_rcp45_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/190_tasmax_rcp45_rp100_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/191_tasmax_rcp45_rp100_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/192_tasmax_rcp45_rp100_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/193_tasmax_rcp45_rp100_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/194_tasmax_rcp45_rp100_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/195_tasmax_rcp45_rp100_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/196_tasmax_rcp45_rp100_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/197_tasmax_rcp45_rp100_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/198_tasmax_rcp45_rp100_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/199_tasmax_rcp60_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/200_tasmax_rcp60_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/201_tasmax_rcp60_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/202_tasmax_rcp60_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/203_tasmax_rcp60_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/204_tasmax_rcp60_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/205_tasmax_rcp60_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/206_tasmax_rcp60_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/207_tasmax_rcp60_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/208_tasmax_rcp60_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/209_tasmax_rcp60_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/210_tasmax_rcp60_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/211_tasmax_rcp60_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/212_tasmax_rcp60_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/213_tasmax_rcp60_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/214_tasmax_rcp60_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/215_tasmax_rcp60_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/216_tasmax_rcp60_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/217_tasmax_rcp60_rp100_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/218_tasmax_rcp60_rp100_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/219_tasmax_rcp60_rp100_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/220_tasmax_rcp60_rp100_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/221_tasmax_rcp60_rp100_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/222_tasmax_rcp60_rp100_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/223_tasmax_rcp60_rp100_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/224_tasmax_rcp60_rp100_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/225_tasmax_rcp60_rp100_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/226_tasmax_rcp85_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/227_tasmax_rcp85_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/228_tasmax_rcp85_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/229_tasmax_rcp85_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/230_tasmax_rcp85_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/231_tasmax_rcp85_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/232_tasmax_rcp85_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/233_tasmax_rcp85_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/234_tasmax_rcp85_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/235_tasmax_rcp85_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/236_tasmax_rcp85_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/237_tasmax_rcp85_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/238_tasmax_rcp85_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/239_tasmax_rcp85_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/240_tasmax_rcp85_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/241_tasmax_rcp85_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/242_tasmax_rcp85_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/243_tasmax_rcp85_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/244_tasmax_rcp85_rp100_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/245_tasmax_rcp85_rp100_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/246_tasmax_rcp85_rp100_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/247_tasmax_rcp85_rp100_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/248_tasmax_rcp85_rp100_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/249_tasmax_rcp85_rp100_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/250_tasmax_rcp85_rp100_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/251_tasmax_rcp85_rp100_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/252_tasmax_rcp85_rp100_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/253_z_ar_tasmax_rcp26_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/254_z_ar_tasmax_rcp26_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/255_z_ar_tasmax_rcp26_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/256_z_ar_tasmax_rcp26_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/257_z_ar_tasmax_rcp26_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/258_z_ar_tasmax_rcp26_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/259_z_ar_tasmax_rcp26_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/260_z_ar_tasmax_rcp26_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/261_z_ar_tasmax_rcp26_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/262_z_ar_tasmax_rcp26_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/263_z_ar_tasmax_rcp26_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/264_z_ar_tasmax_rcp26_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/265_z_ar_tasmax_rcp26_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/266_z_ar_tasmax_rcp26_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/267_z_ar_tasmax_rcp26_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/268_z_ar_tasmax_rcp26_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/269_z_ar_tasmax_rcp26_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/270_z_ar_tasmax_rcp26_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/271_z_ar_tasmax_rcp26_rp100_2020_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/272_z_ar_tasmax_rcp26_rp100_2020_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/273_z_ar_tasmax_rcp26_rp100_2020_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/274_z_ar_tasmax_rcp26_rp100_2050_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/275_z_ar_tasmax_rcp26_rp100_2050_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/276_z_ar_tasmax_rcp26_rp100_2050_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/277_z_ar_tasmax_rcp26_rp100_2080_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/278_z_ar_tasmax_rcp26_rp100_2080_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/279_z_ar_tasmax_rcp26_rp100_2080_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/280_z_ar_tasmax_rcp45_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/281_z_ar_tasmax_rcp45_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/282_z_ar_tasmax_rcp45_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/283_z_ar_tasmax_rcp45_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/284_z_ar_tasmax_rcp45_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/285_z_ar_tasmax_rcp45_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/286_z_ar_tasmax_rcp45_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/287_z_ar_tasmax_rcp45_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/288_z_ar_tasmax_rcp45_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/289_z_ar_tasmax_rcp45_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/290_z_ar_tasmax_rcp45_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/291_z_ar_tasmax_rcp45_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/292_z_ar_tasmax_rcp45_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/293_z_ar_tasmax_rcp45_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/294_z_ar_tasmax_rcp45_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/295_z_ar_tasmax_rcp45_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/296_z_ar_tasmax_rcp45_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/297_z_ar_tasmax_rcp45_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/298_z_ar_tasmax_rcp45_rp100_2020_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/299_z_ar_tasmax_rcp45_rp100_2020_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/300_z_ar_tasmax_rcp45_rp100_2020_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/301_z_ar_tasmax_rcp45_rp100_2050_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/302_z_ar_tasmax_rcp45_rp100_2050_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/303_z_ar_tasmax_rcp45_rp100_2050_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/304_z_ar_tasmax_rcp45_rp100_2080_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/305_z_ar_tasmax_rcp45_rp100_2080_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/306_z_ar_tasmax_rcp45_rp100_2080_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/307_z_ar_tasmax_rcp60_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/308_z_ar_tasmax_rcp60_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/309_z_ar_tasmax_rcp60_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/310_z_ar_tasmax_rcp60_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/311_z_ar_tasmax_rcp60_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/312_z_ar_tasmax_rcp60_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/313_z_ar_tasmax_rcp60_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/314_z_ar_tasmax_rcp60_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/315_z_ar_tasmax_rcp60_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/316_z_ar_tasmax_rcp60_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/317_z_ar_tasmax_rcp60_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/318_z_ar_tasmax_rcp60_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/319_z_ar_tasmax_rcp60_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/320_z_ar_tasmax_rcp60_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/321_z_ar_tasmax_rcp60_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/322_z_ar_tasmax_rcp60_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/323_z_ar_tasmax_rcp60_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/324_z_ar_tasmax_rcp60_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/325_z_ar_tasmax_rcp60_rp100_2020_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/326_z_ar_tasmax_rcp60_rp100_2020_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/327_z_ar_tasmax_rcp60_rp100_2020_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/328_z_ar_tasmax_rcp60_rp100_2050_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/329_z_ar_tasmax_rcp60_rp100_2050_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/330_z_ar_tasmax_rcp60_rp100_2050_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/331_z_ar_tasmax_rcp60_rp100_2080_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/332_z_ar_tasmax_rcp60_rp100_2080_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/333_z_ar_tasmax_rcp60_rp100_2080_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/334_z_ar_tasmax_rcp85_rp20_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/335_z_ar_tasmax_rcp85_rp20_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/336_z_ar_tasmax_rcp85_rp20_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/337_z_ar_tasmax_rcp85_rp20_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/338_z_ar_tasmax_rcp85_rp20_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/339_z_ar_tasmax_rcp85_rp20_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/340_z_ar_tasmax_rcp85_rp20_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/341_z_ar_tasmax_rcp85_rp20_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/342_z_ar_tasmax_rcp85_rp20_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/343_z_ar_tasmax_rcp85_rp50_2020_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/344_z_ar_tasmax_rcp85_rp50_2020_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/345_z_ar_tasmax_rcp85_rp50_2020_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/346_z_ar_tasmax_rcp85_rp50_2050_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/347_z_ar_tasmax_rcp85_rp50_2050_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/348_z_ar_tasmax_rcp85_rp50_2050_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/349_z_ar_tasmax_rcp85_rp50_2080_10p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/350_z_ar_tasmax_rcp85_rp50_2080_50p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/351_z_ar_tasmax_rcp85_rp50_2080_90p.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/352_z_ar_tasmax_rcp85_rp100_2020_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/353_z_ar_tasmax_rcp85_rp100_2020_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/354_z_ar_tasmax_rcp85_rp100_2020_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/355_z_ar_tasmax_rcp85_rp100_2050_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/356_z_ar_tasmax_rcp85_rp100_2050_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/357_z_ar_tasmax_rcp85_rp100_2050_90.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/358_z_ar_tasmax_rcp85_rp100_2080_10.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/359_z_ar_tasmax_rcp85_rp100_2080_50.json</t>
-  </si>
-  <si>
-    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/climatejust_grid_uk_ukcp18/360_z_ar_tasmax_rcp85_rp100_2080_90.json</t>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/001_tas_rcp26_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/002_tas_rcp26_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/003_tas_rcp26_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/004_tas_rcp26_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/005_tas_rcp26_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/006_tas_rcp26_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/007_tas_rcp26_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/008_tas_rcp26_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/009_tas_rcp26_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/010_tas_rcp45_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/011_tas_rcp45_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/012_tas_rcp45_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/013_tas_rcp45_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/014_tas_rcp45_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/015_tas_rcp45_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/016_tas_rcp45_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/017_tas_rcp45_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/018_tas_rcp45_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/019_tas_rcp60_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/020_tas_rcp60_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/021_tas_rcp60_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/022_tas_rcp60_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/023_tas_rcp60_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/024_tas_rcp60_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/025_tas_rcp60_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/026_tas_rcp60_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/027_tas_rcp60_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/028_tas_rcp85_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/029_tas_rcp85_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/030_tas_rcp85_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/031_tas_rcp85_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/032_tas_rcp85_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/033_tas_rcp85_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/034_tas_rcp85_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/035_tas_rcp85_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/036_tas_rcp85_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/037_tasmax_rcp26_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/038_tasmax_rcp26_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/039_tasmax_rcp26_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/040_tasmax_rcp26_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/041_tasmax_rcp26_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/042_tasmax_rcp26_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/043_tasmax_rcp26_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/044_tasmax_rcp26_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/045_tasmax_rcp26_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/046_tasmax_rcp45_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/047_tasmax_rcp45_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/048_tasmax_rcp45_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/049_tasmax_rcp45_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/050_tasmax_rcp45_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/051_tasmax_rcp45_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/052_tasmax_rcp45_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/053_tasmax_rcp45_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/054_tasmax_rcp45_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/055_tasmax_rcp60_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/056_tasmax_rcp60_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/057_tasmax_rcp60_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/058_tasmax_rcp60_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/059_tasmax_rcp60_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/060_tasmax_rcp60_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/061_tasmax_rcp60_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/062_tasmax_rcp60_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/063_tasmax_rcp60_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/064_tasmax_rcp85_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/065_tasmax_rcp85_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/066_tasmax_rcp85_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/067_tasmax_rcp85_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/068_tasmax_rcp85_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/069_tasmax_rcp85_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/070_tasmax_rcp85_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/071_tasmax_rcp85_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/072_tasmax_rcp85_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/073_z_all_rel_tas_rcp26_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/074_z_all_rel_tas_rcp26_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/075_z_all_rel_tas_rcp26_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/076_z_all_rel_tas_rcp26_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/077_z_all_rel_tas_rcp26_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/078_z_all_rel_tas_rcp26_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/079_z_all_rel_tas_rcp26_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/080_z_all_rel_tas_rcp26_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/081_z_all_rel_tas_rcp26_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/082_z_all_rel_tas_rcp45_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/083_z_all_rel_tas_rcp45_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/084_z_all_rel_tas_rcp45_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/085_z_all_rel_tas_rcp45_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/086_z_all_rel_tas_rcp45_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/087_z_all_rel_tas_rcp45_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/088_z_all_rel_tas_rcp45_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/089_z_all_rel_tas_rcp45_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/090_z_all_rel_tas_rcp45_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/091_z_all_rel_tas_rcp60_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/092_z_all_rel_tas_rcp60_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/093_z_all_rel_tas_rcp60_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/094_z_all_rel_tas_rcp60_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/095_z_all_rel_tas_rcp60_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/096_z_all_rel_tas_rcp60_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/097_z_all_rel_tas_rcp60_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/098_z_all_rel_tas_rcp60_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/099_z_all_rel_tas_rcp60_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/100_z_all_rel_tas_rcp85_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/101_z_all_rel_tas_rcp85_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/102_z_all_rel_tas_rcp85_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/103_z_all_rel_tas_rcp85_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/104_z_all_rel_tas_rcp85_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/105_z_all_rel_tas_rcp85_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/106_z_all_rel_tas_rcp85_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/107_z_all_rel_tas_rcp85_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/108_z_all_rel_tas_rcp85_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/109_z_all_rel_tasmax_rcp26_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/110_z_all_rel_tasmax_rcp26_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/111_z_all_rel_tasmax_rcp26_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/112_z_all_rel_tasmax_rcp26_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/113_z_all_rel_tasmax_rcp26_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/114_z_all_rel_tasmax_rcp26_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/115_z_all_rel_tasmax_rcp26_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/116_z_all_rel_tasmax_rcp26_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/117_z_all_rel_tasmax_rcp26_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/118_z_all_rel_tasmax_rcp45_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/119_z_all_rel_tasmax_rcp45_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/120_z_all_rel_tasmax_rcp45_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/121_z_all_rel_tasmax_rcp45_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/122_z_all_rel_tasmax_rcp45_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/123_z_all_rel_tasmax_rcp45_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/124_z_all_rel_tasmax_rcp45_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/125_z_all_rel_tasmax_rcp45_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/126_z_all_rel_tasmax_rcp45_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/127_z_all_rel_tasmax_rcp60_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/128_z_all_rel_tasmax_rcp60_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/129_z_all_rel_tasmax_rcp60_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/130_z_all_rel_tasmax_rcp60_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/131_z_all_rel_tasmax_rcp60_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/132_z_all_rel_tasmax_rcp60_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/133_z_all_rel_tasmax_rcp60_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/134_z_all_rel_tasmax_rcp60_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/135_z_all_rel_tasmax_rcp60_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/136_z_all_rel_tasmax_rcp85_2019_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/137_z_all_rel_tasmax_rcp85_2019_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/138_z_all_rel_tasmax_rcp85_2019_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/139_z_all_rel_tasmax_rcp85_2049_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/140_z_all_rel_tasmax_rcp85_2049_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/141_z_all_rel_tasmax_rcp85_2049_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/142_z_all_rel_tasmax_rcp85_2079_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/143_z_all_rel_tasmax_rcp85_2079_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/144_z_all_rel_tasmax_rcp85_2079_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/145_tasmax_rcp26_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/146_tasmax_rcp26_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/147_tasmax_rcp26_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/148_tasmax_rcp26_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/149_tasmax_rcp26_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/150_tasmax_rcp26_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/151_tasmax_rcp26_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/152_tasmax_rcp26_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/153_tasmax_rcp26_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/154_tasmax_rcp26_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/155_tasmax_rcp26_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/156_tasmax_rcp26_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/157_tasmax_rcp26_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/158_tasmax_rcp26_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/159_tasmax_rcp26_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/160_tasmax_rcp26_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/161_tasmax_rcp26_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/162_tasmax_rcp26_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/163_tasmax_rcp26_rp100_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/164_tasmax_rcp26_rp100_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/165_tasmax_rcp26_rp100_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/166_tasmax_rcp26_rp100_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/167_tasmax_rcp26_rp100_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/168_tasmax_rcp26_rp100_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/169_tasmax_rcp26_rp100_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/170_tasmax_rcp26_rp100_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/171_tasmax_rcp26_rp100_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/172_tasmax_rcp45_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/173_tasmax_rcp45_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/174_tasmax_rcp45_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/175_tasmax_rcp45_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/176_tasmax_rcp45_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/177_tasmax_rcp45_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/178_tasmax_rcp45_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/179_tasmax_rcp45_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/180_tasmax_rcp45_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/181_tasmax_rcp45_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/182_tasmax_rcp45_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/183_tasmax_rcp45_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/184_tasmax_rcp45_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/185_tasmax_rcp45_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/186_tasmax_rcp45_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/187_tasmax_rcp45_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/188_tasmax_rcp45_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/189_tasmax_rcp45_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/190_tasmax_rcp45_rp100_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/191_tasmax_rcp45_rp100_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/192_tasmax_rcp45_rp100_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/193_tasmax_rcp45_rp100_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/194_tasmax_rcp45_rp100_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/195_tasmax_rcp45_rp100_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/196_tasmax_rcp45_rp100_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/197_tasmax_rcp45_rp100_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/198_tasmax_rcp45_rp100_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/199_tasmax_rcp60_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/200_tasmax_rcp60_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/201_tasmax_rcp60_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/202_tasmax_rcp60_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/203_tasmax_rcp60_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/204_tasmax_rcp60_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/205_tasmax_rcp60_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/206_tasmax_rcp60_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/207_tasmax_rcp60_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/208_tasmax_rcp60_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/209_tasmax_rcp60_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/210_tasmax_rcp60_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/211_tasmax_rcp60_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/212_tasmax_rcp60_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/213_tasmax_rcp60_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/214_tasmax_rcp60_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/215_tasmax_rcp60_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/216_tasmax_rcp60_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/217_tasmax_rcp60_rp100_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/218_tasmax_rcp60_rp100_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/219_tasmax_rcp60_rp100_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/220_tasmax_rcp60_rp100_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/221_tasmax_rcp60_rp100_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/222_tasmax_rcp60_rp100_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/223_tasmax_rcp60_rp100_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/224_tasmax_rcp60_rp100_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/225_tasmax_rcp60_rp100_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/226_tasmax_rcp85_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/227_tasmax_rcp85_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/228_tasmax_rcp85_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/229_tasmax_rcp85_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/230_tasmax_rcp85_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/231_tasmax_rcp85_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/232_tasmax_rcp85_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/233_tasmax_rcp85_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/234_tasmax_rcp85_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/235_tasmax_rcp85_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/236_tasmax_rcp85_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/237_tasmax_rcp85_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/238_tasmax_rcp85_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/239_tasmax_rcp85_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/240_tasmax_rcp85_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/241_tasmax_rcp85_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/242_tasmax_rcp85_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/243_tasmax_rcp85_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/244_tasmax_rcp85_rp100_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/245_tasmax_rcp85_rp100_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/246_tasmax_rcp85_rp100_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/247_tasmax_rcp85_rp100_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/248_tasmax_rcp85_rp100_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/249_tasmax_rcp85_rp100_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/250_tasmax_rcp85_rp100_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/251_tasmax_rcp85_rp100_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/252_tasmax_rcp85_rp100_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/253_z_ar_tasmax_rcp26_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/254_z_ar_tasmax_rcp26_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/255_z_ar_tasmax_rcp26_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/256_z_ar_tasmax_rcp26_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/257_z_ar_tasmax_rcp26_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/258_z_ar_tasmax_rcp26_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/259_z_ar_tasmax_rcp26_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/260_z_ar_tasmax_rcp26_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/261_z_ar_tasmax_rcp26_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/262_z_ar_tasmax_rcp26_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/263_z_ar_tasmax_rcp26_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/264_z_ar_tasmax_rcp26_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/265_z_ar_tasmax_rcp26_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/266_z_ar_tasmax_rcp26_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/267_z_ar_tasmax_rcp26_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/268_z_ar_tasmax_rcp26_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/269_z_ar_tasmax_rcp26_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/270_z_ar_tasmax_rcp26_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/271_z_ar_tasmax_rcp26_rp100_2020_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/272_z_ar_tasmax_rcp26_rp100_2020_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/273_z_ar_tasmax_rcp26_rp100_2020_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/274_z_ar_tasmax_rcp26_rp100_2050_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/275_z_ar_tasmax_rcp26_rp100_2050_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/276_z_ar_tasmax_rcp26_rp100_2050_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/277_z_ar_tasmax_rcp26_rp100_2080_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/278_z_ar_tasmax_rcp26_rp100_2080_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/279_z_ar_tasmax_rcp26_rp100_2080_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/280_z_ar_tasmax_rcp45_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/281_z_ar_tasmax_rcp45_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/282_z_ar_tasmax_rcp45_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/283_z_ar_tasmax_rcp45_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/284_z_ar_tasmax_rcp45_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/285_z_ar_tasmax_rcp45_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/286_z_ar_tasmax_rcp45_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/287_z_ar_tasmax_rcp45_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/288_z_ar_tasmax_rcp45_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/289_z_ar_tasmax_rcp45_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/290_z_ar_tasmax_rcp45_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/291_z_ar_tasmax_rcp45_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/292_z_ar_tasmax_rcp45_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/293_z_ar_tasmax_rcp45_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/294_z_ar_tasmax_rcp45_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/295_z_ar_tasmax_rcp45_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/296_z_ar_tasmax_rcp45_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/297_z_ar_tasmax_rcp45_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/298_z_ar_tasmax_rcp45_rp100_2020_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/299_z_ar_tasmax_rcp45_rp100_2020_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/300_z_ar_tasmax_rcp45_rp100_2020_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/301_z_ar_tasmax_rcp45_rp100_2050_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/302_z_ar_tasmax_rcp45_rp100_2050_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/303_z_ar_tasmax_rcp45_rp100_2050_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/304_z_ar_tasmax_rcp45_rp100_2080_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/305_z_ar_tasmax_rcp45_rp100_2080_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/306_z_ar_tasmax_rcp45_rp100_2080_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/307_z_ar_tasmax_rcp60_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/308_z_ar_tasmax_rcp60_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/309_z_ar_tasmax_rcp60_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/310_z_ar_tasmax_rcp60_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/311_z_ar_tasmax_rcp60_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/312_z_ar_tasmax_rcp60_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/313_z_ar_tasmax_rcp60_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/314_z_ar_tasmax_rcp60_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/315_z_ar_tasmax_rcp60_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/316_z_ar_tasmax_rcp60_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/317_z_ar_tasmax_rcp60_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/318_z_ar_tasmax_rcp60_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/319_z_ar_tasmax_rcp60_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/320_z_ar_tasmax_rcp60_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/321_z_ar_tasmax_rcp60_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/322_z_ar_tasmax_rcp60_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/323_z_ar_tasmax_rcp60_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/324_z_ar_tasmax_rcp60_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/325_z_ar_tasmax_rcp60_rp100_2020_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/326_z_ar_tasmax_rcp60_rp100_2020_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/327_z_ar_tasmax_rcp60_rp100_2020_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/328_z_ar_tasmax_rcp60_rp100_2050_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/329_z_ar_tasmax_rcp60_rp100_2050_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/330_z_ar_tasmax_rcp60_rp100_2050_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/331_z_ar_tasmax_rcp60_rp100_2080_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/332_z_ar_tasmax_rcp60_rp100_2080_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/333_z_ar_tasmax_rcp60_rp100_2080_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/334_z_ar_tasmax_rcp85_rp20_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/335_z_ar_tasmax_rcp85_rp20_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/336_z_ar_tasmax_rcp85_rp20_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/337_z_ar_tasmax_rcp85_rp20_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/338_z_ar_tasmax_rcp85_rp20_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/339_z_ar_tasmax_rcp85_rp20_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/340_z_ar_tasmax_rcp85_rp20_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/341_z_ar_tasmax_rcp85_rp20_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/342_z_ar_tasmax_rcp85_rp20_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/343_z_ar_tasmax_rcp85_rp50_2020_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/344_z_ar_tasmax_rcp85_rp50_2020_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/345_z_ar_tasmax_rcp85_rp50_2020_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/346_z_ar_tasmax_rcp85_rp50_2050_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/347_z_ar_tasmax_rcp85_rp50_2050_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/348_z_ar_tasmax_rcp85_rp50_2050_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/349_z_ar_tasmax_rcp85_rp50_2080_10p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/350_z_ar_tasmax_rcp85_rp50_2080_50p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/351_z_ar_tasmax_rcp85_rp50_2080_90p.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/352_z_ar_tasmax_rcp85_rp100_2020_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/353_z_ar_tasmax_rcp85_rp100_2020_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/354_z_ar_tasmax_rcp85_rp100_2020_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/355_z_ar_tasmax_rcp85_rp100_2050_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/356_z_ar_tasmax_rcp85_rp100_2050_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/357_z_ar_tasmax_rcp85_rp100_2050_90.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/358_z_ar_tasmax_rcp85_rp100_2080_10.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/359_z_ar_tasmax_rcp85_rp100_2080_50.json</t>
+  </si>
+  <si>
+    <t>https://nerc-digital-solutions-hub.github.io/dsh-metadata/UPRN/ClimateJust/md/climatejust_grid_uk_ukcp18/360_z_ar_tasmax_rcp85_rp100_2080_90.json</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
chore(uprn-service): AQREAN NH4 layers are now hidden from treeview due to being missing from postgres database
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12362C1F-B6B9-4DE1-88E1-1C6C9A2B0253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7758E5C-E726-42D2-ABB0-3E340545D61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70193,10 +70193,10 @@
         <v>1834</v>
       </c>
       <c r="G1207" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1207" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1207" t="b">
         <v>0</v>
@@ -70241,10 +70241,10 @@
         <v>1834</v>
       </c>
       <c r="G1208" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1208" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1208" t="b">
         <v>0</v>
@@ -70289,10 +70289,10 @@
         <v>1834</v>
       </c>
       <c r="G1209" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1209" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1209" t="b">
         <v>0</v>
@@ -70337,10 +70337,10 @@
         <v>1834</v>
       </c>
       <c r="G1210" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1210" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1210" t="b">
         <v>0</v>
@@ -70385,10 +70385,10 @@
         <v>1834</v>
       </c>
       <c r="G1211" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1211" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1211" t="b">
         <v>0</v>
@@ -70433,10 +70433,10 @@
         <v>1834</v>
       </c>
       <c r="G1212" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1212" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1212" t="b">
         <v>0</v>
@@ -70481,10 +70481,10 @@
         <v>1834</v>
       </c>
       <c r="G1213" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1213" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1213" t="b">
         <v>0</v>
@@ -70529,10 +70529,10 @@
         <v>1834</v>
       </c>
       <c r="G1214" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1214" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1214" t="b">
         <v>0</v>
@@ -70577,10 +70577,10 @@
         <v>1834</v>
       </c>
       <c r="G1215" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1215" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1215" t="b">
         <v>0</v>
@@ -70625,10 +70625,10 @@
         <v>1834</v>
       </c>
       <c r="G1216" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1216" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1216" t="b">
         <v>0</v>
@@ -70673,10 +70673,10 @@
         <v>1834</v>
       </c>
       <c r="G1217" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1217" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1217" t="b">
         <v>0</v>
@@ -70721,10 +70721,10 @@
         <v>1834</v>
       </c>
       <c r="G1218" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1218" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1218" t="b">
         <v>0</v>
@@ -70769,10 +70769,10 @@
         <v>1834</v>
       </c>
       <c r="G1219" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1219" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1219" t="b">
         <v>0</v>
@@ -70817,10 +70817,10 @@
         <v>1834</v>
       </c>
       <c r="G1220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1220" t="b">
         <v>0</v>
@@ -70865,10 +70865,10 @@
         <v>1834</v>
       </c>
       <c r="G1221" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1221" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1221" t="b">
         <v>0</v>
@@ -70913,10 +70913,10 @@
         <v>1834</v>
       </c>
       <c r="G1222" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1222" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1222" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
chore(uprn-service): hid parent NH4 layer
</commit_message>
<xml_diff>
--- a/pages/apps/uprn-service/config.xlsx
+++ b/pages/apps/uprn-service/config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NDSH\GitHub\dsh-content\dev\pages\apps\uprn-service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7758E5C-E726-42D2-ABB0-3E340545D61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DF1FA3-D949-47ED-AC24-764547C1198F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="388" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="folders" sheetId="1" r:id="rId1"/>
@@ -16025,10 +16025,10 @@
         <v>1834</v>
       </c>
       <c r="H46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J46">
         <v>2</v>

</xml_diff>